<commit_message>
docs: test workbook v2.1 with 60-second SOS countdown
</commit_message>
<xml_diff>
--- a/MediFind_Test_Requirements_v2.xlsx
+++ b/MediFind_Test_Requirements_v2.xlsx
@@ -741,7 +741,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Project: MediFind FYP  |  Date: 2026-09-17  |  Version: 2.0 (aligned with SRS; v1.0 dated 2026-05-30)</t>
+          <t>Project: MediFind FYP  |  Date: 2026-09-17  |  Version: 2.1 (aligned with SRS; 60-second SOS countdown; v1.0 dated 2026-05-30)</t>
         </is>
       </c>
     </row>
@@ -894,7 +894,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Hold-to-SOS, 10-second Countdown, Categories, Tracking, ETA, Cancellation</t>
+          <t>Hold-to-SOS, 60-second Countdown, Categories, Tracking, ETA, Cancellation</t>
         </is>
       </c>
     </row>
@@ -5604,7 +5604,7 @@
       </c>
       <c r="D9" s="47" t="inlineStr">
         <is>
-          <t>Aligned with SRS FR4.1/FR4.3: press-and-hold plus a 10-second pre-send countdown (false SOS prevention).</t>
+          <t>Aligned with SRS FR4.1/FR4.3: press-and-hold plus a pre-send countdown (false SOS prevention). The SRS 10 s window was extended to 60 s by project decision; Send SOS now skips the wait.</t>
         </is>
       </c>
     </row>
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C81" s="47" t="inlineStr">
         <is>
-          <t>Cancelling during the 10-second countdown sends nothing to the server</t>
+          <t>Cancelling during the 60-second countdown sends nothing to the server</t>
         </is>
       </c>
       <c r="D81" s="47" t="inlineStr">
@@ -9206,7 +9206,7 @@
       </c>
       <c r="C22" s="31" t="inlineStr">
         <is>
-          <t>10-second cancellation window with countdown timer</t>
+          <t>Cancellation window with countdown timer (SRS: 10 s; implemented as 60 s by project decision)</t>
         </is>
       </c>
       <c r="D22" s="32">
@@ -11097,14 +11097,14 @@
       </c>
       <c r="D4" s="39" t="inlineStr">
         <is>
-          <t>Patient triggers SOS by holding the SOS button, choosing an emergency type, then a 10-second countdown before the alert is sent</t>
+          <t>Patient triggers SOS by holding the SOS button, choosing an emergency type, then a 60-second countdown before the alert is sent</t>
         </is>
       </c>
       <c r="E4" s="39" t="inlineStr">
         <is>
           <t>1. Press and hold SOS for ~2 s (progress ring fills)
 2. Select emergency type
-3. Watch the 10-second countdown reach 0</t>
+3. Watch the 60-second countdown reach 0 (or tap Send SOS now)</t>
         </is>
       </c>
       <c r="F4" s="39" t="inlineStr">
@@ -11188,7 +11188,7 @@
       </c>
       <c r="D6" s="39" t="inlineStr">
         <is>
-          <t>SOS can be cancelled during the 10-second countdown without contacting the server</t>
+          <t>SOS can be cancelled during the 60-second countdown without contacting the server</t>
         </is>
       </c>
       <c r="E6" s="39" t="inlineStr">
@@ -11980,12 +11980,12 @@
       </c>
       <c r="D5" s="43" t="inlineStr">
         <is>
-          <t>Cancelling during the 10-second countdown sends nothing to the server</t>
+          <t>Cancelling during the 60-second countdown sends nothing to the server</t>
         </is>
       </c>
       <c r="E5" s="43" t="inlineStr">
         <is>
-          <t>Start SOS and cancel at 5 s</t>
+          <t>Start SOS and cancel at 30 s</t>
         </is>
       </c>
       <c r="F5" s="43" t="inlineStr">

</xml_diff>

<commit_message>
test: in-app call UI results (missed, voice, video, background, Deaf, emergency end)
</commit_message>
<xml_diff>
--- a/MediFind_Test_Requirements_v2.xlsx
+++ b/MediFind_Test_Requirements_v2.xlsx
@@ -2749,12 +2749,16 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H25" s="40" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="I25" s="39" t="n"/>
+      <c r="H25" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I25" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-17: emulator — incoming voice call rang 45 s unanswered, screen closed; caller got call:missed</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="50" customHeight="1">
       <c r="A26" s="41" t="inlineStr">
@@ -2801,7 +2805,7 @@
       </c>
       <c r="I26" s="43" t="inlineStr">
         <is>
-          <t>2026-09-17: call_signal_e2e — responder callable only during the emergency; resolve ends the call for both (EMERGENCY_ENDED)</t>
+          <t>2026-09-17: call_signal_e2e — responder callable only during the emergency; resolve ends the call for both (EMERGENCY_ENDED); emulator: connected voice call closed on resolve</t>
         </is>
       </c>
     </row>
@@ -2888,12 +2892,16 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="H28" s="40" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="I28" s="43" t="n"/>
+      <c r="H28" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I28" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-17: emulator ↔ browser peer — voice call accepted, timer running, audio bytes flowing both ways. Fixed: offer arriving while the camera started was dropped (now queued), stuck on "Connecting…" (now polls ICE state)</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="40" customHeight="1">
       <c r="A29" s="37" t="inlineStr">
@@ -2931,12 +2939,16 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H29" s="40" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="I29" s="39" t="n"/>
+      <c r="H29" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I29" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-17: emulator ↔ browser peer — video call, remote video decoded (158 frames) and local preview shown. Fixed: emulator crash on video (run emulator without Vulkan)</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="40" customHeight="1">
       <c r="A30" s="41" t="inlineStr">
@@ -2974,12 +2986,16 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H30" s="40" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="I30" s="43" t="n"/>
+      <c r="H30" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I30" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-17: app in background — "Incoming video call / Sara Malik is calling you" notification; tapping it opens the Accept/Decline screen</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="40" customHeight="1">
       <c r="A31" s="37" t="inlineStr">
@@ -3017,12 +3033,16 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H31" s="40" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="I31" s="39" t="n"/>
+      <c r="H31" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I31" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-17: Deaf patient — chat header and tracking show only Video call; voice call refused (VIDEO_ONLY); incoming video connects with remote video</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="36" t="inlineStr">

</xml_diff>

<commit_message>
test: layout and orientation results (UX-01, UX-02)
</commit_message>
<xml_diff>
--- a/MediFind_Test_Requirements_v2.xlsx
+++ b/MediFind_Test_Requirements_v2.xlsx
@@ -970,7 +970,7 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Contact Privacy, Emergency Chat Lock, Phone Calls, In-app Voice/Video Calls, Performance &amp; AI</t>
+          <t>Contact Privacy, Emergency Chat Lock, Phone Calls, In-app Voice/Video Calls, Performance, AI &amp; Layout</t>
         </is>
       </c>
     </row>
@@ -1759,7 +1759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3286,16 +3286,118 @@
         </is>
       </c>
     </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  LAYOUT &amp; ORIENTATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="40" customHeight="1">
+      <c r="A39" s="37" t="inlineStr">
+        <is>
+          <t>UX-01</t>
+        </is>
+      </c>
+      <c r="B39" s="38" t="inlineStr">
+        <is>
+          <t>NFR</t>
+        </is>
+      </c>
+      <c r="C39" s="39" t="inlineStr">
+        <is>
+          <t>Usability</t>
+        </is>
+      </c>
+      <c r="D39" s="39" t="inlineStr">
+        <is>
+          <t>App stays in portrait when the phone is rotated</t>
+        </is>
+      </c>
+      <c r="E39" s="39" t="inlineStr">
+        <is>
+          <t>Open the responder dashboard and rotate the phone</t>
+        </is>
+      </c>
+      <c r="F39" s="39" t="inlineStr">
+        <is>
+          <t>Screen stays portrait; nothing squeezed or cut off</t>
+        </is>
+      </c>
+      <c r="G39" s="38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H39" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I39" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18: responder app on emulator rotated to landscape stays portrait (before: dashboard squeezed into a strip)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="50" customHeight="1">
+      <c r="A40" s="41" t="inlineStr">
+        <is>
+          <t>UX-02</t>
+        </is>
+      </c>
+      <c r="B40" s="42" t="inlineStr">
+        <is>
+          <t>NFR</t>
+        </is>
+      </c>
+      <c r="C40" s="43" t="inlineStr">
+        <is>
+          <t>Usability</t>
+        </is>
+      </c>
+      <c r="D40" s="43" t="inlineStr">
+        <is>
+          <t>On a tablet or wide screen the app is centred, not stretched or stuck to one side</t>
+        </is>
+      </c>
+      <c r="E40" s="43" t="inlineStr">
+        <is>
+          <t>Open the app on a tablet (or web/desktop)</t>
+        </is>
+      </c>
+      <c r="F40" s="43" t="inlineStr">
+        <is>
+          <t>App shown as a centred column with even margins</t>
+        </is>
+      </c>
+      <c r="G40" s="42" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H40" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I40" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-18: emulator resized to 1600x2560 tablet, portrait and landscape: centred 600dp column, no stretched or one-sided layout</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A15:I15"/>
     <mergeCell ref="A11:I11"/>
     <mergeCell ref="A32:I32"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A38:I38"/>
   </mergeCells>
-  <conditionalFormatting sqref="H4:H37">
+  <conditionalFormatting sqref="H4:H40">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -3313,7 +3415,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H4:H37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid status" error="Choose PASS, FAIL, PENDING, BLOCKED or N/A" type="list">
+    <dataValidation sqref="H4:H40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid status" error="Choose PASS, FAIL, PENDING, BLOCKED or N/A" type="list">
       <formula1>"PENDING,PASS,FAIL,BLOCKED,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7004,7 +7106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D145"/>
+  <dimension ref="A1:D147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9201,7 +9303,7 @@
     <row r="101">
       <c r="A101" s="48" t="inlineStr">
         <is>
-          <t>MED-01</t>
+          <t>UX-01</t>
         </is>
       </c>
       <c r="B101" s="48" t="inlineStr">
@@ -9211,19 +9313,19 @@
       </c>
       <c r="C101" s="48" t="inlineStr">
         <is>
-          <t>Patient creates and edits the medical profile</t>
+          <t>App stays in portrait when the phone is rotated</t>
         </is>
       </c>
       <c r="D101" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.1, FR2.2</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="48" t="inlineStr">
         <is>
-          <t>MED-02</t>
+          <t>UX-02</t>
         </is>
       </c>
       <c r="B102" s="48" t="inlineStr">
@@ -9233,19 +9335,19 @@
       </c>
       <c r="C102" s="48" t="inlineStr">
         <is>
-          <t>Saving the medical profile keeps emergency contacts and quick phrases</t>
+          <t>On a tablet or wide screen the app is centred, not stretched or stuck to one side</t>
         </is>
       </c>
       <c r="D102" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.1</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="48" t="inlineStr">
         <is>
-          <t>MED-03</t>
+          <t>MED-01</t>
         </is>
       </c>
       <c r="B103" s="48" t="inlineStr">
@@ -9255,19 +9357,19 @@
       </c>
       <c r="C103" s="48" t="inlineStr">
         <is>
-          <t>Patient adds, calls and deletes emergency contacts</t>
+          <t>Patient creates and edits the medical profile</t>
         </is>
       </c>
       <c r="D103" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.1</t>
+          <t>New sheet MEDICAL; SRS FR2.1, FR2.2</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="48" t="inlineStr">
         <is>
-          <t>MED-04</t>
+          <t>MED-02</t>
         </is>
       </c>
       <c r="B104" s="48" t="inlineStr">
@@ -9277,19 +9379,19 @@
       </c>
       <c r="C104" s="48" t="inlineStr">
         <is>
-          <t>Sensitive medical fields are encrypted at rest</t>
+          <t>Saving the medical profile keeps emergency contacts and quick phrases</t>
         </is>
       </c>
       <c r="D104" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.2</t>
+          <t>New sheet MEDICAL; SRS FR2.1</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="48" t="inlineStr">
         <is>
-          <t>MED-05</t>
+          <t>MED-03</t>
         </is>
       </c>
       <c r="B105" s="48" t="inlineStr">
@@ -9299,19 +9401,19 @@
       </c>
       <c r="C105" s="48" t="inlineStr">
         <is>
-          <t>Upload a report from camera, gallery (image) and PDF</t>
+          <t>Patient adds, calls and deletes emergency contacts</t>
         </is>
       </c>
       <c r="D105" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.3</t>
+          <t>New sheet MEDICAL; SRS FR2.1</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="48" t="inlineStr">
         <is>
-          <t>MED-06</t>
+          <t>MED-04</t>
         </is>
       </c>
       <c r="B106" s="48" t="inlineStr">
@@ -9321,19 +9423,19 @@
       </c>
       <c r="C106" s="48" t="inlineStr">
         <is>
-          <t>Unsupported or oversized files are rejected with a clear message</t>
+          <t>Sensitive medical fields are encrypted at rest</t>
         </is>
       </c>
       <c r="D106" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.3</t>
+          <t>New sheet MEDICAL; SRS FR2.2</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="48" t="inlineStr">
         <is>
-          <t>MED-07</t>
+          <t>MED-05</t>
         </is>
       </c>
       <c r="B107" s="48" t="inlineStr">
@@ -9343,19 +9445,19 @@
       </c>
       <c r="C107" s="48" t="inlineStr">
         <is>
-          <t>View, rename and delete a report</t>
+          <t>Upload a report from camera, gallery (image) and PDF</t>
         </is>
       </c>
       <c r="D107" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.4</t>
+          <t>New sheet MEDICAL; SRS FR2.3</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="48" t="inlineStr">
         <is>
-          <t>MED-08</t>
+          <t>MED-06</t>
         </is>
       </c>
       <c r="B108" s="48" t="inlineStr">
@@ -9365,19 +9467,19 @@
       </c>
       <c r="C108" s="48" t="inlineStr">
         <is>
-          <t>Assigned responder receives the patient medical summary on accept</t>
+          <t>Unsupported or oversized files are rejected with a clear message</t>
         </is>
       </c>
       <c r="D108" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.5</t>
+          <t>New sheet MEDICAL; SRS FR2.3</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="48" t="inlineStr">
         <is>
-          <t>MED-09</t>
+          <t>MED-07</t>
         </is>
       </c>
       <c r="B109" s="48" t="inlineStr">
@@ -9387,19 +9489,19 @@
       </c>
       <c r="C109" s="48" t="inlineStr">
         <is>
-          <t>Report files are visible only to the patient, linked caregivers, the active responder and admins</t>
+          <t>View, rename and delete a report</t>
         </is>
       </c>
       <c r="D109" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.6</t>
+          <t>New sheet MEDICAL; SRS FR2.4</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="48" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>MED-08</t>
         </is>
       </c>
       <c r="B110" s="48" t="inlineStr">
@@ -9409,19 +9511,19 @@
       </c>
       <c r="C110" s="48" t="inlineStr">
         <is>
-          <t>SOS requires press-and-hold before it starts</t>
+          <t>Assigned responder receives the patient medical summary on accept</t>
         </is>
       </c>
       <c r="D110" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.1</t>
+          <t>New sheet MEDICAL; SRS FR2.5</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="48" t="inlineStr">
         <is>
-          <t>SEC-02</t>
+          <t>MED-09</t>
         </is>
       </c>
       <c r="B111" s="48" t="inlineStr">
@@ -9431,19 +9533,19 @@
       </c>
       <c r="C111" s="48" t="inlineStr">
         <is>
-          <t>Cancelling during the 60-second countdown sends nothing to the server</t>
+          <t>Report files are visible only to the patient, linked caregivers, the active responder and admins</t>
         </is>
       </c>
       <c r="D111" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.3</t>
+          <t>New sheet MEDICAL; SRS FR2.6</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="48" t="inlineStr">
         <is>
-          <t>SEC-03</t>
+          <t>SEC-01</t>
         </is>
       </c>
       <c r="B112" s="48" t="inlineStr">
@@ -9453,19 +9555,19 @@
       </c>
       <c r="C112" s="48" t="inlineStr">
         <is>
-          <t>SOS from a mock (fake) GPS location is refused in production</t>
+          <t>SOS requires press-and-hold before it starts</t>
         </is>
       </c>
       <c r="D112" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.1</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="48" t="inlineStr">
         <is>
-          <t>SEC-04</t>
+          <t>SEC-02</t>
         </is>
       </c>
       <c r="B113" s="48" t="inlineStr">
@@ -9475,19 +9577,19 @@
       </c>
       <c r="C113" s="48" t="inlineStr">
         <is>
-          <t>More than 5 SOS in one hour is refused</t>
+          <t>Cancelling during the 60-second countdown sends nothing to the server</t>
         </is>
       </c>
       <c r="D113" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.5</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.3</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="48" t="inlineStr">
         <is>
-          <t>SEC-05</t>
+          <t>SEC-03</t>
         </is>
       </c>
       <c r="B114" s="48" t="inlineStr">
@@ -9497,7 +9599,7 @@
       </c>
       <c r="C114" s="48" t="inlineStr">
         <is>
-          <t>SOS outside Pakistan coordinates is refused</t>
+          <t>SOS from a mock (fake) GPS location is refused in production</t>
         </is>
       </c>
       <c r="D114" s="48" t="inlineStr">
@@ -9509,7 +9611,7 @@
     <row r="115">
       <c r="A115" s="48" t="inlineStr">
         <is>
-          <t>SEC-06</t>
+          <t>SEC-04</t>
         </is>
       </c>
       <c r="B115" s="48" t="inlineStr">
@@ -9519,19 +9621,19 @@
       </c>
       <c r="C115" s="48" t="inlineStr">
         <is>
-          <t>Responder must add a note when closing as False alarm or Patient not found</t>
+          <t>More than 5 SOS in one hour is refused</t>
         </is>
       </c>
       <c r="D115" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR6.2</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.5</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="48" t="inlineStr">
         <is>
-          <t>SEC-07</t>
+          <t>SEC-05</t>
         </is>
       </c>
       <c r="B116" s="48" t="inlineStr">
@@ -9541,19 +9643,19 @@
       </c>
       <c r="C116" s="48" t="inlineStr">
         <is>
-          <t>Patient is warned when an SOS is marked as a false alarm</t>
+          <t>SOS outside Pakistan coordinates is refused</t>
         </is>
       </c>
       <c r="D116" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; beyond SRS</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="48" t="inlineStr">
         <is>
-          <t>SEC-08</t>
+          <t>SEC-06</t>
         </is>
       </c>
       <c r="B117" s="48" t="inlineStr">
@@ -9563,19 +9665,19 @@
       </c>
       <c r="C117" s="48" t="inlineStr">
         <is>
-          <t>3 false alarms in 30 days alerts admins for review</t>
+          <t>Responder must add a note when closing as False alarm or Patient not found</t>
         </is>
       </c>
       <c r="D117" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; beyond SRS</t>
+          <t>New sheet SECURITY_SOS; SRS FR6.2</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="48" t="inlineStr">
         <is>
-          <t>SEC-09</t>
+          <t>SEC-07</t>
         </is>
       </c>
       <c r="B118" s="48" t="inlineStr">
@@ -9585,7 +9687,7 @@
       </c>
       <c r="C118" s="48" t="inlineStr">
         <is>
-          <t>Patient-cancelled SOS never counts as a false alarm</t>
+          <t>Patient is warned when an SOS is marked as a false alarm</t>
         </is>
       </c>
       <c r="D118" s="48" t="inlineStr">
@@ -9597,7 +9699,7 @@
     <row r="119">
       <c r="A119" s="48" t="inlineStr">
         <is>
-          <t>SEC-10</t>
+          <t>SEC-08</t>
         </is>
       </c>
       <c r="B119" s="48" t="inlineStr">
@@ -9607,19 +9709,19 @@
       </c>
       <c r="C119" s="48" t="inlineStr">
         <is>
-          <t>Refresh token cannot be used as an access token</t>
+          <t>3 false alarms in 30 days alerts admins for review</t>
         </is>
       </c>
       <c r="D119" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
+          <t>New sheet SECURITY_SOS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="48" t="inlineStr">
         <is>
-          <t>SEC-11</t>
+          <t>SEC-09</t>
         </is>
       </c>
       <c r="B120" s="48" t="inlineStr">
@@ -9629,19 +9731,19 @@
       </c>
       <c r="C120" s="48" t="inlineStr">
         <is>
-          <t>Users cannot join emergency or chat rooms they do not belong to</t>
+          <t>Patient-cancelled SOS never counts as a false alarm</t>
         </is>
       </c>
       <c r="D120" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
+          <t>New sheet SECURITY_SOS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="48" t="inlineStr">
         <is>
-          <t>SEC-12</t>
+          <t>SEC-10</t>
         </is>
       </c>
       <c r="B121" s="48" t="inlineStr">
@@ -9651,19 +9753,19 @@
       </c>
       <c r="C121" s="48" t="inlineStr">
         <is>
-          <t>Paid plan upgrade requires a verified Stripe payment</t>
+          <t>Refresh token cannot be used as an access token</t>
         </is>
       </c>
       <c r="D121" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; beyond SRS</t>
+          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="48" t="inlineStr">
         <is>
-          <t>SEC-13</t>
+          <t>SEC-11</t>
         </is>
       </c>
       <c r="B122" s="48" t="inlineStr">
@@ -9673,19 +9775,19 @@
       </c>
       <c r="C122" s="48" t="inlineStr">
         <is>
-          <t>Only the assigned responder can update or resolve an emergency</t>
+          <t>Users cannot join emergency or chat rooms they do not belong to</t>
         </is>
       </c>
       <c r="D122" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR5.1</t>
+          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="48" t="inlineStr">
         <is>
-          <t>NAV-01</t>
+          <t>SEC-12</t>
         </is>
       </c>
       <c r="B123" s="48" t="inlineStr">
@@ -9695,19 +9797,19 @@
       </c>
       <c r="C123" s="48" t="inlineStr">
         <is>
-          <t>Each role has a unified sidebar (AppDrawer) with role-specific items</t>
+          <t>Paid plan upgrade requires a verified Stripe payment</t>
         </is>
       </c>
       <c r="D123" s="48" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.1</t>
+          <t>New sheet SECURITY_SOS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="48" t="inlineStr">
         <is>
-          <t>NAV-02</t>
+          <t>SEC-13</t>
         </is>
       </c>
       <c r="B124" s="48" t="inlineStr">
@@ -9717,19 +9819,19 @@
       </c>
       <c r="C124" s="48" t="inlineStr">
         <is>
-          <t>Switching tabs preserves each tab's state and back navigation works</t>
+          <t>Only the assigned responder can update or resolve an emergency</t>
         </is>
       </c>
       <c r="D124" s="48" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.2</t>
+          <t>New sheet SECURITY_SOS; SRS FR5.1</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="48" t="inlineStr">
         <is>
-          <t>NAV-03</t>
+          <t>NAV-01</t>
         </is>
       </c>
       <c r="B125" s="48" t="inlineStr">
@@ -9739,19 +9841,19 @@
       </c>
       <c r="C125" s="48" t="inlineStr">
         <is>
-          <t>Role dashboards show quick action grids</t>
+          <t>Each role has a unified sidebar (AppDrawer) with role-specific items</t>
         </is>
       </c>
       <c r="D125" s="48" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.3</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.1</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="48" t="inlineStr">
         <is>
-          <t>NAV-04</t>
+          <t>NAV-02</t>
         </is>
       </c>
       <c r="B126" s="48" t="inlineStr">
@@ -9761,19 +9863,19 @@
       </c>
       <c r="C126" s="48" t="inlineStr">
         <is>
-          <t>Map and chat screens render smoothly (~60 FPS)</t>
+          <t>Switching tabs preserves each tab's state and back navigation works</t>
         </is>
       </c>
       <c r="D126" s="48" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.4</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.2</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="48" t="inlineStr">
         <is>
-          <t>NAV-05</t>
+          <t>NAV-03</t>
         </is>
       </c>
       <c r="B127" s="48" t="inlineStr">
@@ -9783,63 +9885,63 @@
       </c>
       <c r="C127" s="48" t="inlineStr">
         <is>
-          <t>Large buttons mode enlarges tap targets across screens</t>
+          <t>Role dashboards show quick action grids</t>
         </is>
       </c>
       <c r="D127" s="48" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR3.5</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.3</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="48" t="inlineStr">
         <is>
-          <t>PRF-01</t>
+          <t>NAV-04</t>
         </is>
       </c>
       <c r="B128" s="48" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C128" s="48" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Map and chat screens render smoothly (~60 FPS)</t>
         </is>
       </c>
       <c r="D128" s="48" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.4</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="48" t="inlineStr">
         <is>
-          <t>PRF-02</t>
+          <t>NAV-05</t>
         </is>
       </c>
       <c r="B129" s="48" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C129" s="48" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Large buttons mode enlarges tap targets across screens</t>
         </is>
       </c>
       <c r="D129" s="48" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR3.5</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="48" t="inlineStr">
         <is>
-          <t>PRF-03</t>
+          <t>PRF-01</t>
         </is>
       </c>
       <c r="B130" s="48" t="inlineStr">
@@ -9861,7 +9963,7 @@
     <row r="131">
       <c r="A131" s="48" t="inlineStr">
         <is>
-          <t>PRF-05</t>
+          <t>PRF-02</t>
         </is>
       </c>
       <c r="B131" s="48" t="inlineStr">
@@ -9883,7 +9985,7 @@
     <row r="132">
       <c r="A132" s="48" t="inlineStr">
         <is>
-          <t>NTF-01</t>
+          <t>PRF-03</t>
         </is>
       </c>
       <c r="B132" s="48" t="inlineStr">
@@ -9905,7 +10007,7 @@
     <row r="133">
       <c r="A133" s="48" t="inlineStr">
         <is>
-          <t>NTF-02</t>
+          <t>PRF-05</t>
         </is>
       </c>
       <c r="B133" s="48" t="inlineStr">
@@ -9927,7 +10029,7 @@
     <row r="134">
       <c r="A134" s="48" t="inlineStr">
         <is>
-          <t>NTF-03</t>
+          <t>NTF-01</t>
         </is>
       </c>
       <c r="B134" s="48" t="inlineStr">
@@ -9949,7 +10051,7 @@
     <row r="135">
       <c r="A135" s="48" t="inlineStr">
         <is>
-          <t>NTF-04</t>
+          <t>NTF-02</t>
         </is>
       </c>
       <c r="B135" s="48" t="inlineStr">
@@ -9971,7 +10073,7 @@
     <row r="136">
       <c r="A136" s="48" t="inlineStr">
         <is>
-          <t>NTF-05</t>
+          <t>NTF-03</t>
         </is>
       </c>
       <c r="B136" s="48" t="inlineStr">
@@ -9993,7 +10095,7 @@
     <row r="137">
       <c r="A137" s="48" t="inlineStr">
         <is>
-          <t>NTF-07</t>
+          <t>NTF-04</t>
         </is>
       </c>
       <c r="B137" s="48" t="inlineStr">
@@ -10015,7 +10117,7 @@
     <row r="138">
       <c r="A138" s="48" t="inlineStr">
         <is>
-          <t>NTF-08</t>
+          <t>NTF-05</t>
         </is>
       </c>
       <c r="B138" s="48" t="inlineStr">
@@ -10037,7 +10139,7 @@
     <row r="139">
       <c r="A139" s="48" t="inlineStr">
         <is>
-          <t>ACC-06</t>
+          <t>NTF-07</t>
         </is>
       </c>
       <c r="B139" s="48" t="inlineStr">
@@ -10059,7 +10161,7 @@
     <row r="140">
       <c r="A140" s="48" t="inlineStr">
         <is>
-          <t>ACC-07</t>
+          <t>NTF-08</t>
         </is>
       </c>
       <c r="B140" s="48" t="inlineStr">
@@ -10081,7 +10183,7 @@
     <row r="141">
       <c r="A141" s="48" t="inlineStr">
         <is>
-          <t>ACC-11</t>
+          <t>ACC-06</t>
         </is>
       </c>
       <c r="B141" s="48" t="inlineStr">
@@ -10103,7 +10205,7 @@
     <row r="142">
       <c r="A142" s="48" t="inlineStr">
         <is>
-          <t>AUTH-12</t>
+          <t>ACC-07</t>
         </is>
       </c>
       <c r="B142" s="48" t="inlineStr">
@@ -10125,7 +10227,7 @@
     <row r="143">
       <c r="A143" s="48" t="inlineStr">
         <is>
-          <t>API-04</t>
+          <t>ACC-11</t>
         </is>
       </c>
       <c r="B143" s="48" t="inlineStr">
@@ -10147,7 +10249,7 @@
     <row r="144">
       <c r="A144" s="48" t="inlineStr">
         <is>
-          <t>API-08</t>
+          <t>AUTH-12</t>
         </is>
       </c>
       <c r="B144" s="48" t="inlineStr">
@@ -10169,20 +10271,64 @@
     <row r="145">
       <c r="A145" s="48" t="inlineStr">
         <is>
+          <t>API-04</t>
+        </is>
+      </c>
+      <c r="B145" s="48" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C145" s="48" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D145" s="48" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="48" t="inlineStr">
+        <is>
+          <t>API-08</t>
+        </is>
+      </c>
+      <c r="B146" s="48" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C146" s="48" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D146" s="48" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="48" t="inlineStr">
+        <is>
           <t>API-09</t>
         </is>
       </c>
-      <c r="B145" s="48" t="inlineStr">
+      <c r="B147" s="48" t="inlineStr">
         <is>
           <t>Re-classified</t>
         </is>
       </c>
-      <c r="C145" s="48" t="inlineStr">
+      <c r="C147" s="48" t="inlineStr">
         <is>
           <t>Marked "Beyond SRS" in the SRS Ref column</t>
         </is>
       </c>
-      <c r="D145" s="48" t="inlineStr">
+      <c r="D147" s="48" t="inlineStr">
         <is>
           <t>Valid feature test with no matching SRS functional requirement</t>
         </is>
@@ -10546,27 +10692,27 @@
         </is>
       </c>
       <c r="C11" s="19">
-        <f>COUNTA(PRIVACY_CALLS!$A$4:$A$37)-COUNTIF(PRIVACY_CALLS!$A$4:$A$37,"  *")</f>
+        <f>COUNTA(PRIVACY_CALLS!$A$4:$A$40)-COUNTIF(PRIVACY_CALLS!$A$4:$A$40,"  *")</f>
         <v/>
       </c>
       <c r="D11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$37,"PASS")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$40,"PASS")</f>
         <v/>
       </c>
       <c r="E11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$37,"FAIL")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$40,"FAIL")</f>
         <v/>
       </c>
       <c r="F11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$37,"PENDING")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$40,"PENDING")</f>
         <v/>
       </c>
       <c r="G11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$37,"BLOCKED")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$40,"BLOCKED")</f>
         <v/>
       </c>
       <c r="H11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$37,"N/A")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$40,"N/A")</f>
         <v/>
       </c>
       <c r="I11" s="21">
@@ -10926,7 +11072,7 @@
         </is>
       </c>
       <c r="D3" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR1.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR1.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.1*")</f>
         <v/>
       </c>
       <c r="E3" s="29">
@@ -10956,7 +11102,7 @@
         </is>
       </c>
       <c r="D4" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR1.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR1.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.2*")</f>
         <v/>
       </c>
       <c r="E4" s="32">
@@ -10986,7 +11132,7 @@
         </is>
       </c>
       <c r="D5" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR1.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR1.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.3*")</f>
         <v/>
       </c>
       <c r="E5" s="29">
@@ -11016,7 +11162,7 @@
         </is>
       </c>
       <c r="D6" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR1.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR1.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.4*")</f>
         <v/>
       </c>
       <c r="E6" s="32">
@@ -11046,7 +11192,7 @@
         </is>
       </c>
       <c r="D7" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR1.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR1.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.5*")</f>
         <v/>
       </c>
       <c r="E7" s="29">
@@ -11076,7 +11222,7 @@
         </is>
       </c>
       <c r="D8" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR1.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR1.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.6*")</f>
         <v/>
       </c>
       <c r="E8" s="32">
@@ -11106,7 +11252,7 @@
         </is>
       </c>
       <c r="D9" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR2.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR2.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.1*")</f>
         <v/>
       </c>
       <c r="E9" s="29">
@@ -11136,7 +11282,7 @@
         </is>
       </c>
       <c r="D10" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR2.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR2.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.2*")</f>
         <v/>
       </c>
       <c r="E10" s="32">
@@ -11166,7 +11312,7 @@
         </is>
       </c>
       <c r="D11" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR2.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR2.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.3*")</f>
         <v/>
       </c>
       <c r="E11" s="29">
@@ -11196,7 +11342,7 @@
         </is>
       </c>
       <c r="D12" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR2.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR2.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.4*")</f>
         <v/>
       </c>
       <c r="E12" s="32">
@@ -11226,7 +11372,7 @@
         </is>
       </c>
       <c r="D13" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR2.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR2.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.5*")</f>
         <v/>
       </c>
       <c r="E13" s="29">
@@ -11256,7 +11402,7 @@
         </is>
       </c>
       <c r="D14" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR2.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR2.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.6*")</f>
         <v/>
       </c>
       <c r="E14" s="32">
@@ -11286,7 +11432,7 @@
         </is>
       </c>
       <c r="D15" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR3.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR3.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.1*")</f>
         <v/>
       </c>
       <c r="E15" s="29">
@@ -11316,7 +11462,7 @@
         </is>
       </c>
       <c r="D16" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR3.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR3.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.2*")</f>
         <v/>
       </c>
       <c r="E16" s="32">
@@ -11346,7 +11492,7 @@
         </is>
       </c>
       <c r="D17" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR3.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR3.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.3*")</f>
         <v/>
       </c>
       <c r="E17" s="29">
@@ -11376,7 +11522,7 @@
         </is>
       </c>
       <c r="D18" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR3.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR3.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.4*")</f>
         <v/>
       </c>
       <c r="E18" s="32">
@@ -11406,7 +11552,7 @@
         </is>
       </c>
       <c r="D19" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR3.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR3.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.5*")</f>
         <v/>
       </c>
       <c r="E19" s="29">
@@ -11436,7 +11582,7 @@
         </is>
       </c>
       <c r="D20" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR4.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR4.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.1*")</f>
         <v/>
       </c>
       <c r="E20" s="32">
@@ -11466,7 +11612,7 @@
         </is>
       </c>
       <c r="D21" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR4.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR4.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.2*")</f>
         <v/>
       </c>
       <c r="E21" s="29">
@@ -11496,7 +11642,7 @@
         </is>
       </c>
       <c r="D22" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR4.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR4.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.3*")</f>
         <v/>
       </c>
       <c r="E22" s="32">
@@ -11526,7 +11672,7 @@
         </is>
       </c>
       <c r="D23" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR4.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR4.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.4*")</f>
         <v/>
       </c>
       <c r="E23" s="29">
@@ -11556,7 +11702,7 @@
         </is>
       </c>
       <c r="D24" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR4.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR4.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.5*")</f>
         <v/>
       </c>
       <c r="E24" s="32">
@@ -11586,7 +11732,7 @@
         </is>
       </c>
       <c r="D25" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR4.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR4.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.6*")</f>
         <v/>
       </c>
       <c r="E25" s="29">
@@ -11616,7 +11762,7 @@
         </is>
       </c>
       <c r="D26" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR5.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR5.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.1*")</f>
         <v/>
       </c>
       <c r="E26" s="32">
@@ -11646,7 +11792,7 @@
         </is>
       </c>
       <c r="D27" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR5.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR5.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.2*")</f>
         <v/>
       </c>
       <c r="E27" s="29">
@@ -11676,7 +11822,7 @@
         </is>
       </c>
       <c r="D28" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR5.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR5.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.3*")</f>
         <v/>
       </c>
       <c r="E28" s="32">
@@ -11706,7 +11852,7 @@
         </is>
       </c>
       <c r="D29" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR5.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR5.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.4*")</f>
         <v/>
       </c>
       <c r="E29" s="29">
@@ -11736,7 +11882,7 @@
         </is>
       </c>
       <c r="D30" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR6.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR6.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.1*")</f>
         <v/>
       </c>
       <c r="E30" s="32">
@@ -11766,7 +11912,7 @@
         </is>
       </c>
       <c r="D31" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR6.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR6.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.2*")</f>
         <v/>
       </c>
       <c r="E31" s="29">
@@ -11796,7 +11942,7 @@
         </is>
       </c>
       <c r="D32" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR6.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR6.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.3*")</f>
         <v/>
       </c>
       <c r="E32" s="32">
@@ -11826,7 +11972,7 @@
         </is>
       </c>
       <c r="D33" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR6.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR6.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.4*")</f>
         <v/>
       </c>
       <c r="E33" s="29">
@@ -11856,7 +12002,7 @@
         </is>
       </c>
       <c r="D34" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR7.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR7.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.1*")</f>
         <v/>
       </c>
       <c r="E34" s="32">
@@ -11886,7 +12032,7 @@
         </is>
       </c>
       <c r="D35" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR7.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR7.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.2*")</f>
         <v/>
       </c>
       <c r="E35" s="29">
@@ -11916,7 +12062,7 @@
         </is>
       </c>
       <c r="D36" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR7.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR7.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.3*")</f>
         <v/>
       </c>
       <c r="E36" s="32">
@@ -11946,7 +12092,7 @@
         </is>
       </c>
       <c r="D37" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR7.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR7.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.4*")</f>
         <v/>
       </c>
       <c r="E37" s="29">
@@ -11976,7 +12122,7 @@
         </is>
       </c>
       <c r="D38" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR7.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR7.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.5*")</f>
         <v/>
       </c>
       <c r="E38" s="32">
@@ -12006,7 +12152,7 @@
         </is>
       </c>
       <c r="D39" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR8.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR8.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.1*")</f>
         <v/>
       </c>
       <c r="E39" s="29">
@@ -12036,7 +12182,7 @@
         </is>
       </c>
       <c r="D40" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR8.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR8.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.2*")</f>
         <v/>
       </c>
       <c r="E40" s="32">
@@ -12066,7 +12212,7 @@
         </is>
       </c>
       <c r="D41" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR8.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR8.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.3*")</f>
         <v/>
       </c>
       <c r="E41" s="29">
@@ -12096,7 +12242,7 @@
         </is>
       </c>
       <c r="D42" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR8.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR8.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.4*")</f>
         <v/>
       </c>
       <c r="E42" s="32">
@@ -12126,7 +12272,7 @@
         </is>
       </c>
       <c r="D43" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR9.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR9.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.1*")</f>
         <v/>
       </c>
       <c r="E43" s="29">
@@ -12156,7 +12302,7 @@
         </is>
       </c>
       <c r="D44" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR9.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR9.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.2*")</f>
         <v/>
       </c>
       <c r="E44" s="32">
@@ -12186,7 +12332,7 @@
         </is>
       </c>
       <c r="D45" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR9.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR9.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.3*")</f>
         <v/>
       </c>
       <c r="E45" s="29">
@@ -12216,7 +12362,7 @@
         </is>
       </c>
       <c r="D46" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR9.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR9.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.4*")</f>
         <v/>
       </c>
       <c r="E46" s="32">
@@ -12246,7 +12392,7 @@
         </is>
       </c>
       <c r="D47" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR9.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR9.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.5*")</f>
         <v/>
       </c>
       <c r="E47" s="29">
@@ -12276,7 +12422,7 @@
         </is>
       </c>
       <c r="D48" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR9.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR9.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.6*")</f>
         <v/>
       </c>
       <c r="E48" s="32">
@@ -12306,7 +12452,7 @@
         </is>
       </c>
       <c r="D49" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.7*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.7*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.7*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.7*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.7*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.7*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.7*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$37,"*FR9.7*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.7*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.7*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.7*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.7*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.7*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.7*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.7*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.7*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.7*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.7*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.7*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.7*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.7*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR9.7*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.7*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.7*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.7*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.7*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.7*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.7*")</f>
         <v/>
       </c>
       <c r="E49" s="29">

</xml_diff>

<commit_message>
test: payment speed, test transaction and logo consistency results
</commit_message>
<xml_diff>
--- a/MediFind_Test_Requirements_v2.xlsx
+++ b/MediFind_Test_Requirements_v2.xlsx
@@ -970,7 +970,7 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Contact Privacy, Emergency Chat Lock, Phone Calls, In-app Voice/Video Calls, Performance, AI &amp; Layout</t>
+          <t>Contact Privacy, Emergency Chat Lock, Phone Calls, In-app Voice/Video Calls, Performance, AI, Payments &amp; Layout</t>
         </is>
       </c>
     </row>
@@ -1759,7 +1759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3289,115 +3289,311 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  LAYOUT &amp; ORIENTATION</t>
+          <t xml:space="preserve">  PAYMENTS (STRIPE SANDBOX)</t>
         </is>
       </c>
     </row>
     <row r="39" ht="40" customHeight="1">
       <c r="A39" s="37" t="inlineStr">
         <is>
+          <t>PAY-01</t>
+        </is>
+      </c>
+      <c r="B39" s="44" t="inlineStr">
+        <is>
+          <t>Beyond SRS</t>
+        </is>
+      </c>
+      <c r="C39" s="39" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="D39" s="39" t="inlineStr">
+        <is>
+          <t>Stripe card form opens quickly after tapping Pay</t>
+        </is>
+      </c>
+      <c r="E39" s="39" t="inlineStr">
+        <is>
+          <t>Open checkout for a paid plan, wait a moment, tap Pay</t>
+        </is>
+      </c>
+      <c r="F39" s="39" t="inlineStr">
+        <is>
+          <t>Card form ready within ~5 s on the emulator (no long spinner)</t>
+        </is>
+      </c>
+      <c r="G39" s="38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H39" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I39" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18: emulator — Pay tap to card form ~4.8 s (was ~9.5 s: intent + sheet now prepared when checkout opens, FlowController)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="40" customHeight="1">
+      <c r="A40" s="41" t="inlineStr">
+        <is>
+          <t>PAY-02</t>
+        </is>
+      </c>
+      <c r="B40" s="46" t="inlineStr">
+        <is>
+          <t>Beyond SRS</t>
+        </is>
+      </c>
+      <c r="C40" s="43" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="D40" s="43" t="inlineStr">
+        <is>
+          <t>Test card payment upgrades the plan</t>
+        </is>
+      </c>
+      <c r="E40" s="43" t="inlineStr">
+        <is>
+          <t>Pay with 4242 4242 4242 4242, any future date, any CVC</t>
+        </is>
+      </c>
+      <c r="F40" s="43" t="inlineStr">
+        <is>
+          <t>Payment successful screen with receipt; plan upgraded on the server</t>
+        </is>
+      </c>
+      <c r="G40" s="42" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="H40" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I40" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-18: test card 4242 → "Payment successful" ~4.5 s after Continue; receipt shown; user plan FREE → PROFESSIONAL (demo reset after)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="40" customHeight="1">
+      <c r="A41" s="37" t="inlineStr">
+        <is>
+          <t>PAY-03</t>
+        </is>
+      </c>
+      <c r="B41" s="44" t="inlineStr">
+        <is>
+          <t>Beyond SRS</t>
+        </is>
+      </c>
+      <c r="C41" s="39" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="D41" s="39" t="inlineStr">
+        <is>
+          <t>Cancelling the payment sheet does not charge</t>
+        </is>
+      </c>
+      <c r="E41" s="39" t="inlineStr">
+        <is>
+          <t>Open the sheet and close it</t>
+        </is>
+      </c>
+      <c r="F41" s="39" t="inlineStr">
+        <is>
+          <t>Message: payment cancelled, not charged; Pay works again</t>
+        </is>
+      </c>
+      <c r="G41" s="38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H41" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I41" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18: closing the sheet shows "Payment cancelled. You have not been charged."; Pay again opens a fresh prepared sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  LAYOUT &amp; ORIENTATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="40" customHeight="1">
+      <c r="A43" s="37" t="inlineStr">
+        <is>
           <t>UX-01</t>
         </is>
       </c>
-      <c r="B39" s="38" t="inlineStr">
+      <c r="B43" s="38" t="inlineStr">
         <is>
           <t>NFR</t>
         </is>
       </c>
-      <c r="C39" s="39" t="inlineStr">
+      <c r="C43" s="39" t="inlineStr">
         <is>
           <t>Usability</t>
         </is>
       </c>
-      <c r="D39" s="39" t="inlineStr">
+      <c r="D43" s="39" t="inlineStr">
         <is>
           <t>App stays in portrait when the phone is rotated</t>
         </is>
       </c>
-      <c r="E39" s="39" t="inlineStr">
+      <c r="E43" s="39" t="inlineStr">
         <is>
           <t>Open the responder dashboard and rotate the phone</t>
         </is>
       </c>
-      <c r="F39" s="39" t="inlineStr">
+      <c r="F43" s="39" t="inlineStr">
         <is>
           <t>Screen stays portrait; nothing squeezed or cut off</t>
         </is>
       </c>
-      <c r="G39" s="38" t="inlineStr">
+      <c r="G43" s="38" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H39" s="45" t="inlineStr">
+      <c r="H43" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I39" s="39" t="inlineStr">
+      <c r="I43" s="39" t="inlineStr">
         <is>
           <t>2026-09-18: responder app on emulator rotated to landscape stays portrait (before: dashboard squeezed into a strip)</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="50" customHeight="1">
-      <c r="A40" s="41" t="inlineStr">
+    <row r="44" ht="50" customHeight="1">
+      <c r="A44" s="41" t="inlineStr">
         <is>
           <t>UX-02</t>
         </is>
       </c>
-      <c r="B40" s="42" t="inlineStr">
+      <c r="B44" s="42" t="inlineStr">
         <is>
           <t>NFR</t>
         </is>
       </c>
-      <c r="C40" s="43" t="inlineStr">
+      <c r="C44" s="43" t="inlineStr">
         <is>
           <t>Usability</t>
         </is>
       </c>
-      <c r="D40" s="43" t="inlineStr">
+      <c r="D44" s="43" t="inlineStr">
         <is>
           <t>On a tablet or wide screen the app is centred, not stretched or stuck to one side</t>
         </is>
       </c>
-      <c r="E40" s="43" t="inlineStr">
+      <c r="E44" s="43" t="inlineStr">
         <is>
           <t>Open the app on a tablet (or web/desktop)</t>
         </is>
       </c>
-      <c r="F40" s="43" t="inlineStr">
+      <c r="F44" s="43" t="inlineStr">
         <is>
           <t>App shown as a centred column with even margins</t>
         </is>
       </c>
-      <c r="G40" s="42" t="inlineStr">
+      <c r="G44" s="42" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H40" s="45" t="inlineStr">
+      <c r="H44" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I40" s="43" t="inlineStr">
+      <c r="I44" s="43" t="inlineStr">
         <is>
           <t>2026-09-18: emulator resized to 1600x2560 tablet, portrait and landscape: centred 600dp column, no stretched or one-sided layout</t>
         </is>
       </c>
     </row>
+    <row r="45" ht="40" customHeight="1">
+      <c r="A45" s="37" t="inlineStr">
+        <is>
+          <t>UX-03</t>
+        </is>
+      </c>
+      <c r="B45" s="38" t="inlineStr">
+        <is>
+          <t>NFR</t>
+        </is>
+      </c>
+      <c r="C45" s="39" t="inlineStr">
+        <is>
+          <t>Branding</t>
+        </is>
+      </c>
+      <c r="D45" s="39" t="inlineStr">
+        <is>
+          <t>The same MediFind logo is used in the mobile app and the web portal</t>
+        </is>
+      </c>
+      <c r="E45" s="39" t="inlineStr">
+        <is>
+          <t>Compare app launcher, splash, headers with portal sidebar, login, landing, 404, legal, favicon</t>
+        </is>
+      </c>
+      <c r="F45" s="39" t="inlineStr">
+        <is>
+          <t>One consistent logo everywhere</t>
+        </is>
+      </c>
+      <c r="G45" s="38" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H45" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I45" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18: portal sidebar, login, landing, 404, legal and favicon use the same pin-with-rings logo as the mobile app</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A15:I15"/>
     <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A42:I42"/>
     <mergeCell ref="A32:I32"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A20:I20"/>
     <mergeCell ref="A38:I38"/>
   </mergeCells>
-  <conditionalFormatting sqref="H4:H40">
+  <conditionalFormatting sqref="H4:H45">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -3415,7 +3611,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H4:H40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid status" error="Choose PASS, FAIL, PENDING, BLOCKED or N/A" type="list">
+    <dataValidation sqref="H4:H45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid status" error="Choose PASS, FAIL, PENDING, BLOCKED or N/A" type="list">
       <formula1>"PENDING,PASS,FAIL,BLOCKED,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7106,7 +7302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D147"/>
+  <dimension ref="A1:D151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9303,7 +9499,7 @@
     <row r="101">
       <c r="A101" s="48" t="inlineStr">
         <is>
-          <t>UX-01</t>
+          <t>PAY-01</t>
         </is>
       </c>
       <c r="B101" s="48" t="inlineStr">
@@ -9313,19 +9509,19 @@
       </c>
       <c r="C101" s="48" t="inlineStr">
         <is>
-          <t>App stays in portrait when the phone is rotated</t>
+          <t>Stripe card form opens quickly after tapping Pay</t>
         </is>
       </c>
       <c r="D101" s="48" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="48" t="inlineStr">
         <is>
-          <t>UX-02</t>
+          <t>PAY-02</t>
         </is>
       </c>
       <c r="B102" s="48" t="inlineStr">
@@ -9335,19 +9531,19 @@
       </c>
       <c r="C102" s="48" t="inlineStr">
         <is>
-          <t>On a tablet or wide screen the app is centred, not stretched or stuck to one side</t>
+          <t>Test card payment upgrades the plan</t>
         </is>
       </c>
       <c r="D102" s="48" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="48" t="inlineStr">
         <is>
-          <t>MED-01</t>
+          <t>PAY-03</t>
         </is>
       </c>
       <c r="B103" s="48" t="inlineStr">
@@ -9357,19 +9553,19 @@
       </c>
       <c r="C103" s="48" t="inlineStr">
         <is>
-          <t>Patient creates and edits the medical profile</t>
+          <t>Cancelling the payment sheet does not charge</t>
         </is>
       </c>
       <c r="D103" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.1, FR2.2</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="48" t="inlineStr">
         <is>
-          <t>MED-02</t>
+          <t>UX-01</t>
         </is>
       </c>
       <c r="B104" s="48" t="inlineStr">
@@ -9379,19 +9575,19 @@
       </c>
       <c r="C104" s="48" t="inlineStr">
         <is>
-          <t>Saving the medical profile keeps emergency contacts and quick phrases</t>
+          <t>App stays in portrait when the phone is rotated</t>
         </is>
       </c>
       <c r="D104" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.1</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="48" t="inlineStr">
         <is>
-          <t>MED-03</t>
+          <t>UX-02</t>
         </is>
       </c>
       <c r="B105" s="48" t="inlineStr">
@@ -9401,19 +9597,19 @@
       </c>
       <c r="C105" s="48" t="inlineStr">
         <is>
-          <t>Patient adds, calls and deletes emergency contacts</t>
+          <t>On a tablet or wide screen the app is centred, not stretched or stuck to one side</t>
         </is>
       </c>
       <c r="D105" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.1</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="48" t="inlineStr">
         <is>
-          <t>MED-04</t>
+          <t>UX-03</t>
         </is>
       </c>
       <c r="B106" s="48" t="inlineStr">
@@ -9423,19 +9619,19 @@
       </c>
       <c r="C106" s="48" t="inlineStr">
         <is>
-          <t>Sensitive medical fields are encrypted at rest</t>
+          <t>The same MediFind logo is used in the mobile app and the web portal</t>
         </is>
       </c>
       <c r="D106" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.2</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="48" t="inlineStr">
         <is>
-          <t>MED-05</t>
+          <t>MED-01</t>
         </is>
       </c>
       <c r="B107" s="48" t="inlineStr">
@@ -9445,19 +9641,19 @@
       </c>
       <c r="C107" s="48" t="inlineStr">
         <is>
-          <t>Upload a report from camera, gallery (image) and PDF</t>
+          <t>Patient creates and edits the medical profile</t>
         </is>
       </c>
       <c r="D107" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.3</t>
+          <t>New sheet MEDICAL; SRS FR2.1, FR2.2</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="48" t="inlineStr">
         <is>
-          <t>MED-06</t>
+          <t>MED-02</t>
         </is>
       </c>
       <c r="B108" s="48" t="inlineStr">
@@ -9467,19 +9663,19 @@
       </c>
       <c r="C108" s="48" t="inlineStr">
         <is>
-          <t>Unsupported or oversized files are rejected with a clear message</t>
+          <t>Saving the medical profile keeps emergency contacts and quick phrases</t>
         </is>
       </c>
       <c r="D108" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.3</t>
+          <t>New sheet MEDICAL; SRS FR2.1</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="48" t="inlineStr">
         <is>
-          <t>MED-07</t>
+          <t>MED-03</t>
         </is>
       </c>
       <c r="B109" s="48" t="inlineStr">
@@ -9489,19 +9685,19 @@
       </c>
       <c r="C109" s="48" t="inlineStr">
         <is>
-          <t>View, rename and delete a report</t>
+          <t>Patient adds, calls and deletes emergency contacts</t>
         </is>
       </c>
       <c r="D109" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.4</t>
+          <t>New sheet MEDICAL; SRS FR2.1</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="48" t="inlineStr">
         <is>
-          <t>MED-08</t>
+          <t>MED-04</t>
         </is>
       </c>
       <c r="B110" s="48" t="inlineStr">
@@ -9511,19 +9707,19 @@
       </c>
       <c r="C110" s="48" t="inlineStr">
         <is>
-          <t>Assigned responder receives the patient medical summary on accept</t>
+          <t>Sensitive medical fields are encrypted at rest</t>
         </is>
       </c>
       <c r="D110" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.5</t>
+          <t>New sheet MEDICAL; SRS FR2.2</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="48" t="inlineStr">
         <is>
-          <t>MED-09</t>
+          <t>MED-05</t>
         </is>
       </c>
       <c r="B111" s="48" t="inlineStr">
@@ -9533,19 +9729,19 @@
       </c>
       <c r="C111" s="48" t="inlineStr">
         <is>
-          <t>Report files are visible only to the patient, linked caregivers, the active responder and admins</t>
+          <t>Upload a report from camera, gallery (image) and PDF</t>
         </is>
       </c>
       <c r="D111" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.6</t>
+          <t>New sheet MEDICAL; SRS FR2.3</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="48" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>MED-06</t>
         </is>
       </c>
       <c r="B112" s="48" t="inlineStr">
@@ -9555,19 +9751,19 @@
       </c>
       <c r="C112" s="48" t="inlineStr">
         <is>
-          <t>SOS requires press-and-hold before it starts</t>
+          <t>Unsupported or oversized files are rejected with a clear message</t>
         </is>
       </c>
       <c r="D112" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.1</t>
+          <t>New sheet MEDICAL; SRS FR2.3</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="48" t="inlineStr">
         <is>
-          <t>SEC-02</t>
+          <t>MED-07</t>
         </is>
       </c>
       <c r="B113" s="48" t="inlineStr">
@@ -9577,19 +9773,19 @@
       </c>
       <c r="C113" s="48" t="inlineStr">
         <is>
-          <t>Cancelling during the 60-second countdown sends nothing to the server</t>
+          <t>View, rename and delete a report</t>
         </is>
       </c>
       <c r="D113" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.3</t>
+          <t>New sheet MEDICAL; SRS FR2.4</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="48" t="inlineStr">
         <is>
-          <t>SEC-03</t>
+          <t>MED-08</t>
         </is>
       </c>
       <c r="B114" s="48" t="inlineStr">
@@ -9599,19 +9795,19 @@
       </c>
       <c r="C114" s="48" t="inlineStr">
         <is>
-          <t>SOS from a mock (fake) GPS location is refused in production</t>
+          <t>Assigned responder receives the patient medical summary on accept</t>
         </is>
       </c>
       <c r="D114" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
+          <t>New sheet MEDICAL; SRS FR2.5</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="48" t="inlineStr">
         <is>
-          <t>SEC-04</t>
+          <t>MED-09</t>
         </is>
       </c>
       <c r="B115" s="48" t="inlineStr">
@@ -9621,19 +9817,19 @@
       </c>
       <c r="C115" s="48" t="inlineStr">
         <is>
-          <t>More than 5 SOS in one hour is refused</t>
+          <t>Report files are visible only to the patient, linked caregivers, the active responder and admins</t>
         </is>
       </c>
       <c r="D115" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.5</t>
+          <t>New sheet MEDICAL; SRS FR2.6</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="48" t="inlineStr">
         <is>
-          <t>SEC-05</t>
+          <t>SEC-01</t>
         </is>
       </c>
       <c r="B116" s="48" t="inlineStr">
@@ -9643,19 +9839,19 @@
       </c>
       <c r="C116" s="48" t="inlineStr">
         <is>
-          <t>SOS outside Pakistan coordinates is refused</t>
+          <t>SOS requires press-and-hold before it starts</t>
         </is>
       </c>
       <c r="D116" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.1</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="48" t="inlineStr">
         <is>
-          <t>SEC-06</t>
+          <t>SEC-02</t>
         </is>
       </c>
       <c r="B117" s="48" t="inlineStr">
@@ -9665,19 +9861,19 @@
       </c>
       <c r="C117" s="48" t="inlineStr">
         <is>
-          <t>Responder must add a note when closing as False alarm or Patient not found</t>
+          <t>Cancelling during the 60-second countdown sends nothing to the server</t>
         </is>
       </c>
       <c r="D117" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR6.2</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.3</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="48" t="inlineStr">
         <is>
-          <t>SEC-07</t>
+          <t>SEC-03</t>
         </is>
       </c>
       <c r="B118" s="48" t="inlineStr">
@@ -9687,19 +9883,19 @@
       </c>
       <c r="C118" s="48" t="inlineStr">
         <is>
-          <t>Patient is warned when an SOS is marked as a false alarm</t>
+          <t>SOS from a mock (fake) GPS location is refused in production</t>
         </is>
       </c>
       <c r="D118" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; beyond SRS</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="48" t="inlineStr">
         <is>
-          <t>SEC-08</t>
+          <t>SEC-04</t>
         </is>
       </c>
       <c r="B119" s="48" t="inlineStr">
@@ -9709,19 +9905,19 @@
       </c>
       <c r="C119" s="48" t="inlineStr">
         <is>
-          <t>3 false alarms in 30 days alerts admins for review</t>
+          <t>More than 5 SOS in one hour is refused</t>
         </is>
       </c>
       <c r="D119" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; beyond SRS</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.5</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="48" t="inlineStr">
         <is>
-          <t>SEC-09</t>
+          <t>SEC-05</t>
         </is>
       </c>
       <c r="B120" s="48" t="inlineStr">
@@ -9731,19 +9927,19 @@
       </c>
       <c r="C120" s="48" t="inlineStr">
         <is>
-          <t>Patient-cancelled SOS never counts as a false alarm</t>
+          <t>SOS outside Pakistan coordinates is refused</t>
         </is>
       </c>
       <c r="D120" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; beyond SRS</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="48" t="inlineStr">
         <is>
-          <t>SEC-10</t>
+          <t>SEC-06</t>
         </is>
       </c>
       <c r="B121" s="48" t="inlineStr">
@@ -9753,19 +9949,19 @@
       </c>
       <c r="C121" s="48" t="inlineStr">
         <is>
-          <t>Refresh token cannot be used as an access token</t>
+          <t>Responder must add a note when closing as False alarm or Patient not found</t>
         </is>
       </c>
       <c r="D121" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
+          <t>New sheet SECURITY_SOS; SRS FR6.2</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="48" t="inlineStr">
         <is>
-          <t>SEC-11</t>
+          <t>SEC-07</t>
         </is>
       </c>
       <c r="B122" s="48" t="inlineStr">
@@ -9775,19 +9971,19 @@
       </c>
       <c r="C122" s="48" t="inlineStr">
         <is>
-          <t>Users cannot join emergency or chat rooms they do not belong to</t>
+          <t>Patient is warned when an SOS is marked as a false alarm</t>
         </is>
       </c>
       <c r="D122" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
+          <t>New sheet SECURITY_SOS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="48" t="inlineStr">
         <is>
-          <t>SEC-12</t>
+          <t>SEC-08</t>
         </is>
       </c>
       <c r="B123" s="48" t="inlineStr">
@@ -9797,7 +9993,7 @@
       </c>
       <c r="C123" s="48" t="inlineStr">
         <is>
-          <t>Paid plan upgrade requires a verified Stripe payment</t>
+          <t>3 false alarms in 30 days alerts admins for review</t>
         </is>
       </c>
       <c r="D123" s="48" t="inlineStr">
@@ -9809,7 +10005,7 @@
     <row r="124">
       <c r="A124" s="48" t="inlineStr">
         <is>
-          <t>SEC-13</t>
+          <t>SEC-09</t>
         </is>
       </c>
       <c r="B124" s="48" t="inlineStr">
@@ -9819,19 +10015,19 @@
       </c>
       <c r="C124" s="48" t="inlineStr">
         <is>
-          <t>Only the assigned responder can update or resolve an emergency</t>
+          <t>Patient-cancelled SOS never counts as a false alarm</t>
         </is>
       </c>
       <c r="D124" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR5.1</t>
+          <t>New sheet SECURITY_SOS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="48" t="inlineStr">
         <is>
-          <t>NAV-01</t>
+          <t>SEC-10</t>
         </is>
       </c>
       <c r="B125" s="48" t="inlineStr">
@@ -9841,19 +10037,19 @@
       </c>
       <c r="C125" s="48" t="inlineStr">
         <is>
-          <t>Each role has a unified sidebar (AppDrawer) with role-specific items</t>
+          <t>Refresh token cannot be used as an access token</t>
         </is>
       </c>
       <c r="D125" s="48" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.1</t>
+          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="48" t="inlineStr">
         <is>
-          <t>NAV-02</t>
+          <t>SEC-11</t>
         </is>
       </c>
       <c r="B126" s="48" t="inlineStr">
@@ -9863,19 +10059,19 @@
       </c>
       <c r="C126" s="48" t="inlineStr">
         <is>
-          <t>Switching tabs preserves each tab's state and back navigation works</t>
+          <t>Users cannot join emergency or chat rooms they do not belong to</t>
         </is>
       </c>
       <c r="D126" s="48" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.2</t>
+          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="48" t="inlineStr">
         <is>
-          <t>NAV-03</t>
+          <t>SEC-12</t>
         </is>
       </c>
       <c r="B127" s="48" t="inlineStr">
@@ -9885,19 +10081,19 @@
       </c>
       <c r="C127" s="48" t="inlineStr">
         <is>
-          <t>Role dashboards show quick action grids</t>
+          <t>Paid plan upgrade requires a verified Stripe payment</t>
         </is>
       </c>
       <c r="D127" s="48" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.3</t>
+          <t>New sheet SECURITY_SOS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="48" t="inlineStr">
         <is>
-          <t>NAV-04</t>
+          <t>SEC-13</t>
         </is>
       </c>
       <c r="B128" s="48" t="inlineStr">
@@ -9907,19 +10103,19 @@
       </c>
       <c r="C128" s="48" t="inlineStr">
         <is>
-          <t>Map and chat screens render smoothly (~60 FPS)</t>
+          <t>Only the assigned responder can update or resolve an emergency</t>
         </is>
       </c>
       <c r="D128" s="48" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.4</t>
+          <t>New sheet SECURITY_SOS; SRS FR5.1</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="48" t="inlineStr">
         <is>
-          <t>NAV-05</t>
+          <t>NAV-01</t>
         </is>
       </c>
       <c r="B129" s="48" t="inlineStr">
@@ -9929,107 +10125,107 @@
       </c>
       <c r="C129" s="48" t="inlineStr">
         <is>
-          <t>Large buttons mode enlarges tap targets across screens</t>
+          <t>Each role has a unified sidebar (AppDrawer) with role-specific items</t>
         </is>
       </c>
       <c r="D129" s="48" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR3.5</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.1</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="48" t="inlineStr">
         <is>
-          <t>PRF-01</t>
+          <t>NAV-02</t>
         </is>
       </c>
       <c r="B130" s="48" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C130" s="48" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Switching tabs preserves each tab's state and back navigation works</t>
         </is>
       </c>
       <c r="D130" s="48" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.2</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="48" t="inlineStr">
         <is>
-          <t>PRF-02</t>
+          <t>NAV-03</t>
         </is>
       </c>
       <c r="B131" s="48" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C131" s="48" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Role dashboards show quick action grids</t>
         </is>
       </c>
       <c r="D131" s="48" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.3</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="48" t="inlineStr">
         <is>
-          <t>PRF-03</t>
+          <t>NAV-04</t>
         </is>
       </c>
       <c r="B132" s="48" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C132" s="48" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Map and chat screens render smoothly (~60 FPS)</t>
         </is>
       </c>
       <c r="D132" s="48" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.4</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="48" t="inlineStr">
         <is>
-          <t>PRF-05</t>
+          <t>NAV-05</t>
         </is>
       </c>
       <c r="B133" s="48" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C133" s="48" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Large buttons mode enlarges tap targets across screens</t>
         </is>
       </c>
       <c r="D133" s="48" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR3.5</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="48" t="inlineStr">
         <is>
-          <t>NTF-01</t>
+          <t>PRF-01</t>
         </is>
       </c>
       <c r="B134" s="48" t="inlineStr">
@@ -10051,7 +10247,7 @@
     <row r="135">
       <c r="A135" s="48" t="inlineStr">
         <is>
-          <t>NTF-02</t>
+          <t>PRF-02</t>
         </is>
       </c>
       <c r="B135" s="48" t="inlineStr">
@@ -10073,7 +10269,7 @@
     <row r="136">
       <c r="A136" s="48" t="inlineStr">
         <is>
-          <t>NTF-03</t>
+          <t>PRF-03</t>
         </is>
       </c>
       <c r="B136" s="48" t="inlineStr">
@@ -10095,7 +10291,7 @@
     <row r="137">
       <c r="A137" s="48" t="inlineStr">
         <is>
-          <t>NTF-04</t>
+          <t>PRF-05</t>
         </is>
       </c>
       <c r="B137" s="48" t="inlineStr">
@@ -10117,7 +10313,7 @@
     <row r="138">
       <c r="A138" s="48" t="inlineStr">
         <is>
-          <t>NTF-05</t>
+          <t>NTF-01</t>
         </is>
       </c>
       <c r="B138" s="48" t="inlineStr">
@@ -10139,7 +10335,7 @@
     <row r="139">
       <c r="A139" s="48" t="inlineStr">
         <is>
-          <t>NTF-07</t>
+          <t>NTF-02</t>
         </is>
       </c>
       <c r="B139" s="48" t="inlineStr">
@@ -10161,7 +10357,7 @@
     <row r="140">
       <c r="A140" s="48" t="inlineStr">
         <is>
-          <t>NTF-08</t>
+          <t>NTF-03</t>
         </is>
       </c>
       <c r="B140" s="48" t="inlineStr">
@@ -10183,7 +10379,7 @@
     <row r="141">
       <c r="A141" s="48" t="inlineStr">
         <is>
-          <t>ACC-06</t>
+          <t>NTF-04</t>
         </is>
       </c>
       <c r="B141" s="48" t="inlineStr">
@@ -10205,7 +10401,7 @@
     <row r="142">
       <c r="A142" s="48" t="inlineStr">
         <is>
-          <t>ACC-07</t>
+          <t>NTF-05</t>
         </is>
       </c>
       <c r="B142" s="48" t="inlineStr">
@@ -10227,7 +10423,7 @@
     <row r="143">
       <c r="A143" s="48" t="inlineStr">
         <is>
-          <t>ACC-11</t>
+          <t>NTF-07</t>
         </is>
       </c>
       <c r="B143" s="48" t="inlineStr">
@@ -10249,7 +10445,7 @@
     <row r="144">
       <c r="A144" s="48" t="inlineStr">
         <is>
-          <t>AUTH-12</t>
+          <t>NTF-08</t>
         </is>
       </c>
       <c r="B144" s="48" t="inlineStr">
@@ -10271,7 +10467,7 @@
     <row r="145">
       <c r="A145" s="48" t="inlineStr">
         <is>
-          <t>API-04</t>
+          <t>ACC-06</t>
         </is>
       </c>
       <c r="B145" s="48" t="inlineStr">
@@ -10293,7 +10489,7 @@
     <row r="146">
       <c r="A146" s="48" t="inlineStr">
         <is>
-          <t>API-08</t>
+          <t>ACC-07</t>
         </is>
       </c>
       <c r="B146" s="48" t="inlineStr">
@@ -10315,20 +10511,108 @@
     <row r="147">
       <c r="A147" s="48" t="inlineStr">
         <is>
+          <t>ACC-11</t>
+        </is>
+      </c>
+      <c r="B147" s="48" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C147" s="48" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D147" s="48" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="48" t="inlineStr">
+        <is>
+          <t>AUTH-12</t>
+        </is>
+      </c>
+      <c r="B148" s="48" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C148" s="48" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D148" s="48" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="48" t="inlineStr">
+        <is>
+          <t>API-04</t>
+        </is>
+      </c>
+      <c r="B149" s="48" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C149" s="48" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D149" s="48" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="48" t="inlineStr">
+        <is>
+          <t>API-08</t>
+        </is>
+      </c>
+      <c r="B150" s="48" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C150" s="48" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D150" s="48" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="48" t="inlineStr">
+        <is>
           <t>API-09</t>
         </is>
       </c>
-      <c r="B147" s="48" t="inlineStr">
+      <c r="B151" s="48" t="inlineStr">
         <is>
           <t>Re-classified</t>
         </is>
       </c>
-      <c r="C147" s="48" t="inlineStr">
+      <c r="C151" s="48" t="inlineStr">
         <is>
           <t>Marked "Beyond SRS" in the SRS Ref column</t>
         </is>
       </c>
-      <c r="D147" s="48" t="inlineStr">
+      <c r="D151" s="48" t="inlineStr">
         <is>
           <t>Valid feature test with no matching SRS functional requirement</t>
         </is>
@@ -10692,27 +10976,27 @@
         </is>
       </c>
       <c r="C11" s="19">
-        <f>COUNTA(PRIVACY_CALLS!$A$4:$A$40)-COUNTIF(PRIVACY_CALLS!$A$4:$A$40,"  *")</f>
+        <f>COUNTA(PRIVACY_CALLS!$A$4:$A$45)-COUNTIF(PRIVACY_CALLS!$A$4:$A$45,"  *")</f>
         <v/>
       </c>
       <c r="D11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$40,"PASS")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$45,"PASS")</f>
         <v/>
       </c>
       <c r="E11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$40,"FAIL")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$45,"FAIL")</f>
         <v/>
       </c>
       <c r="F11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$40,"PENDING")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$45,"PENDING")</f>
         <v/>
       </c>
       <c r="G11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$40,"BLOCKED")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$45,"BLOCKED")</f>
         <v/>
       </c>
       <c r="H11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$40,"N/A")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$45,"N/A")</f>
         <v/>
       </c>
       <c r="I11" s="21">
@@ -11072,7 +11356,7 @@
         </is>
       </c>
       <c r="D3" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR1.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR1.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.1*")</f>
         <v/>
       </c>
       <c r="E3" s="29">
@@ -11102,7 +11386,7 @@
         </is>
       </c>
       <c r="D4" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR1.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR1.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.2*")</f>
         <v/>
       </c>
       <c r="E4" s="32">
@@ -11132,7 +11416,7 @@
         </is>
       </c>
       <c r="D5" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR1.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR1.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.3*")</f>
         <v/>
       </c>
       <c r="E5" s="29">
@@ -11162,7 +11446,7 @@
         </is>
       </c>
       <c r="D6" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR1.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR1.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.4*")</f>
         <v/>
       </c>
       <c r="E6" s="32">
@@ -11192,7 +11476,7 @@
         </is>
       </c>
       <c r="D7" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR1.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR1.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.5*")</f>
         <v/>
       </c>
       <c r="E7" s="29">
@@ -11222,7 +11506,7 @@
         </is>
       </c>
       <c r="D8" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR1.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR1.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.6*")</f>
         <v/>
       </c>
       <c r="E8" s="32">
@@ -11252,7 +11536,7 @@
         </is>
       </c>
       <c r="D9" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR2.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR2.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.1*")</f>
         <v/>
       </c>
       <c r="E9" s="29">
@@ -11282,7 +11566,7 @@
         </is>
       </c>
       <c r="D10" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR2.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR2.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.2*")</f>
         <v/>
       </c>
       <c r="E10" s="32">
@@ -11312,7 +11596,7 @@
         </is>
       </c>
       <c r="D11" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR2.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR2.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.3*")</f>
         <v/>
       </c>
       <c r="E11" s="29">
@@ -11342,7 +11626,7 @@
         </is>
       </c>
       <c r="D12" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR2.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR2.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.4*")</f>
         <v/>
       </c>
       <c r="E12" s="32">
@@ -11372,7 +11656,7 @@
         </is>
       </c>
       <c r="D13" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR2.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR2.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.5*")</f>
         <v/>
       </c>
       <c r="E13" s="29">
@@ -11402,7 +11686,7 @@
         </is>
       </c>
       <c r="D14" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR2.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR2.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.6*")</f>
         <v/>
       </c>
       <c r="E14" s="32">
@@ -11432,7 +11716,7 @@
         </is>
       </c>
       <c r="D15" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR3.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR3.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.1*")</f>
         <v/>
       </c>
       <c r="E15" s="29">
@@ -11462,7 +11746,7 @@
         </is>
       </c>
       <c r="D16" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR3.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR3.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.2*")</f>
         <v/>
       </c>
       <c r="E16" s="32">
@@ -11492,7 +11776,7 @@
         </is>
       </c>
       <c r="D17" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR3.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR3.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.3*")</f>
         <v/>
       </c>
       <c r="E17" s="29">
@@ -11522,7 +11806,7 @@
         </is>
       </c>
       <c r="D18" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR3.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR3.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.4*")</f>
         <v/>
       </c>
       <c r="E18" s="32">
@@ -11552,7 +11836,7 @@
         </is>
       </c>
       <c r="D19" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR3.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR3.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.5*")</f>
         <v/>
       </c>
       <c r="E19" s="29">
@@ -11582,7 +11866,7 @@
         </is>
       </c>
       <c r="D20" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR4.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR4.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.1*")</f>
         <v/>
       </c>
       <c r="E20" s="32">
@@ -11612,7 +11896,7 @@
         </is>
       </c>
       <c r="D21" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR4.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR4.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.2*")</f>
         <v/>
       </c>
       <c r="E21" s="29">
@@ -11642,7 +11926,7 @@
         </is>
       </c>
       <c r="D22" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR4.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR4.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.3*")</f>
         <v/>
       </c>
       <c r="E22" s="32">
@@ -11672,7 +11956,7 @@
         </is>
       </c>
       <c r="D23" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR4.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR4.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.4*")</f>
         <v/>
       </c>
       <c r="E23" s="29">
@@ -11702,7 +11986,7 @@
         </is>
       </c>
       <c r="D24" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR4.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR4.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.5*")</f>
         <v/>
       </c>
       <c r="E24" s="32">
@@ -11732,7 +12016,7 @@
         </is>
       </c>
       <c r="D25" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR4.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR4.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.6*")</f>
         <v/>
       </c>
       <c r="E25" s="29">
@@ -11762,7 +12046,7 @@
         </is>
       </c>
       <c r="D26" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR5.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR5.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.1*")</f>
         <v/>
       </c>
       <c r="E26" s="32">
@@ -11792,7 +12076,7 @@
         </is>
       </c>
       <c r="D27" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR5.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR5.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.2*")</f>
         <v/>
       </c>
       <c r="E27" s="29">
@@ -11822,7 +12106,7 @@
         </is>
       </c>
       <c r="D28" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR5.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR5.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.3*")</f>
         <v/>
       </c>
       <c r="E28" s="32">
@@ -11852,7 +12136,7 @@
         </is>
       </c>
       <c r="D29" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR5.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR5.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.4*")</f>
         <v/>
       </c>
       <c r="E29" s="29">
@@ -11882,7 +12166,7 @@
         </is>
       </c>
       <c r="D30" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR6.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR6.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.1*")</f>
         <v/>
       </c>
       <c r="E30" s="32">
@@ -11912,7 +12196,7 @@
         </is>
       </c>
       <c r="D31" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR6.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR6.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.2*")</f>
         <v/>
       </c>
       <c r="E31" s="29">
@@ -11942,7 +12226,7 @@
         </is>
       </c>
       <c r="D32" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR6.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR6.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.3*")</f>
         <v/>
       </c>
       <c r="E32" s="32">
@@ -11972,7 +12256,7 @@
         </is>
       </c>
       <c r="D33" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR6.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR6.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.4*")</f>
         <v/>
       </c>
       <c r="E33" s="29">
@@ -12002,7 +12286,7 @@
         </is>
       </c>
       <c r="D34" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR7.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR7.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.1*")</f>
         <v/>
       </c>
       <c r="E34" s="32">
@@ -12032,7 +12316,7 @@
         </is>
       </c>
       <c r="D35" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR7.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR7.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.2*")</f>
         <v/>
       </c>
       <c r="E35" s="29">
@@ -12062,7 +12346,7 @@
         </is>
       </c>
       <c r="D36" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR7.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR7.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.3*")</f>
         <v/>
       </c>
       <c r="E36" s="32">
@@ -12092,7 +12376,7 @@
         </is>
       </c>
       <c r="D37" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR7.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR7.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.4*")</f>
         <v/>
       </c>
       <c r="E37" s="29">
@@ -12122,7 +12406,7 @@
         </is>
       </c>
       <c r="D38" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR7.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR7.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.5*")</f>
         <v/>
       </c>
       <c r="E38" s="32">
@@ -12152,7 +12436,7 @@
         </is>
       </c>
       <c r="D39" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR8.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR8.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.1*")</f>
         <v/>
       </c>
       <c r="E39" s="29">
@@ -12182,7 +12466,7 @@
         </is>
       </c>
       <c r="D40" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR8.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR8.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.2*")</f>
         <v/>
       </c>
       <c r="E40" s="32">
@@ -12212,7 +12496,7 @@
         </is>
       </c>
       <c r="D41" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR8.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR8.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.3*")</f>
         <v/>
       </c>
       <c r="E41" s="29">
@@ -12242,7 +12526,7 @@
         </is>
       </c>
       <c r="D42" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR8.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR8.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.4*")</f>
         <v/>
       </c>
       <c r="E42" s="32">
@@ -12272,7 +12556,7 @@
         </is>
       </c>
       <c r="D43" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR9.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR9.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.1*")</f>
         <v/>
       </c>
       <c r="E43" s="29">
@@ -12302,7 +12586,7 @@
         </is>
       </c>
       <c r="D44" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR9.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR9.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.2*")</f>
         <v/>
       </c>
       <c r="E44" s="32">
@@ -12332,7 +12616,7 @@
         </is>
       </c>
       <c r="D45" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR9.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR9.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.3*")</f>
         <v/>
       </c>
       <c r="E45" s="29">
@@ -12362,7 +12646,7 @@
         </is>
       </c>
       <c r="D46" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR9.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR9.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.4*")</f>
         <v/>
       </c>
       <c r="E46" s="32">
@@ -12392,7 +12676,7 @@
         </is>
       </c>
       <c r="D47" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR9.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR9.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.5*")</f>
         <v/>
       </c>
       <c r="E47" s="29">
@@ -12422,7 +12706,7 @@
         </is>
       </c>
       <c r="D48" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR9.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR9.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.6*")</f>
         <v/>
       </c>
       <c r="E48" s="32">
@@ -12452,7 +12736,7 @@
         </is>
       </c>
       <c r="D49" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.7*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.7*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.7*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.7*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.7*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.7*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.7*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$40,"*FR9.7*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.7*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.7*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.7*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.7*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.7*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.7*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.7*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.7*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.7*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.7*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.7*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.7*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.7*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR9.7*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.7*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.7*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.7*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.7*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.7*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.7*")</f>
         <v/>
       </c>
       <c r="E49" s="29">

</xml_diff>

<commit_message>
test: UI/UX polish results (UX-04..UX-07)
</commit_message>
<xml_diff>
--- a/MediFind_Test_Requirements_v2.xlsx
+++ b/MediFind_Test_Requirements_v2.xlsx
@@ -1759,7 +1759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3535,48 +3535,236 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="40" customHeight="1">
+    <row r="45" ht="50" customHeight="1">
       <c r="A45" s="37" t="inlineStr">
         <is>
+          <t>UX-04</t>
+        </is>
+      </c>
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Beyond SRS</t>
+        </is>
+      </c>
+      <c r="C45" s="39" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="D45" s="39" t="inlineStr">
+        <is>
+          <t>Checkout shows clear progress and a Stripe sheet in MediFind style</t>
+        </is>
+      </c>
+      <c r="E45" s="39" t="inlineStr">
+        <is>
+          <t>Tap Pay on checkout</t>
+        </is>
+      </c>
+      <c r="F45" s="39" t="inlineStr">
+        <is>
+          <t>Button says Opening secure payment…; sheet uses app colours and says Pay PKR …</t>
+        </is>
+      </c>
+      <c r="G45" s="38" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H45" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I45" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18: Pay shows "Opening secure payment…" then "Confirming payment…"; Stripe sheet in app colours (light) with "Pay PKR 499" button</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="50" customHeight="1">
+      <c r="A46" s="41" t="inlineStr">
+        <is>
+          <t>UX-05</t>
+        </is>
+      </c>
+      <c r="B46" s="42" t="inlineStr">
+        <is>
+          <t>FR6.2</t>
+        </is>
+      </c>
+      <c r="C46" s="43" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="D46" s="43" t="inlineStr">
+        <is>
+          <t>Unrealistic GPS distance is not shown as an ETA</t>
+        </is>
+      </c>
+      <c r="E46" s="43" t="inlineStr">
+        <is>
+          <t>Responder phone reports a location hundreds of km away</t>
+        </is>
+      </c>
+      <c r="F46" s="43" t="inlineStr">
+        <is>
+          <t>Shows Locating / Waiting for GPS; no route line; map stays on the patient</t>
+        </is>
+      </c>
+      <c r="G46" s="42" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H46" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I46" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-18: responder GPS set to California: "Locating you / Waiting for GPS", no route line, camera on patient (was "17913 min, 11941 km"); back to Lahore: marker placed directly, "2 min · 1.3 km", normal zoom</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="40" customHeight="1">
+      <c r="A47" s="37" t="inlineStr">
+        <is>
+          <t>UX-06</t>
+        </is>
+      </c>
+      <c r="B47" s="38" t="inlineStr">
+        <is>
+          <t>NFR</t>
+        </is>
+      </c>
+      <c r="C47" s="39" t="inlineStr">
+        <is>
+          <t>Usability</t>
+        </is>
+      </c>
+      <c r="D47" s="39" t="inlineStr">
+        <is>
+          <t>Maps show a loading state instead of a blank box</t>
+        </is>
+      </c>
+      <c r="E47" s="39" t="inlineStr">
+        <is>
+          <t>Open a tracking screen</t>
+        </is>
+      </c>
+      <c r="F47" s="39" t="inlineStr">
+        <is>
+          <t>Loading map… until the map appears</t>
+        </is>
+      </c>
+      <c r="G47" s="38" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H47" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I47" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18: responder / patient / caregiver tracking maps show "Loading map…" until the map is ready (was a blank grey box)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="40" customHeight="1">
+      <c r="A48" s="41" t="inlineStr">
+        <is>
+          <t>UX-07</t>
+        </is>
+      </c>
+      <c r="B48" s="42" t="inlineStr">
+        <is>
+          <t>FR3.1</t>
+        </is>
+      </c>
+      <c r="C48" s="43" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="D48" s="43" t="inlineStr">
+        <is>
+          <t>Deaf quick phrases are fully readable on the home screen</t>
+        </is>
+      </c>
+      <c r="E48" s="43" t="inlineStr">
+        <is>
+          <t>Open the Deaf patient home screen</t>
+        </is>
+      </c>
+      <c r="F48" s="43" t="inlineStr">
+        <is>
+          <t>Each phrase shown in full, wrapping onto lines</t>
+        </is>
+      </c>
+      <c r="G48" s="42" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H48" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I48" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-18: Deaf home quick phrases wrap onto lines and are fully readable (was cut off "I am de…")</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="40" customHeight="1">
+      <c r="A49" s="37" t="inlineStr">
+        <is>
           <t>UX-03</t>
         </is>
       </c>
-      <c r="B45" s="38" t="inlineStr">
+      <c r="B49" s="38" t="inlineStr">
         <is>
           <t>NFR</t>
         </is>
       </c>
-      <c r="C45" s="39" t="inlineStr">
+      <c r="C49" s="39" t="inlineStr">
         <is>
           <t>Branding</t>
         </is>
       </c>
-      <c r="D45" s="39" t="inlineStr">
+      <c r="D49" s="39" t="inlineStr">
         <is>
           <t>The same MediFind logo is used in the mobile app and the web portal</t>
         </is>
       </c>
-      <c r="E45" s="39" t="inlineStr">
+      <c r="E49" s="39" t="inlineStr">
         <is>
           <t>Compare app launcher, splash, headers with portal sidebar, login, landing, 404, legal, favicon</t>
         </is>
       </c>
-      <c r="F45" s="39" t="inlineStr">
+      <c r="F49" s="39" t="inlineStr">
         <is>
           <t>One consistent logo everywhere</t>
         </is>
       </c>
-      <c r="G45" s="38" t="inlineStr">
+      <c r="G49" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H45" s="45" t="inlineStr">
+      <c r="H49" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I45" s="39" t="inlineStr">
+      <c r="I49" s="39" t="inlineStr">
         <is>
           <t>2026-09-18: portal sidebar, login, landing, 404, legal and favicon use the same pin-with-rings logo as the mobile app</t>
         </is>
@@ -3593,7 +3781,7 @@
     <mergeCell ref="A20:I20"/>
     <mergeCell ref="A38:I38"/>
   </mergeCells>
-  <conditionalFormatting sqref="H4:H45">
+  <conditionalFormatting sqref="H4:H49">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -3611,7 +3799,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H4:H45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid status" error="Choose PASS, FAIL, PENDING, BLOCKED or N/A" type="list">
+    <dataValidation sqref="H4:H49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid status" error="Choose PASS, FAIL, PENDING, BLOCKED or N/A" type="list">
       <formula1>"PENDING,PASS,FAIL,BLOCKED,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7302,7 +7490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D151"/>
+  <dimension ref="A1:D155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9609,7 +9797,7 @@
     <row r="106">
       <c r="A106" s="48" t="inlineStr">
         <is>
-          <t>UX-03</t>
+          <t>UX-04</t>
         </is>
       </c>
       <c r="B106" s="48" t="inlineStr">
@@ -9619,19 +9807,19 @@
       </c>
       <c r="C106" s="48" t="inlineStr">
         <is>
-          <t>The same MediFind logo is used in the mobile app and the web portal</t>
+          <t>Checkout shows clear progress and a Stripe sheet in MediFind style</t>
         </is>
       </c>
       <c r="D106" s="48" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="48" t="inlineStr">
         <is>
-          <t>MED-01</t>
+          <t>UX-05</t>
         </is>
       </c>
       <c r="B107" s="48" t="inlineStr">
@@ -9641,19 +9829,19 @@
       </c>
       <c r="C107" s="48" t="inlineStr">
         <is>
-          <t>Patient creates and edits the medical profile</t>
+          <t>Unrealistic GPS distance is not shown as an ETA</t>
         </is>
       </c>
       <c r="D107" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.1, FR2.2</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR6.2</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="48" t="inlineStr">
         <is>
-          <t>MED-02</t>
+          <t>UX-06</t>
         </is>
       </c>
       <c r="B108" s="48" t="inlineStr">
@@ -9663,19 +9851,19 @@
       </c>
       <c r="C108" s="48" t="inlineStr">
         <is>
-          <t>Saving the medical profile keeps emergency contacts and quick phrases</t>
+          <t>Maps show a loading state instead of a blank box</t>
         </is>
       </c>
       <c r="D108" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.1</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="48" t="inlineStr">
         <is>
-          <t>MED-03</t>
+          <t>UX-07</t>
         </is>
       </c>
       <c r="B109" s="48" t="inlineStr">
@@ -9685,19 +9873,19 @@
       </c>
       <c r="C109" s="48" t="inlineStr">
         <is>
-          <t>Patient adds, calls and deletes emergency contacts</t>
+          <t>Deaf quick phrases are fully readable on the home screen</t>
         </is>
       </c>
       <c r="D109" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.1</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR3.1</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="48" t="inlineStr">
         <is>
-          <t>MED-04</t>
+          <t>UX-03</t>
         </is>
       </c>
       <c r="B110" s="48" t="inlineStr">
@@ -9707,19 +9895,19 @@
       </c>
       <c r="C110" s="48" t="inlineStr">
         <is>
-          <t>Sensitive medical fields are encrypted at rest</t>
+          <t>The same MediFind logo is used in the mobile app and the web portal</t>
         </is>
       </c>
       <c r="D110" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.2</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="48" t="inlineStr">
         <is>
-          <t>MED-05</t>
+          <t>MED-01</t>
         </is>
       </c>
       <c r="B111" s="48" t="inlineStr">
@@ -9729,19 +9917,19 @@
       </c>
       <c r="C111" s="48" t="inlineStr">
         <is>
-          <t>Upload a report from camera, gallery (image) and PDF</t>
+          <t>Patient creates and edits the medical profile</t>
         </is>
       </c>
       <c r="D111" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.3</t>
+          <t>New sheet MEDICAL; SRS FR2.1, FR2.2</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="48" t="inlineStr">
         <is>
-          <t>MED-06</t>
+          <t>MED-02</t>
         </is>
       </c>
       <c r="B112" s="48" t="inlineStr">
@@ -9751,19 +9939,19 @@
       </c>
       <c r="C112" s="48" t="inlineStr">
         <is>
-          <t>Unsupported or oversized files are rejected with a clear message</t>
+          <t>Saving the medical profile keeps emergency contacts and quick phrases</t>
         </is>
       </c>
       <c r="D112" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.3</t>
+          <t>New sheet MEDICAL; SRS FR2.1</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="48" t="inlineStr">
         <is>
-          <t>MED-07</t>
+          <t>MED-03</t>
         </is>
       </c>
       <c r="B113" s="48" t="inlineStr">
@@ -9773,19 +9961,19 @@
       </c>
       <c r="C113" s="48" t="inlineStr">
         <is>
-          <t>View, rename and delete a report</t>
+          <t>Patient adds, calls and deletes emergency contacts</t>
         </is>
       </c>
       <c r="D113" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.4</t>
+          <t>New sheet MEDICAL; SRS FR2.1</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="48" t="inlineStr">
         <is>
-          <t>MED-08</t>
+          <t>MED-04</t>
         </is>
       </c>
       <c r="B114" s="48" t="inlineStr">
@@ -9795,19 +9983,19 @@
       </c>
       <c r="C114" s="48" t="inlineStr">
         <is>
-          <t>Assigned responder receives the patient medical summary on accept</t>
+          <t>Sensitive medical fields are encrypted at rest</t>
         </is>
       </c>
       <c r="D114" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.5</t>
+          <t>New sheet MEDICAL; SRS FR2.2</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="48" t="inlineStr">
         <is>
-          <t>MED-09</t>
+          <t>MED-05</t>
         </is>
       </c>
       <c r="B115" s="48" t="inlineStr">
@@ -9817,19 +10005,19 @@
       </c>
       <c r="C115" s="48" t="inlineStr">
         <is>
-          <t>Report files are visible only to the patient, linked caregivers, the active responder and admins</t>
+          <t>Upload a report from camera, gallery (image) and PDF</t>
         </is>
       </c>
       <c r="D115" s="48" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.6</t>
+          <t>New sheet MEDICAL; SRS FR2.3</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="48" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>MED-06</t>
         </is>
       </c>
       <c r="B116" s="48" t="inlineStr">
@@ -9839,19 +10027,19 @@
       </c>
       <c r="C116" s="48" t="inlineStr">
         <is>
-          <t>SOS requires press-and-hold before it starts</t>
+          <t>Unsupported or oversized files are rejected with a clear message</t>
         </is>
       </c>
       <c r="D116" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.1</t>
+          <t>New sheet MEDICAL; SRS FR2.3</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="48" t="inlineStr">
         <is>
-          <t>SEC-02</t>
+          <t>MED-07</t>
         </is>
       </c>
       <c r="B117" s="48" t="inlineStr">
@@ -9861,19 +10049,19 @@
       </c>
       <c r="C117" s="48" t="inlineStr">
         <is>
-          <t>Cancelling during the 60-second countdown sends nothing to the server</t>
+          <t>View, rename and delete a report</t>
         </is>
       </c>
       <c r="D117" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.3</t>
+          <t>New sheet MEDICAL; SRS FR2.4</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="48" t="inlineStr">
         <is>
-          <t>SEC-03</t>
+          <t>MED-08</t>
         </is>
       </c>
       <c r="B118" s="48" t="inlineStr">
@@ -9883,19 +10071,19 @@
       </c>
       <c r="C118" s="48" t="inlineStr">
         <is>
-          <t>SOS from a mock (fake) GPS location is refused in production</t>
+          <t>Assigned responder receives the patient medical summary on accept</t>
         </is>
       </c>
       <c r="D118" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
+          <t>New sheet MEDICAL; SRS FR2.5</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="48" t="inlineStr">
         <is>
-          <t>SEC-04</t>
+          <t>MED-09</t>
         </is>
       </c>
       <c r="B119" s="48" t="inlineStr">
@@ -9905,19 +10093,19 @@
       </c>
       <c r="C119" s="48" t="inlineStr">
         <is>
-          <t>More than 5 SOS in one hour is refused</t>
+          <t>Report files are visible only to the patient, linked caregivers, the active responder and admins</t>
         </is>
       </c>
       <c r="D119" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.5</t>
+          <t>New sheet MEDICAL; SRS FR2.6</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="48" t="inlineStr">
         <is>
-          <t>SEC-05</t>
+          <t>SEC-01</t>
         </is>
       </c>
       <c r="B120" s="48" t="inlineStr">
@@ -9927,19 +10115,19 @@
       </c>
       <c r="C120" s="48" t="inlineStr">
         <is>
-          <t>SOS outside Pakistan coordinates is refused</t>
+          <t>SOS requires press-and-hold before it starts</t>
         </is>
       </c>
       <c r="D120" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.1</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="48" t="inlineStr">
         <is>
-          <t>SEC-06</t>
+          <t>SEC-02</t>
         </is>
       </c>
       <c r="B121" s="48" t="inlineStr">
@@ -9949,19 +10137,19 @@
       </c>
       <c r="C121" s="48" t="inlineStr">
         <is>
-          <t>Responder must add a note when closing as False alarm or Patient not found</t>
+          <t>Cancelling during the 60-second countdown sends nothing to the server</t>
         </is>
       </c>
       <c r="D121" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR6.2</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.3</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="48" t="inlineStr">
         <is>
-          <t>SEC-07</t>
+          <t>SEC-03</t>
         </is>
       </c>
       <c r="B122" s="48" t="inlineStr">
@@ -9971,19 +10159,19 @@
       </c>
       <c r="C122" s="48" t="inlineStr">
         <is>
-          <t>Patient is warned when an SOS is marked as a false alarm</t>
+          <t>SOS from a mock (fake) GPS location is refused in production</t>
         </is>
       </c>
       <c r="D122" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; beyond SRS</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="48" t="inlineStr">
         <is>
-          <t>SEC-08</t>
+          <t>SEC-04</t>
         </is>
       </c>
       <c r="B123" s="48" t="inlineStr">
@@ -9993,19 +10181,19 @@
       </c>
       <c r="C123" s="48" t="inlineStr">
         <is>
-          <t>3 false alarms in 30 days alerts admins for review</t>
+          <t>More than 5 SOS in one hour is refused</t>
         </is>
       </c>
       <c r="D123" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; beyond SRS</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.5</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="48" t="inlineStr">
         <is>
-          <t>SEC-09</t>
+          <t>SEC-05</t>
         </is>
       </c>
       <c r="B124" s="48" t="inlineStr">
@@ -10015,19 +10203,19 @@
       </c>
       <c r="C124" s="48" t="inlineStr">
         <is>
-          <t>Patient-cancelled SOS never counts as a false alarm</t>
+          <t>SOS outside Pakistan coordinates is refused</t>
         </is>
       </c>
       <c r="D124" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; beyond SRS</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="48" t="inlineStr">
         <is>
-          <t>SEC-10</t>
+          <t>SEC-06</t>
         </is>
       </c>
       <c r="B125" s="48" t="inlineStr">
@@ -10037,19 +10225,19 @@
       </c>
       <c r="C125" s="48" t="inlineStr">
         <is>
-          <t>Refresh token cannot be used as an access token</t>
+          <t>Responder must add a note when closing as False alarm or Patient not found</t>
         </is>
       </c>
       <c r="D125" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
+          <t>New sheet SECURITY_SOS; SRS FR6.2</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="48" t="inlineStr">
         <is>
-          <t>SEC-11</t>
+          <t>SEC-07</t>
         </is>
       </c>
       <c r="B126" s="48" t="inlineStr">
@@ -10059,19 +10247,19 @@
       </c>
       <c r="C126" s="48" t="inlineStr">
         <is>
-          <t>Users cannot join emergency or chat rooms they do not belong to</t>
+          <t>Patient is warned when an SOS is marked as a false alarm</t>
         </is>
       </c>
       <c r="D126" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
+          <t>New sheet SECURITY_SOS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="48" t="inlineStr">
         <is>
-          <t>SEC-12</t>
+          <t>SEC-08</t>
         </is>
       </c>
       <c r="B127" s="48" t="inlineStr">
@@ -10081,7 +10269,7 @@
       </c>
       <c r="C127" s="48" t="inlineStr">
         <is>
-          <t>Paid plan upgrade requires a verified Stripe payment</t>
+          <t>3 false alarms in 30 days alerts admins for review</t>
         </is>
       </c>
       <c r="D127" s="48" t="inlineStr">
@@ -10093,7 +10281,7 @@
     <row r="128">
       <c r="A128" s="48" t="inlineStr">
         <is>
-          <t>SEC-13</t>
+          <t>SEC-09</t>
         </is>
       </c>
       <c r="B128" s="48" t="inlineStr">
@@ -10103,19 +10291,19 @@
       </c>
       <c r="C128" s="48" t="inlineStr">
         <is>
-          <t>Only the assigned responder can update or resolve an emergency</t>
+          <t>Patient-cancelled SOS never counts as a false alarm</t>
         </is>
       </c>
       <c r="D128" s="48" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR5.1</t>
+          <t>New sheet SECURITY_SOS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="48" t="inlineStr">
         <is>
-          <t>NAV-01</t>
+          <t>SEC-10</t>
         </is>
       </c>
       <c r="B129" s="48" t="inlineStr">
@@ -10125,19 +10313,19 @@
       </c>
       <c r="C129" s="48" t="inlineStr">
         <is>
-          <t>Each role has a unified sidebar (AppDrawer) with role-specific items</t>
+          <t>Refresh token cannot be used as an access token</t>
         </is>
       </c>
       <c r="D129" s="48" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.1</t>
+          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="48" t="inlineStr">
         <is>
-          <t>NAV-02</t>
+          <t>SEC-11</t>
         </is>
       </c>
       <c r="B130" s="48" t="inlineStr">
@@ -10147,19 +10335,19 @@
       </c>
       <c r="C130" s="48" t="inlineStr">
         <is>
-          <t>Switching tabs preserves each tab's state and back navigation works</t>
+          <t>Users cannot join emergency or chat rooms they do not belong to</t>
         </is>
       </c>
       <c r="D130" s="48" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.2</t>
+          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="48" t="inlineStr">
         <is>
-          <t>NAV-03</t>
+          <t>SEC-12</t>
         </is>
       </c>
       <c r="B131" s="48" t="inlineStr">
@@ -10169,19 +10357,19 @@
       </c>
       <c r="C131" s="48" t="inlineStr">
         <is>
-          <t>Role dashboards show quick action grids</t>
+          <t>Paid plan upgrade requires a verified Stripe payment</t>
         </is>
       </c>
       <c r="D131" s="48" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.3</t>
+          <t>New sheet SECURITY_SOS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="48" t="inlineStr">
         <is>
-          <t>NAV-04</t>
+          <t>SEC-13</t>
         </is>
       </c>
       <c r="B132" s="48" t="inlineStr">
@@ -10191,19 +10379,19 @@
       </c>
       <c r="C132" s="48" t="inlineStr">
         <is>
-          <t>Map and chat screens render smoothly (~60 FPS)</t>
+          <t>Only the assigned responder can update or resolve an emergency</t>
         </is>
       </c>
       <c r="D132" s="48" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.4</t>
+          <t>New sheet SECURITY_SOS; SRS FR5.1</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="48" t="inlineStr">
         <is>
-          <t>NAV-05</t>
+          <t>NAV-01</t>
         </is>
       </c>
       <c r="B133" s="48" t="inlineStr">
@@ -10213,107 +10401,107 @@
       </c>
       <c r="C133" s="48" t="inlineStr">
         <is>
-          <t>Large buttons mode enlarges tap targets across screens</t>
+          <t>Each role has a unified sidebar (AppDrawer) with role-specific items</t>
         </is>
       </c>
       <c r="D133" s="48" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR3.5</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.1</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="48" t="inlineStr">
         <is>
-          <t>PRF-01</t>
+          <t>NAV-02</t>
         </is>
       </c>
       <c r="B134" s="48" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C134" s="48" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Switching tabs preserves each tab's state and back navigation works</t>
         </is>
       </c>
       <c r="D134" s="48" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.2</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="48" t="inlineStr">
         <is>
-          <t>PRF-02</t>
+          <t>NAV-03</t>
         </is>
       </c>
       <c r="B135" s="48" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C135" s="48" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Role dashboards show quick action grids</t>
         </is>
       </c>
       <c r="D135" s="48" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.3</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="48" t="inlineStr">
         <is>
-          <t>PRF-03</t>
+          <t>NAV-04</t>
         </is>
       </c>
       <c r="B136" s="48" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C136" s="48" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Map and chat screens render smoothly (~60 FPS)</t>
         </is>
       </c>
       <c r="D136" s="48" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.4</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="48" t="inlineStr">
         <is>
-          <t>PRF-05</t>
+          <t>NAV-05</t>
         </is>
       </c>
       <c r="B137" s="48" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C137" s="48" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Large buttons mode enlarges tap targets across screens</t>
         </is>
       </c>
       <c r="D137" s="48" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR3.5</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="48" t="inlineStr">
         <is>
-          <t>NTF-01</t>
+          <t>PRF-01</t>
         </is>
       </c>
       <c r="B138" s="48" t="inlineStr">
@@ -10335,7 +10523,7 @@
     <row r="139">
       <c r="A139" s="48" t="inlineStr">
         <is>
-          <t>NTF-02</t>
+          <t>PRF-02</t>
         </is>
       </c>
       <c r="B139" s="48" t="inlineStr">
@@ -10357,7 +10545,7 @@
     <row r="140">
       <c r="A140" s="48" t="inlineStr">
         <is>
-          <t>NTF-03</t>
+          <t>PRF-03</t>
         </is>
       </c>
       <c r="B140" s="48" t="inlineStr">
@@ -10379,7 +10567,7 @@
     <row r="141">
       <c r="A141" s="48" t="inlineStr">
         <is>
-          <t>NTF-04</t>
+          <t>PRF-05</t>
         </is>
       </c>
       <c r="B141" s="48" t="inlineStr">
@@ -10401,7 +10589,7 @@
     <row r="142">
       <c r="A142" s="48" t="inlineStr">
         <is>
-          <t>NTF-05</t>
+          <t>NTF-01</t>
         </is>
       </c>
       <c r="B142" s="48" t="inlineStr">
@@ -10423,7 +10611,7 @@
     <row r="143">
       <c r="A143" s="48" t="inlineStr">
         <is>
-          <t>NTF-07</t>
+          <t>NTF-02</t>
         </is>
       </c>
       <c r="B143" s="48" t="inlineStr">
@@ -10445,7 +10633,7 @@
     <row r="144">
       <c r="A144" s="48" t="inlineStr">
         <is>
-          <t>NTF-08</t>
+          <t>NTF-03</t>
         </is>
       </c>
       <c r="B144" s="48" t="inlineStr">
@@ -10467,7 +10655,7 @@
     <row r="145">
       <c r="A145" s="48" t="inlineStr">
         <is>
-          <t>ACC-06</t>
+          <t>NTF-04</t>
         </is>
       </c>
       <c r="B145" s="48" t="inlineStr">
@@ -10489,7 +10677,7 @@
     <row r="146">
       <c r="A146" s="48" t="inlineStr">
         <is>
-          <t>ACC-07</t>
+          <t>NTF-05</t>
         </is>
       </c>
       <c r="B146" s="48" t="inlineStr">
@@ -10511,7 +10699,7 @@
     <row r="147">
       <c r="A147" s="48" t="inlineStr">
         <is>
-          <t>ACC-11</t>
+          <t>NTF-07</t>
         </is>
       </c>
       <c r="B147" s="48" t="inlineStr">
@@ -10533,7 +10721,7 @@
     <row r="148">
       <c r="A148" s="48" t="inlineStr">
         <is>
-          <t>AUTH-12</t>
+          <t>NTF-08</t>
         </is>
       </c>
       <c r="B148" s="48" t="inlineStr">
@@ -10555,7 +10743,7 @@
     <row r="149">
       <c r="A149" s="48" t="inlineStr">
         <is>
-          <t>API-04</t>
+          <t>ACC-06</t>
         </is>
       </c>
       <c r="B149" s="48" t="inlineStr">
@@ -10577,7 +10765,7 @@
     <row r="150">
       <c r="A150" s="48" t="inlineStr">
         <is>
-          <t>API-08</t>
+          <t>ACC-07</t>
         </is>
       </c>
       <c r="B150" s="48" t="inlineStr">
@@ -10599,20 +10787,108 @@
     <row r="151">
       <c r="A151" s="48" t="inlineStr">
         <is>
+          <t>ACC-11</t>
+        </is>
+      </c>
+      <c r="B151" s="48" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C151" s="48" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D151" s="48" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="48" t="inlineStr">
+        <is>
+          <t>AUTH-12</t>
+        </is>
+      </c>
+      <c r="B152" s="48" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C152" s="48" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D152" s="48" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="48" t="inlineStr">
+        <is>
+          <t>API-04</t>
+        </is>
+      </c>
+      <c r="B153" s="48" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C153" s="48" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D153" s="48" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="48" t="inlineStr">
+        <is>
+          <t>API-08</t>
+        </is>
+      </c>
+      <c r="B154" s="48" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C154" s="48" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D154" s="48" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="48" t="inlineStr">
+        <is>
           <t>API-09</t>
         </is>
       </c>
-      <c r="B151" s="48" t="inlineStr">
+      <c r="B155" s="48" t="inlineStr">
         <is>
           <t>Re-classified</t>
         </is>
       </c>
-      <c r="C151" s="48" t="inlineStr">
+      <c r="C155" s="48" t="inlineStr">
         <is>
           <t>Marked "Beyond SRS" in the SRS Ref column</t>
         </is>
       </c>
-      <c r="D151" s="48" t="inlineStr">
+      <c r="D155" s="48" t="inlineStr">
         <is>
           <t>Valid feature test with no matching SRS functional requirement</t>
         </is>
@@ -10976,27 +11252,27 @@
         </is>
       </c>
       <c r="C11" s="19">
-        <f>COUNTA(PRIVACY_CALLS!$A$4:$A$45)-COUNTIF(PRIVACY_CALLS!$A$4:$A$45,"  *")</f>
+        <f>COUNTA(PRIVACY_CALLS!$A$4:$A$49)-COUNTIF(PRIVACY_CALLS!$A$4:$A$49,"  *")</f>
         <v/>
       </c>
       <c r="D11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$45,"PASS")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$49,"PASS")</f>
         <v/>
       </c>
       <c r="E11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$45,"FAIL")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$49,"FAIL")</f>
         <v/>
       </c>
       <c r="F11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$45,"PENDING")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$49,"PENDING")</f>
         <v/>
       </c>
       <c r="G11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$45,"BLOCKED")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$49,"BLOCKED")</f>
         <v/>
       </c>
       <c r="H11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$45,"N/A")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$49,"N/A")</f>
         <v/>
       </c>
       <c r="I11" s="21">
@@ -11356,7 +11632,7 @@
         </is>
       </c>
       <c r="D3" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR1.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR1.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.1*")</f>
         <v/>
       </c>
       <c r="E3" s="29">
@@ -11386,7 +11662,7 @@
         </is>
       </c>
       <c r="D4" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR1.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR1.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.2*")</f>
         <v/>
       </c>
       <c r="E4" s="32">
@@ -11416,7 +11692,7 @@
         </is>
       </c>
       <c r="D5" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR1.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR1.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.3*")</f>
         <v/>
       </c>
       <c r="E5" s="29">
@@ -11446,7 +11722,7 @@
         </is>
       </c>
       <c r="D6" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR1.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR1.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.4*")</f>
         <v/>
       </c>
       <c r="E6" s="32">
@@ -11476,7 +11752,7 @@
         </is>
       </c>
       <c r="D7" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR1.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR1.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.5*")</f>
         <v/>
       </c>
       <c r="E7" s="29">
@@ -11506,7 +11782,7 @@
         </is>
       </c>
       <c r="D8" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR1.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR1.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.6*")</f>
         <v/>
       </c>
       <c r="E8" s="32">
@@ -11536,7 +11812,7 @@
         </is>
       </c>
       <c r="D9" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR2.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR2.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.1*")</f>
         <v/>
       </c>
       <c r="E9" s="29">
@@ -11566,7 +11842,7 @@
         </is>
       </c>
       <c r="D10" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR2.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR2.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.2*")</f>
         <v/>
       </c>
       <c r="E10" s="32">
@@ -11596,7 +11872,7 @@
         </is>
       </c>
       <c r="D11" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR2.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR2.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.3*")</f>
         <v/>
       </c>
       <c r="E11" s="29">
@@ -11626,7 +11902,7 @@
         </is>
       </c>
       <c r="D12" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR2.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR2.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.4*")</f>
         <v/>
       </c>
       <c r="E12" s="32">
@@ -11656,7 +11932,7 @@
         </is>
       </c>
       <c r="D13" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR2.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR2.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.5*")</f>
         <v/>
       </c>
       <c r="E13" s="29">
@@ -11686,7 +11962,7 @@
         </is>
       </c>
       <c r="D14" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR2.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR2.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.6*")</f>
         <v/>
       </c>
       <c r="E14" s="32">
@@ -11716,7 +11992,7 @@
         </is>
       </c>
       <c r="D15" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR3.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR3.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.1*")</f>
         <v/>
       </c>
       <c r="E15" s="29">
@@ -11725,7 +12001,7 @@
       </c>
       <c r="F15" s="28" t="inlineStr">
         <is>
-          <t>AUTH-02, SOS-02, SOS-07, SOS-08, CG-03, CHT-03, CHT-06, PHN-04, CALL-03, CALL-11, ACC-01, ACC-02, ACC-04, ACC-12</t>
+          <t>AUTH-02, SOS-02, SOS-07, SOS-08, CG-03, CHT-03, CHT-06, PHN-04, CALL-03, CALL-11, UX-07, ACC-01, ACC-02, ACC-04, ACC-12</t>
         </is>
       </c>
     </row>
@@ -11746,7 +12022,7 @@
         </is>
       </c>
       <c r="D16" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR3.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR3.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.2*")</f>
         <v/>
       </c>
       <c r="E16" s="32">
@@ -11776,7 +12052,7 @@
         </is>
       </c>
       <c r="D17" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR3.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR3.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.3*")</f>
         <v/>
       </c>
       <c r="E17" s="29">
@@ -11806,7 +12082,7 @@
         </is>
       </c>
       <c r="D18" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR3.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR3.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.4*")</f>
         <v/>
       </c>
       <c r="E18" s="32">
@@ -11836,7 +12112,7 @@
         </is>
       </c>
       <c r="D19" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR3.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR3.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.5*")</f>
         <v/>
       </c>
       <c r="E19" s="29">
@@ -11866,7 +12142,7 @@
         </is>
       </c>
       <c r="D20" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR4.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR4.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.1*")</f>
         <v/>
       </c>
       <c r="E20" s="32">
@@ -11896,7 +12172,7 @@
         </is>
       </c>
       <c r="D21" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR4.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR4.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.2*")</f>
         <v/>
       </c>
       <c r="E21" s="29">
@@ -11926,7 +12202,7 @@
         </is>
       </c>
       <c r="D22" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR4.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR4.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.3*")</f>
         <v/>
       </c>
       <c r="E22" s="32">
@@ -11956,7 +12232,7 @@
         </is>
       </c>
       <c r="D23" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR4.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR4.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.4*")</f>
         <v/>
       </c>
       <c r="E23" s="29">
@@ -11986,7 +12262,7 @@
         </is>
       </c>
       <c r="D24" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR4.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR4.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.5*")</f>
         <v/>
       </c>
       <c r="E24" s="32">
@@ -12016,7 +12292,7 @@
         </is>
       </c>
       <c r="D25" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR4.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR4.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.6*")</f>
         <v/>
       </c>
       <c r="E25" s="29">
@@ -12046,7 +12322,7 @@
         </is>
       </c>
       <c r="D26" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR5.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR5.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.1*")</f>
         <v/>
       </c>
       <c r="E26" s="32">
@@ -12076,7 +12352,7 @@
         </is>
       </c>
       <c r="D27" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR5.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR5.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.2*")</f>
         <v/>
       </c>
       <c r="E27" s="29">
@@ -12106,7 +12382,7 @@
         </is>
       </c>
       <c r="D28" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR5.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR5.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.3*")</f>
         <v/>
       </c>
       <c r="E28" s="32">
@@ -12136,7 +12412,7 @@
         </is>
       </c>
       <c r="D29" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR5.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR5.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.4*")</f>
         <v/>
       </c>
       <c r="E29" s="29">
@@ -12166,7 +12442,7 @@
         </is>
       </c>
       <c r="D30" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR6.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR6.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.1*")</f>
         <v/>
       </c>
       <c r="E30" s="32">
@@ -12196,7 +12472,7 @@
         </is>
       </c>
       <c r="D31" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR6.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR6.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.2*")</f>
         <v/>
       </c>
       <c r="E31" s="29">
@@ -12205,7 +12481,7 @@
       </c>
       <c r="F31" s="28" t="inlineStr">
         <is>
-          <t>SOS-06, SOS-11, SEC-06, RSP-08, RSP-09, RSP-10, CG-08, PERF-03, API-07</t>
+          <t>SOS-06, SOS-11, SEC-06, RSP-08, RSP-09, RSP-10, CG-08, PERF-03, UX-05, API-07</t>
         </is>
       </c>
     </row>
@@ -12226,7 +12502,7 @@
         </is>
       </c>
       <c r="D32" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR6.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR6.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.3*")</f>
         <v/>
       </c>
       <c r="E32" s="32">
@@ -12256,7 +12532,7 @@
         </is>
       </c>
       <c r="D33" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR6.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR6.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.4*")</f>
         <v/>
       </c>
       <c r="E33" s="29">
@@ -12286,7 +12562,7 @@
         </is>
       </c>
       <c r="D34" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR7.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR7.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.1*")</f>
         <v/>
       </c>
       <c r="E34" s="32">
@@ -12316,7 +12592,7 @@
         </is>
       </c>
       <c r="D35" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR7.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR7.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.2*")</f>
         <v/>
       </c>
       <c r="E35" s="29">
@@ -12346,7 +12622,7 @@
         </is>
       </c>
       <c r="D36" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR7.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR7.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.3*")</f>
         <v/>
       </c>
       <c r="E36" s="32">
@@ -12376,7 +12652,7 @@
         </is>
       </c>
       <c r="D37" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR7.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR7.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.4*")</f>
         <v/>
       </c>
       <c r="E37" s="29">
@@ -12406,7 +12682,7 @@
         </is>
       </c>
       <c r="D38" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR7.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR7.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.5*")</f>
         <v/>
       </c>
       <c r="E38" s="32">
@@ -12436,7 +12712,7 @@
         </is>
       </c>
       <c r="D39" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR8.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR8.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.1*")</f>
         <v/>
       </c>
       <c r="E39" s="29">
@@ -12466,7 +12742,7 @@
         </is>
       </c>
       <c r="D40" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR8.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR8.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.2*")</f>
         <v/>
       </c>
       <c r="E40" s="32">
@@ -12496,7 +12772,7 @@
         </is>
       </c>
       <c r="D41" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR8.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR8.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.3*")</f>
         <v/>
       </c>
       <c r="E41" s="29">
@@ -12526,7 +12802,7 @@
         </is>
       </c>
       <c r="D42" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR8.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR8.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.4*")</f>
         <v/>
       </c>
       <c r="E42" s="32">
@@ -12556,7 +12832,7 @@
         </is>
       </c>
       <c r="D43" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR9.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR9.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.1*")</f>
         <v/>
       </c>
       <c r="E43" s="29">
@@ -12586,7 +12862,7 @@
         </is>
       </c>
       <c r="D44" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR9.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR9.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.2*")</f>
         <v/>
       </c>
       <c r="E44" s="32">
@@ -12616,7 +12892,7 @@
         </is>
       </c>
       <c r="D45" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR9.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR9.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.3*")</f>
         <v/>
       </c>
       <c r="E45" s="29">
@@ -12646,7 +12922,7 @@
         </is>
       </c>
       <c r="D46" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR9.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR9.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.4*")</f>
         <v/>
       </c>
       <c r="E46" s="32">
@@ -12676,7 +12952,7 @@
         </is>
       </c>
       <c r="D47" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR9.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR9.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.5*")</f>
         <v/>
       </c>
       <c r="E47" s="29">
@@ -12706,7 +12982,7 @@
         </is>
       </c>
       <c r="D48" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR9.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR9.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.6*")</f>
         <v/>
       </c>
       <c r="E48" s="32">
@@ -12736,7 +13012,7 @@
         </is>
       </c>
       <c r="D49" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.7*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.7*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.7*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.7*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.7*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.7*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.7*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$45,"*FR9.7*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.7*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.7*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.7*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.7*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.7*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.7*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.7*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.7*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.7*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.7*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.7*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.7*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.7*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$49,"*FR9.7*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.7*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.7*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.7*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.7*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.7*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.7*")</f>
         <v/>
       </c>
       <c r="E49" s="29">

</xml_diff>

<commit_message>
test: admin console updates and call records results
</commit_message>
<xml_diff>
--- a/MediFind_Test_Requirements_v2.xlsx
+++ b/MediFind_Test_Requirements_v2.xlsx
@@ -1762,7 +1762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4112,44 +4112,44 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  LAYOUT &amp; ORIENTATION</t>
+          <t xml:space="preserve">  ADMIN CONSOLE UPDATES</t>
         </is>
       </c>
     </row>
     <row r="59" ht="40" customHeight="1">
       <c r="A59" s="37" t="inlineStr">
         <is>
-          <t>UX-01</t>
+          <t>ADM-01</t>
         </is>
       </c>
       <c r="B59" s="38" t="inlineStr">
         <is>
-          <t>NFR</t>
+          <t>FR10</t>
         </is>
       </c>
       <c r="C59" s="39" t="inlineStr">
         <is>
-          <t>Usability</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D59" s="39" t="inlineStr">
         <is>
-          <t>App stays in portrait when the phone is rotated</t>
+          <t>Branded admin sign-in page</t>
         </is>
       </c>
       <c r="E59" s="39" t="inlineStr">
         <is>
-          <t>Open the responder dashboard and rotate the phone</t>
+          <t>Open /login on desktop and mobile</t>
         </is>
       </c>
       <c r="F59" s="39" t="inlineStr">
         <is>
-          <t>Screen stays portrait; nothing squeezed or cut off</t>
+          <t>Brand panel + form; animations; works on mobile</t>
         </is>
       </c>
       <c r="G59" s="38" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H59" s="45" t="inlineStr">
@@ -4159,296 +4159,586 @@
       </c>
       <c r="I59" s="39" t="inlineStr">
         <is>
-          <t>2026-09-18: responder app on emulator rotated to landscape stays portrait (before: dashboard squeezed into a strip)</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="50" customHeight="1">
+          <t>2026-09-18: admin sign-in page split layout (brand panel + form), animated map backdrop on both sides, compact header on mobile; sign-in logic unchanged</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="40" customHeight="1">
       <c r="A60" s="41" t="inlineStr">
         <is>
-          <t>UX-02</t>
+          <t>ADM-02</t>
         </is>
       </c>
       <c r="B60" s="42" t="inlineStr">
         <is>
-          <t>NFR</t>
+          <t>FR10</t>
         </is>
       </c>
       <c r="C60" s="43" t="inlineStr">
         <is>
-          <t>Usability</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D60" s="43" t="inlineStr">
         <is>
-          <t>On a tablet or wide screen the app is centred, not stretched or stuck to one side</t>
+          <t>Maps follow dark mode</t>
         </is>
       </c>
       <c r="E60" s="43" t="inlineStr">
         <is>
-          <t>Open the app on a tablet (or web/desktop)</t>
+          <t>Switch the admin theme to dark and open Overview and SOS Logistics</t>
         </is>
       </c>
       <c r="F60" s="43" t="inlineStr">
         <is>
-          <t>App shown as a centred column with even margins</t>
+          <t>Dark map tiles, no watermark</t>
         </is>
       </c>
       <c r="G60" s="42" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H60" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I60" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-18: Overview and SOS Logistics maps use dark tiles in dark mode (filtered OSM, no API key) and light OSM in light mode</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="40" customHeight="1">
+      <c r="A61" s="37" t="inlineStr">
+        <is>
+          <t>ADM-03</t>
+        </is>
+      </c>
+      <c r="B61" s="38" t="inlineStr">
+        <is>
+          <t>FR10</t>
+        </is>
+      </c>
+      <c r="C61" s="39" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D61" s="39" t="inlineStr">
+        <is>
+          <t>User details open in a centred dialog</t>
+        </is>
+      </c>
+      <c r="E61" s="39" t="inlineStr">
+        <is>
+          <t>Click a user in User Management</t>
+        </is>
+      </c>
+      <c r="F61" s="39" t="inlineStr">
+        <is>
+          <t>Centred dialog with full details</t>
+        </is>
+      </c>
+      <c r="G61" s="38" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H61" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I61" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18: user details open as a centred dialog (light and dark), Escape/outside click close it</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="40" customHeight="1">
+      <c r="A62" s="41" t="inlineStr">
+        <is>
+          <t>ADM-04</t>
+        </is>
+      </c>
+      <c r="B62" s="42" t="inlineStr">
+        <is>
+          <t>FR10</t>
+        </is>
+      </c>
+      <c r="C62" s="43" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D62" s="43" t="inlineStr">
+        <is>
+          <t>Header search only navigates to real matches</t>
+        </is>
+      </c>
+      <c r="E62" s="43" t="inlineStr">
+        <is>
+          <t>Type random text, a page keyword and a user name; press Enter</t>
+        </is>
+      </c>
+      <c r="F62" s="43" t="inlineStr">
+        <is>
+          <t>Random text stays with a no-match message; matches open</t>
+        </is>
+      </c>
+      <c r="G62" s="42" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H60" s="45" t="inlineStr">
+      <c r="H62" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I60" s="43" t="inlineStr">
-        <is>
-          <t>2026-09-18: emulator resized to 1600x2560 tablet, portrait and landscape: centred 600dp column, no stretched or one-sided layout</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="50" customHeight="1">
-      <c r="A61" s="37" t="inlineStr">
-        <is>
-          <t>UX-04</t>
-        </is>
-      </c>
-      <c r="B61" s="44" t="inlineStr">
-        <is>
-          <t>Beyond SRS</t>
-        </is>
-      </c>
-      <c r="C61" s="39" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="D61" s="39" t="inlineStr">
-        <is>
-          <t>Checkout shows clear progress and a Stripe sheet in MediFind style</t>
-        </is>
-      </c>
-      <c r="E61" s="39" t="inlineStr">
-        <is>
-          <t>Tap Pay on checkout</t>
-        </is>
-      </c>
-      <c r="F61" s="39" t="inlineStr">
-        <is>
-          <t>Button says Opening secure payment…; sheet uses app colours and says Pay PKR …</t>
-        </is>
-      </c>
-      <c r="G61" s="38" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H61" s="45" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="I61" s="39" t="inlineStr">
-        <is>
-          <t>2026-09-18: Pay shows "Opening secure payment…" then "Confirming payment…"; Stripe sheet in app colours (light) with "Pay PKR 499" button</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="50" customHeight="1">
-      <c r="A62" s="41" t="inlineStr">
-        <is>
-          <t>UX-05</t>
-        </is>
-      </c>
-      <c r="B62" s="42" t="inlineStr">
-        <is>
-          <t>FR6.2</t>
-        </is>
-      </c>
-      <c r="C62" s="43" t="inlineStr">
-        <is>
-          <t>Tracking</t>
-        </is>
-      </c>
-      <c r="D62" s="43" t="inlineStr">
-        <is>
-          <t>Unrealistic GPS distance is not shown as an ETA</t>
-        </is>
-      </c>
-      <c r="E62" s="43" t="inlineStr">
-        <is>
-          <t>Responder phone reports a location hundreds of km away</t>
-        </is>
-      </c>
-      <c r="F62" s="43" t="inlineStr">
-        <is>
-          <t>Shows Locating / Waiting for GPS; no route line; map stays on the patient</t>
-        </is>
-      </c>
-      <c r="G62" s="42" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H62" s="45" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
       <c r="I62" s="43" t="inlineStr">
         <is>
-          <t>2026-09-18: responder GPS set to California: "Locating you / Waiting for GPS", no route line, camera on patient (was "17913 min, 11941 km"); back to Lahore: marker placed directly, "2 min · 1.3 km", normal zoom</t>
+          <t>2026-09-18: header search — random text shows "No pages or users match" and stays; "map" → SOS Logistics; "bilal" → user; ↑/↓ + Enter opens highlighted result</t>
         </is>
       </c>
     </row>
     <row r="63" ht="40" customHeight="1">
       <c r="A63" s="37" t="inlineStr">
         <is>
+          <t>ADM-05</t>
+        </is>
+      </c>
+      <c r="B63" s="38" t="inlineStr">
+        <is>
+          <t>NFR</t>
+        </is>
+      </c>
+      <c r="C63" s="39" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D63" s="39" t="inlineStr">
+        <is>
+          <t>Unknown URLs show a 404 page</t>
+        </is>
+      </c>
+      <c r="E63" s="39" t="inlineStr">
+        <is>
+          <t>Open a wrong public URL and a wrong /admin URL</t>
+        </is>
+      </c>
+      <c r="F63" s="39" t="inlineStr">
+        <is>
+          <t>Branded 404 pages</t>
+        </is>
+      </c>
+      <c r="G63" s="38" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H63" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I63" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18: wrong URLs show 404 — public /kuch-bhi-galat and admin /admin/galat-page</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="50" customHeight="1">
+      <c r="A64" s="41" t="inlineStr">
+        <is>
+          <t>CALL-12</t>
+        </is>
+      </c>
+      <c r="B64" s="46" t="inlineStr">
+        <is>
+          <t>Beyond SRS</t>
+        </is>
+      </c>
+      <c r="C64" s="43" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D64" s="43" t="inlineStr">
+        <is>
+          <t>Admin can review emergency call records</t>
+        </is>
+      </c>
+      <c r="E64" s="43" t="inlineStr">
+        <is>
+          <t>Make responder ↔ patient/caregiver calls, open Communication &gt; Call Records</t>
+        </is>
+      </c>
+      <c r="F64" s="43" t="inlineStr">
+        <is>
+          <t>Each call listed with outcome and duration; family calls not shown; no audio stored</t>
+        </is>
+      </c>
+      <c r="G64" s="42" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H64" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I64" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-18: Call Records page lists responder ↔ patient/caregiver calls (4 test calls: 3 completed, 1 not connected) with duration, outcome, end reason and emergency; patient ↔ caregiver calls excluded; non-admin gets 401</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  LAYOUT &amp; ORIENTATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="40" customHeight="1">
+      <c r="A66" s="37" t="inlineStr">
+        <is>
+          <t>UX-01</t>
+        </is>
+      </c>
+      <c r="B66" s="38" t="inlineStr">
+        <is>
+          <t>NFR</t>
+        </is>
+      </c>
+      <c r="C66" s="39" t="inlineStr">
+        <is>
+          <t>Usability</t>
+        </is>
+      </c>
+      <c r="D66" s="39" t="inlineStr">
+        <is>
+          <t>App stays in portrait when the phone is rotated</t>
+        </is>
+      </c>
+      <c r="E66" s="39" t="inlineStr">
+        <is>
+          <t>Open the responder dashboard and rotate the phone</t>
+        </is>
+      </c>
+      <c r="F66" s="39" t="inlineStr">
+        <is>
+          <t>Screen stays portrait; nothing squeezed or cut off</t>
+        </is>
+      </c>
+      <c r="G66" s="38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H66" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I66" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18: responder app on emulator rotated to landscape stays portrait (before: dashboard squeezed into a strip)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="50" customHeight="1">
+      <c r="A67" s="41" t="inlineStr">
+        <is>
+          <t>UX-02</t>
+        </is>
+      </c>
+      <c r="B67" s="42" t="inlineStr">
+        <is>
+          <t>NFR</t>
+        </is>
+      </c>
+      <c r="C67" s="43" t="inlineStr">
+        <is>
+          <t>Usability</t>
+        </is>
+      </c>
+      <c r="D67" s="43" t="inlineStr">
+        <is>
+          <t>On a tablet or wide screen the app is centred, not stretched or stuck to one side</t>
+        </is>
+      </c>
+      <c r="E67" s="43" t="inlineStr">
+        <is>
+          <t>Open the app on a tablet (or web/desktop)</t>
+        </is>
+      </c>
+      <c r="F67" s="43" t="inlineStr">
+        <is>
+          <t>App shown as a centred column with even margins</t>
+        </is>
+      </c>
+      <c r="G67" s="42" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H67" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I67" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-18: emulator resized to 1600x2560 tablet, portrait and landscape: centred 600dp column, no stretched or one-sided layout</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="50" customHeight="1">
+      <c r="A68" s="37" t="inlineStr">
+        <is>
+          <t>UX-04</t>
+        </is>
+      </c>
+      <c r="B68" s="44" t="inlineStr">
+        <is>
+          <t>Beyond SRS</t>
+        </is>
+      </c>
+      <c r="C68" s="39" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="D68" s="39" t="inlineStr">
+        <is>
+          <t>Checkout shows clear progress and a Stripe sheet in MediFind style</t>
+        </is>
+      </c>
+      <c r="E68" s="39" t="inlineStr">
+        <is>
+          <t>Tap Pay on checkout</t>
+        </is>
+      </c>
+      <c r="F68" s="39" t="inlineStr">
+        <is>
+          <t>Button says Opening secure payment…; sheet uses app colours and says Pay PKR …</t>
+        </is>
+      </c>
+      <c r="G68" s="38" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H68" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I68" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18: Pay shows "Opening secure payment…" then "Confirming payment…"; Stripe sheet in app colours (light) with "Pay PKR 499" button</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="50" customHeight="1">
+      <c r="A69" s="41" t="inlineStr">
+        <is>
+          <t>UX-05</t>
+        </is>
+      </c>
+      <c r="B69" s="42" t="inlineStr">
+        <is>
+          <t>FR6.2</t>
+        </is>
+      </c>
+      <c r="C69" s="43" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="D69" s="43" t="inlineStr">
+        <is>
+          <t>Unrealistic GPS distance is not shown as an ETA</t>
+        </is>
+      </c>
+      <c r="E69" s="43" t="inlineStr">
+        <is>
+          <t>Responder phone reports a location hundreds of km away</t>
+        </is>
+      </c>
+      <c r="F69" s="43" t="inlineStr">
+        <is>
+          <t>Shows Locating / Waiting for GPS; no route line; map stays on the patient</t>
+        </is>
+      </c>
+      <c r="G69" s="42" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H69" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I69" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-18: responder GPS set to California: "Locating you / Waiting for GPS", no route line, camera on patient (was "17913 min, 11941 km"); back to Lahore: marker placed directly, "2 min · 1.3 km", normal zoom</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="40" customHeight="1">
+      <c r="A70" s="37" t="inlineStr">
+        <is>
           <t>UX-06</t>
         </is>
       </c>
-      <c r="B63" s="38" t="inlineStr">
+      <c r="B70" s="38" t="inlineStr">
         <is>
           <t>NFR</t>
         </is>
       </c>
-      <c r="C63" s="39" t="inlineStr">
+      <c r="C70" s="39" t="inlineStr">
         <is>
           <t>Usability</t>
         </is>
       </c>
-      <c r="D63" s="39" t="inlineStr">
+      <c r="D70" s="39" t="inlineStr">
         <is>
           <t>Maps show a loading state instead of a blank box</t>
         </is>
       </c>
-      <c r="E63" s="39" t="inlineStr">
+      <c r="E70" s="39" t="inlineStr">
         <is>
           <t>Open a tracking screen</t>
         </is>
       </c>
-      <c r="F63" s="39" t="inlineStr">
+      <c r="F70" s="39" t="inlineStr">
         <is>
           <t>Loading map… until the map appears</t>
         </is>
       </c>
-      <c r="G63" s="38" t="inlineStr">
+      <c r="G70" s="38" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H63" s="45" t="inlineStr">
+      <c r="H70" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I63" s="39" t="inlineStr">
+      <c r="I70" s="39" t="inlineStr">
         <is>
           <t>2026-09-18: responder / patient / caregiver tracking maps show "Loading map…" until the map is ready (was a blank grey box)</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="40" customHeight="1">
-      <c r="A64" s="41" t="inlineStr">
+    <row r="71" ht="40" customHeight="1">
+      <c r="A71" s="41" t="inlineStr">
         <is>
           <t>UX-07</t>
         </is>
       </c>
-      <c r="B64" s="42" t="inlineStr">
+      <c r="B71" s="42" t="inlineStr">
         <is>
           <t>FR3.1</t>
         </is>
       </c>
-      <c r="C64" s="43" t="inlineStr">
+      <c r="C71" s="43" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D64" s="43" t="inlineStr">
+      <c r="D71" s="43" t="inlineStr">
         <is>
           <t>Deaf quick phrases are fully readable on the home screen</t>
         </is>
       </c>
-      <c r="E64" s="43" t="inlineStr">
+      <c r="E71" s="43" t="inlineStr">
         <is>
           <t>Open the Deaf patient home screen</t>
         </is>
       </c>
-      <c r="F64" s="43" t="inlineStr">
+      <c r="F71" s="43" t="inlineStr">
         <is>
           <t>Each phrase shown in full, wrapping onto lines</t>
         </is>
       </c>
-      <c r="G64" s="42" t="inlineStr">
+      <c r="G71" s="42" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H64" s="45" t="inlineStr">
+      <c r="H71" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I64" s="43" t="inlineStr">
+      <c r="I71" s="43" t="inlineStr">
         <is>
           <t>2026-09-18: Deaf home quick phrases wrap onto lines and are fully readable (was cut off "I am de…")</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="40" customHeight="1">
-      <c r="A65" s="37" t="inlineStr">
+    <row r="72" ht="40" customHeight="1">
+      <c r="A72" s="37" t="inlineStr">
         <is>
           <t>UX-03</t>
         </is>
       </c>
-      <c r="B65" s="38" t="inlineStr">
+      <c r="B72" s="38" t="inlineStr">
         <is>
           <t>NFR</t>
         </is>
       </c>
-      <c r="C65" s="39" t="inlineStr">
+      <c r="C72" s="39" t="inlineStr">
         <is>
           <t>Branding</t>
         </is>
       </c>
-      <c r="D65" s="39" t="inlineStr">
+      <c r="D72" s="39" t="inlineStr">
         <is>
           <t>The same MediFind logo is used in the mobile app and the web portal</t>
         </is>
       </c>
-      <c r="E65" s="39" t="inlineStr">
+      <c r="E72" s="39" t="inlineStr">
         <is>
           <t>Compare app launcher, splash, headers with portal sidebar, login, landing, 404, legal, favicon</t>
         </is>
       </c>
-      <c r="F65" s="39" t="inlineStr">
+      <c r="F72" s="39" t="inlineStr">
         <is>
           <t>One consistent logo everywhere</t>
         </is>
       </c>
-      <c r="G65" s="38" t="inlineStr">
+      <c r="G72" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H65" s="45" t="inlineStr">
+      <c r="H72" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I65" s="39" t="inlineStr">
+      <c r="I72" s="39" t="inlineStr">
         <is>
           <t>2026-09-18: portal sidebar, login, landing, 404, legal and favicon use the same pin-with-rings logo as the mobile app</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A15:I15"/>
     <mergeCell ref="A52:I52"/>
+    <mergeCell ref="A65:I65"/>
     <mergeCell ref="A11:I11"/>
     <mergeCell ref="A42:I42"/>
     <mergeCell ref="A32:I32"/>
@@ -4458,7 +4748,7 @@
     <mergeCell ref="A20:I20"/>
     <mergeCell ref="A38:I38"/>
   </mergeCells>
-  <conditionalFormatting sqref="H4:H65">
+  <conditionalFormatting sqref="H4:H72">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -4476,7 +4766,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H4:H65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid status" error="Choose PASS, FAIL, PENDING, BLOCKED or N/A" type="list">
+    <dataValidation sqref="H4:H72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid status" error="Choose PASS, FAIL, PENDING, BLOCKED or N/A" type="list">
       <formula1>"PENDING,PASS,FAIL,BLOCKED,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6732,12 +7022,16 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H4" s="40" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="I4" s="39" t="n"/>
+      <c r="H4" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I4" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18: admin sign-in page split layout (brand panel + form), animated map backdrop on both sides, compact header on mobile; sign-in logic unchanged</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="41" t="inlineStr">
@@ -6775,12 +7069,16 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H5" s="40" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="I5" s="43" t="n"/>
+      <c r="H5" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I5" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-18: Overview and SOS Logistics maps use dark tiles in dark mode (filtered OSM, no API key) and light OSM in light mode</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="37" t="inlineStr">
@@ -6819,12 +7117,16 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H6" s="40" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="I6" s="39" t="n"/>
+      <c r="H6" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I6" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18: user details open as a centred dialog (light and dark), Escape/outside click close it</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="36" t="inlineStr">
@@ -6871,12 +7173,16 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="H8" s="40" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="I8" s="39" t="n"/>
+      <c r="H8" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I8" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18: header search — random text shows "No pages or users match" and stays; "map" → SOS Logistics; "bilal" → user; ↑/↓ + Enter opens highlighted result</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="50" customHeight="1">
       <c r="A9" s="41" t="inlineStr">
@@ -6915,12 +7221,16 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="H9" s="40" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="I9" s="43" t="n"/>
+      <c r="H9" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I9" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-18: wrong URLs show 404 — public /kuch-bhi-galat and admin /admin/galat-page</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="37" t="inlineStr">
@@ -8167,7 +8477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D169"/>
+  <dimension ref="A1:D175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10738,7 +11048,7 @@
     <row r="118">
       <c r="A118" s="49" t="inlineStr">
         <is>
-          <t>UX-01</t>
+          <t>ADM-01</t>
         </is>
       </c>
       <c r="B118" s="49" t="inlineStr">
@@ -10748,19 +11058,19 @@
       </c>
       <c r="C118" s="49" t="inlineStr">
         <is>
-          <t>App stays in portrait when the phone is rotated</t>
+          <t>Branded admin sign-in page</t>
         </is>
       </c>
       <c r="D118" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR10</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="49" t="inlineStr">
         <is>
-          <t>UX-02</t>
+          <t>ADM-02</t>
         </is>
       </c>
       <c r="B119" s="49" t="inlineStr">
@@ -10770,19 +11080,19 @@
       </c>
       <c r="C119" s="49" t="inlineStr">
         <is>
-          <t>On a tablet or wide screen the app is centred, not stretched or stuck to one side</t>
+          <t>Maps follow dark mode</t>
         </is>
       </c>
       <c r="D119" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR10</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="49" t="inlineStr">
         <is>
-          <t>UX-04</t>
+          <t>ADM-03</t>
         </is>
       </c>
       <c r="B120" s="49" t="inlineStr">
@@ -10792,19 +11102,19 @@
       </c>
       <c r="C120" s="49" t="inlineStr">
         <is>
-          <t>Checkout shows clear progress and a Stripe sheet in MediFind style</t>
+          <t>User details open in a centred dialog</t>
         </is>
       </c>
       <c r="D120" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR10</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="49" t="inlineStr">
         <is>
-          <t>UX-05</t>
+          <t>ADM-04</t>
         </is>
       </c>
       <c r="B121" s="49" t="inlineStr">
@@ -10814,19 +11124,19 @@
       </c>
       <c r="C121" s="49" t="inlineStr">
         <is>
-          <t>Unrealistic GPS distance is not shown as an ETA</t>
+          <t>Header search only navigates to real matches</t>
         </is>
       </c>
       <c r="D121" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS FR6.2</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR10</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="49" t="inlineStr">
         <is>
-          <t>UX-06</t>
+          <t>ADM-05</t>
         </is>
       </c>
       <c r="B122" s="49" t="inlineStr">
@@ -10836,7 +11146,7 @@
       </c>
       <c r="C122" s="49" t="inlineStr">
         <is>
-          <t>Maps show a loading state instead of a blank box</t>
+          <t>Unknown URLs show a 404 page</t>
         </is>
       </c>
       <c r="D122" s="49" t="inlineStr">
@@ -10848,7 +11158,7 @@
     <row r="123">
       <c r="A123" s="49" t="inlineStr">
         <is>
-          <t>UX-07</t>
+          <t>CALL-12</t>
         </is>
       </c>
       <c r="B123" s="49" t="inlineStr">
@@ -10858,19 +11168,19 @@
       </c>
       <c r="C123" s="49" t="inlineStr">
         <is>
-          <t>Deaf quick phrases are fully readable on the home screen</t>
+          <t>Admin can review emergency call records</t>
         </is>
       </c>
       <c r="D123" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS FR3.1</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="49" t="inlineStr">
         <is>
-          <t>UX-03</t>
+          <t>UX-01</t>
         </is>
       </c>
       <c r="B124" s="49" t="inlineStr">
@@ -10880,7 +11190,7 @@
       </c>
       <c r="C124" s="49" t="inlineStr">
         <is>
-          <t>The same MediFind logo is used in the mobile app and the web portal</t>
+          <t>App stays in portrait when the phone is rotated</t>
         </is>
       </c>
       <c r="D124" s="49" t="inlineStr">
@@ -10892,7 +11202,7 @@
     <row r="125">
       <c r="A125" s="49" t="inlineStr">
         <is>
-          <t>MED-01</t>
+          <t>UX-02</t>
         </is>
       </c>
       <c r="B125" s="49" t="inlineStr">
@@ -10902,19 +11212,19 @@
       </c>
       <c r="C125" s="49" t="inlineStr">
         <is>
-          <t>Patient creates and edits the medical profile</t>
+          <t>On a tablet or wide screen the app is centred, not stretched or stuck to one side</t>
         </is>
       </c>
       <c r="D125" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.1, FR2.2</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="49" t="inlineStr">
         <is>
-          <t>MED-02</t>
+          <t>UX-04</t>
         </is>
       </c>
       <c r="B126" s="49" t="inlineStr">
@@ -10924,19 +11234,19 @@
       </c>
       <c r="C126" s="49" t="inlineStr">
         <is>
-          <t>Saving the medical profile keeps emergency contacts and quick phrases</t>
+          <t>Checkout shows clear progress and a Stripe sheet in MediFind style</t>
         </is>
       </c>
       <c r="D126" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.1</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="49" t="inlineStr">
         <is>
-          <t>MED-03</t>
+          <t>UX-05</t>
         </is>
       </c>
       <c r="B127" s="49" t="inlineStr">
@@ -10946,19 +11256,19 @@
       </c>
       <c r="C127" s="49" t="inlineStr">
         <is>
-          <t>Patient adds, calls and deletes emergency contacts</t>
+          <t>Unrealistic GPS distance is not shown as an ETA</t>
         </is>
       </c>
       <c r="D127" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.1</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR6.2</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="49" t="inlineStr">
         <is>
-          <t>MED-04</t>
+          <t>UX-06</t>
         </is>
       </c>
       <c r="B128" s="49" t="inlineStr">
@@ -10968,19 +11278,19 @@
       </c>
       <c r="C128" s="49" t="inlineStr">
         <is>
-          <t>Sensitive medical fields are encrypted at rest</t>
+          <t>Maps show a loading state instead of a blank box</t>
         </is>
       </c>
       <c r="D128" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.2</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="49" t="inlineStr">
         <is>
-          <t>MED-05</t>
+          <t>UX-07</t>
         </is>
       </c>
       <c r="B129" s="49" t="inlineStr">
@@ -10990,19 +11300,19 @@
       </c>
       <c r="C129" s="49" t="inlineStr">
         <is>
-          <t>Upload a report from camera, gallery (image) and PDF</t>
+          <t>Deaf quick phrases are fully readable on the home screen</t>
         </is>
       </c>
       <c r="D129" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.3</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR3.1</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="49" t="inlineStr">
         <is>
-          <t>MED-06</t>
+          <t>UX-03</t>
         </is>
       </c>
       <c r="B130" s="49" t="inlineStr">
@@ -11012,19 +11322,19 @@
       </c>
       <c r="C130" s="49" t="inlineStr">
         <is>
-          <t>Unsupported or oversized files are rejected with a clear message</t>
+          <t>The same MediFind logo is used in the mobile app and the web portal</t>
         </is>
       </c>
       <c r="D130" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.3</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="49" t="inlineStr">
         <is>
-          <t>MED-07</t>
+          <t>MED-01</t>
         </is>
       </c>
       <c r="B131" s="49" t="inlineStr">
@@ -11034,19 +11344,19 @@
       </c>
       <c r="C131" s="49" t="inlineStr">
         <is>
-          <t>View, rename and delete a report</t>
+          <t>Patient creates and edits the medical profile</t>
         </is>
       </c>
       <c r="D131" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.4</t>
+          <t>New sheet MEDICAL; SRS FR2.1, FR2.2</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="49" t="inlineStr">
         <is>
-          <t>MED-08</t>
+          <t>MED-02</t>
         </is>
       </c>
       <c r="B132" s="49" t="inlineStr">
@@ -11056,19 +11366,19 @@
       </c>
       <c r="C132" s="49" t="inlineStr">
         <is>
-          <t>Assigned responder receives the patient medical summary on accept</t>
+          <t>Saving the medical profile keeps emergency contacts and quick phrases</t>
         </is>
       </c>
       <c r="D132" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.5</t>
+          <t>New sheet MEDICAL; SRS FR2.1</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="49" t="inlineStr">
         <is>
-          <t>MED-09</t>
+          <t>MED-03</t>
         </is>
       </c>
       <c r="B133" s="49" t="inlineStr">
@@ -11078,19 +11388,19 @@
       </c>
       <c r="C133" s="49" t="inlineStr">
         <is>
-          <t>Report files are visible only to the patient, linked caregivers, the active responder and admins</t>
+          <t>Patient adds, calls and deletes emergency contacts</t>
         </is>
       </c>
       <c r="D133" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.6</t>
+          <t>New sheet MEDICAL; SRS FR2.1</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="49" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>MED-04</t>
         </is>
       </c>
       <c r="B134" s="49" t="inlineStr">
@@ -11100,19 +11410,19 @@
       </c>
       <c r="C134" s="49" t="inlineStr">
         <is>
-          <t>SOS requires press-and-hold before it starts</t>
+          <t>Sensitive medical fields are encrypted at rest</t>
         </is>
       </c>
       <c r="D134" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.1</t>
+          <t>New sheet MEDICAL; SRS FR2.2</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="49" t="inlineStr">
         <is>
-          <t>SEC-02</t>
+          <t>MED-05</t>
         </is>
       </c>
       <c r="B135" s="49" t="inlineStr">
@@ -11122,19 +11432,19 @@
       </c>
       <c r="C135" s="49" t="inlineStr">
         <is>
-          <t>Cancelling during the 60-second countdown sends nothing to the server</t>
+          <t>Upload a report from camera, gallery (image) and PDF</t>
         </is>
       </c>
       <c r="D135" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.3</t>
+          <t>New sheet MEDICAL; SRS FR2.3</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="49" t="inlineStr">
         <is>
-          <t>SEC-03</t>
+          <t>MED-06</t>
         </is>
       </c>
       <c r="B136" s="49" t="inlineStr">
@@ -11144,19 +11454,19 @@
       </c>
       <c r="C136" s="49" t="inlineStr">
         <is>
-          <t>SOS from a mock (fake) GPS location is refused in production</t>
+          <t>Unsupported or oversized files are rejected with a clear message</t>
         </is>
       </c>
       <c r="D136" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
+          <t>New sheet MEDICAL; SRS FR2.3</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="49" t="inlineStr">
         <is>
-          <t>SEC-04</t>
+          <t>MED-07</t>
         </is>
       </c>
       <c r="B137" s="49" t="inlineStr">
@@ -11166,19 +11476,19 @@
       </c>
       <c r="C137" s="49" t="inlineStr">
         <is>
-          <t>More than 5 SOS in one hour is refused</t>
+          <t>View, rename and delete a report</t>
         </is>
       </c>
       <c r="D137" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.5</t>
+          <t>New sheet MEDICAL; SRS FR2.4</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="49" t="inlineStr">
         <is>
-          <t>SEC-05</t>
+          <t>MED-08</t>
         </is>
       </c>
       <c r="B138" s="49" t="inlineStr">
@@ -11188,19 +11498,19 @@
       </c>
       <c r="C138" s="49" t="inlineStr">
         <is>
-          <t>SOS outside Pakistan coordinates is refused</t>
+          <t>Assigned responder receives the patient medical summary on accept</t>
         </is>
       </c>
       <c r="D138" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
+          <t>New sheet MEDICAL; SRS FR2.5</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="49" t="inlineStr">
         <is>
-          <t>SEC-06</t>
+          <t>MED-09</t>
         </is>
       </c>
       <c r="B139" s="49" t="inlineStr">
@@ -11210,19 +11520,19 @@
       </c>
       <c r="C139" s="49" t="inlineStr">
         <is>
-          <t>Responder must add a note when closing as False alarm or Patient not found</t>
+          <t>Report files are visible only to the patient, linked caregivers, the active responder and admins</t>
         </is>
       </c>
       <c r="D139" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR6.2</t>
+          <t>New sheet MEDICAL; SRS FR2.6</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="49" t="inlineStr">
         <is>
-          <t>SEC-07</t>
+          <t>SEC-01</t>
         </is>
       </c>
       <c r="B140" s="49" t="inlineStr">
@@ -11232,19 +11542,19 @@
       </c>
       <c r="C140" s="49" t="inlineStr">
         <is>
-          <t>Patient is warned when an SOS is marked as a false alarm</t>
+          <t>SOS requires press-and-hold before it starts</t>
         </is>
       </c>
       <c r="D140" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; beyond SRS</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.1</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="49" t="inlineStr">
         <is>
-          <t>SEC-08</t>
+          <t>SEC-02</t>
         </is>
       </c>
       <c r="B141" s="49" t="inlineStr">
@@ -11254,19 +11564,19 @@
       </c>
       <c r="C141" s="49" t="inlineStr">
         <is>
-          <t>3 false alarms in 30 days alerts admins for review</t>
+          <t>Cancelling during the 60-second countdown sends nothing to the server</t>
         </is>
       </c>
       <c r="D141" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; beyond SRS</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.3</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="49" t="inlineStr">
         <is>
-          <t>SEC-09</t>
+          <t>SEC-03</t>
         </is>
       </c>
       <c r="B142" s="49" t="inlineStr">
@@ -11276,19 +11586,19 @@
       </c>
       <c r="C142" s="49" t="inlineStr">
         <is>
-          <t>Patient-cancelled SOS never counts as a false alarm</t>
+          <t>SOS from a mock (fake) GPS location is refused in production</t>
         </is>
       </c>
       <c r="D142" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; beyond SRS</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="49" t="inlineStr">
         <is>
-          <t>SEC-10</t>
+          <t>SEC-04</t>
         </is>
       </c>
       <c r="B143" s="49" t="inlineStr">
@@ -11298,19 +11608,19 @@
       </c>
       <c r="C143" s="49" t="inlineStr">
         <is>
-          <t>Refresh token cannot be used as an access token</t>
+          <t>More than 5 SOS in one hour is refused</t>
         </is>
       </c>
       <c r="D143" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.5</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="49" t="inlineStr">
         <is>
-          <t>SEC-11</t>
+          <t>SEC-05</t>
         </is>
       </c>
       <c r="B144" s="49" t="inlineStr">
@@ -11320,19 +11630,19 @@
       </c>
       <c r="C144" s="49" t="inlineStr">
         <is>
-          <t>Users cannot join emergency or chat rooms they do not belong to</t>
+          <t>SOS outside Pakistan coordinates is refused</t>
         </is>
       </c>
       <c r="D144" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="49" t="inlineStr">
         <is>
-          <t>SEC-12</t>
+          <t>SEC-06</t>
         </is>
       </c>
       <c r="B145" s="49" t="inlineStr">
@@ -11342,19 +11652,19 @@
       </c>
       <c r="C145" s="49" t="inlineStr">
         <is>
-          <t>Paid plan upgrade requires a verified Stripe payment</t>
+          <t>Responder must add a note when closing as False alarm or Patient not found</t>
         </is>
       </c>
       <c r="D145" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; beyond SRS</t>
+          <t>New sheet SECURITY_SOS; SRS FR6.2</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="49" t="inlineStr">
         <is>
-          <t>SEC-13</t>
+          <t>SEC-07</t>
         </is>
       </c>
       <c r="B146" s="49" t="inlineStr">
@@ -11364,19 +11674,19 @@
       </c>
       <c r="C146" s="49" t="inlineStr">
         <is>
-          <t>Only the assigned responder can update or resolve an emergency</t>
+          <t>Patient is warned when an SOS is marked as a false alarm</t>
         </is>
       </c>
       <c r="D146" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR5.1</t>
+          <t>New sheet SECURITY_SOS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="49" t="inlineStr">
         <is>
-          <t>NAV-01</t>
+          <t>SEC-08</t>
         </is>
       </c>
       <c r="B147" s="49" t="inlineStr">
@@ -11386,19 +11696,19 @@
       </c>
       <c r="C147" s="49" t="inlineStr">
         <is>
-          <t>Each role has a unified sidebar (AppDrawer) with role-specific items</t>
+          <t>3 false alarms in 30 days alerts admins for review</t>
         </is>
       </c>
       <c r="D147" s="49" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.1</t>
+          <t>New sheet SECURITY_SOS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="49" t="inlineStr">
         <is>
-          <t>NAV-02</t>
+          <t>SEC-09</t>
         </is>
       </c>
       <c r="B148" s="49" t="inlineStr">
@@ -11408,19 +11718,19 @@
       </c>
       <c r="C148" s="49" t="inlineStr">
         <is>
-          <t>Switching tabs preserves each tab's state and back navigation works</t>
+          <t>Patient-cancelled SOS never counts as a false alarm</t>
         </is>
       </c>
       <c r="D148" s="49" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.2</t>
+          <t>New sheet SECURITY_SOS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="49" t="inlineStr">
         <is>
-          <t>NAV-03</t>
+          <t>SEC-10</t>
         </is>
       </c>
       <c r="B149" s="49" t="inlineStr">
@@ -11430,19 +11740,19 @@
       </c>
       <c r="C149" s="49" t="inlineStr">
         <is>
-          <t>Role dashboards show quick action grids</t>
+          <t>Refresh token cannot be used as an access token</t>
         </is>
       </c>
       <c r="D149" s="49" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.3</t>
+          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="49" t="inlineStr">
         <is>
-          <t>NAV-04</t>
+          <t>SEC-11</t>
         </is>
       </c>
       <c r="B150" s="49" t="inlineStr">
@@ -11452,19 +11762,19 @@
       </c>
       <c r="C150" s="49" t="inlineStr">
         <is>
-          <t>Map and chat screens render smoothly (~60 FPS)</t>
+          <t>Users cannot join emergency or chat rooms they do not belong to</t>
         </is>
       </c>
       <c r="D150" s="49" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.4</t>
+          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="49" t="inlineStr">
         <is>
-          <t>NAV-05</t>
+          <t>SEC-12</t>
         </is>
       </c>
       <c r="B151" s="49" t="inlineStr">
@@ -11474,151 +11784,151 @@
       </c>
       <c r="C151" s="49" t="inlineStr">
         <is>
-          <t>Large buttons mode enlarges tap targets across screens</t>
+          <t>Paid plan upgrade requires a verified Stripe payment</t>
         </is>
       </c>
       <c r="D151" s="49" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR3.5</t>
+          <t>New sheet SECURITY_SOS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="49" t="inlineStr">
         <is>
-          <t>PRF-01</t>
+          <t>SEC-13</t>
         </is>
       </c>
       <c r="B152" s="49" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C152" s="49" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Only the assigned responder can update or resolve an emergency</t>
         </is>
       </c>
       <c r="D152" s="49" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet SECURITY_SOS; SRS FR5.1</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="49" t="inlineStr">
         <is>
-          <t>PRF-02</t>
+          <t>NAV-01</t>
         </is>
       </c>
       <c r="B153" s="49" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C153" s="49" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Each role has a unified sidebar (AppDrawer) with role-specific items</t>
         </is>
       </c>
       <c r="D153" s="49" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.1</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="49" t="inlineStr">
         <is>
-          <t>PRF-03</t>
+          <t>NAV-02</t>
         </is>
       </c>
       <c r="B154" s="49" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C154" s="49" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Switching tabs preserves each tab's state and back navigation works</t>
         </is>
       </c>
       <c r="D154" s="49" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.2</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="49" t="inlineStr">
         <is>
-          <t>PRF-05</t>
+          <t>NAV-03</t>
         </is>
       </c>
       <c r="B155" s="49" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C155" s="49" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Role dashboards show quick action grids</t>
         </is>
       </c>
       <c r="D155" s="49" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.3</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="49" t="inlineStr">
         <is>
-          <t>NTF-01</t>
+          <t>NAV-04</t>
         </is>
       </c>
       <c r="B156" s="49" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C156" s="49" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Map and chat screens render smoothly (~60 FPS)</t>
         </is>
       </c>
       <c r="D156" s="49" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.4</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="49" t="inlineStr">
         <is>
-          <t>NTF-02</t>
+          <t>NAV-05</t>
         </is>
       </c>
       <c r="B157" s="49" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C157" s="49" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Large buttons mode enlarges tap targets across screens</t>
         </is>
       </c>
       <c r="D157" s="49" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR3.5</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="49" t="inlineStr">
         <is>
-          <t>NTF-03</t>
+          <t>PRF-01</t>
         </is>
       </c>
       <c r="B158" s="49" t="inlineStr">
@@ -11640,7 +11950,7 @@
     <row r="159">
       <c r="A159" s="49" t="inlineStr">
         <is>
-          <t>NTF-04</t>
+          <t>PRF-02</t>
         </is>
       </c>
       <c r="B159" s="49" t="inlineStr">
@@ -11662,7 +11972,7 @@
     <row r="160">
       <c r="A160" s="49" t="inlineStr">
         <is>
-          <t>NTF-05</t>
+          <t>PRF-03</t>
         </is>
       </c>
       <c r="B160" s="49" t="inlineStr">
@@ -11684,7 +11994,7 @@
     <row r="161">
       <c r="A161" s="49" t="inlineStr">
         <is>
-          <t>NTF-07</t>
+          <t>PRF-05</t>
         </is>
       </c>
       <c r="B161" s="49" t="inlineStr">
@@ -11706,7 +12016,7 @@
     <row r="162">
       <c r="A162" s="49" t="inlineStr">
         <is>
-          <t>NTF-08</t>
+          <t>NTF-01</t>
         </is>
       </c>
       <c r="B162" s="49" t="inlineStr">
@@ -11728,7 +12038,7 @@
     <row r="163">
       <c r="A163" s="49" t="inlineStr">
         <is>
-          <t>ACC-06</t>
+          <t>NTF-02</t>
         </is>
       </c>
       <c r="B163" s="49" t="inlineStr">
@@ -11750,7 +12060,7 @@
     <row r="164">
       <c r="A164" s="49" t="inlineStr">
         <is>
-          <t>ACC-07</t>
+          <t>NTF-03</t>
         </is>
       </c>
       <c r="B164" s="49" t="inlineStr">
@@ -11772,7 +12082,7 @@
     <row r="165">
       <c r="A165" s="49" t="inlineStr">
         <is>
-          <t>ACC-11</t>
+          <t>NTF-04</t>
         </is>
       </c>
       <c r="B165" s="49" t="inlineStr">
@@ -11794,7 +12104,7 @@
     <row r="166">
       <c r="A166" s="49" t="inlineStr">
         <is>
-          <t>AUTH-12</t>
+          <t>NTF-05</t>
         </is>
       </c>
       <c r="B166" s="49" t="inlineStr">
@@ -11816,7 +12126,7 @@
     <row r="167">
       <c r="A167" s="49" t="inlineStr">
         <is>
-          <t>API-04</t>
+          <t>NTF-07</t>
         </is>
       </c>
       <c r="B167" s="49" t="inlineStr">
@@ -11838,7 +12148,7 @@
     <row r="168">
       <c r="A168" s="49" t="inlineStr">
         <is>
-          <t>API-08</t>
+          <t>NTF-08</t>
         </is>
       </c>
       <c r="B168" s="49" t="inlineStr">
@@ -11860,20 +12170,152 @@
     <row r="169">
       <c r="A169" s="49" t="inlineStr">
         <is>
+          <t>ACC-06</t>
+        </is>
+      </c>
+      <c r="B169" s="49" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C169" s="49" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D169" s="49" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="49" t="inlineStr">
+        <is>
+          <t>ACC-07</t>
+        </is>
+      </c>
+      <c r="B170" s="49" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C170" s="49" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D170" s="49" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="49" t="inlineStr">
+        <is>
+          <t>ACC-11</t>
+        </is>
+      </c>
+      <c r="B171" s="49" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C171" s="49" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D171" s="49" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="49" t="inlineStr">
+        <is>
+          <t>AUTH-12</t>
+        </is>
+      </c>
+      <c r="B172" s="49" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C172" s="49" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D172" s="49" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="49" t="inlineStr">
+        <is>
+          <t>API-04</t>
+        </is>
+      </c>
+      <c r="B173" s="49" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C173" s="49" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D173" s="49" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="49" t="inlineStr">
+        <is>
+          <t>API-08</t>
+        </is>
+      </c>
+      <c r="B174" s="49" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C174" s="49" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D174" s="49" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="49" t="inlineStr">
+        <is>
           <t>API-09</t>
         </is>
       </c>
-      <c r="B169" s="49" t="inlineStr">
+      <c r="B175" s="49" t="inlineStr">
         <is>
           <t>Re-classified</t>
         </is>
       </c>
-      <c r="C169" s="49" t="inlineStr">
+      <c r="C175" s="49" t="inlineStr">
         <is>
           <t>Marked "Beyond SRS" in the SRS Ref column</t>
         </is>
       </c>
-      <c r="D169" s="49" t="inlineStr">
+      <c r="D175" s="49" t="inlineStr">
         <is>
           <t>Valid feature test with no matching SRS functional requirement</t>
         </is>
@@ -12237,27 +12679,27 @@
         </is>
       </c>
       <c r="C11" s="19">
-        <f>COUNTA(PRIVACY_CALLS!$A$4:$A$65)-COUNTIF(PRIVACY_CALLS!$A$4:$A$65,"  *")</f>
+        <f>COUNTA(PRIVACY_CALLS!$A$4:$A$72)-COUNTIF(PRIVACY_CALLS!$A$4:$A$72,"  *")</f>
         <v/>
       </c>
       <c r="D11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$65,"PASS")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$72,"PASS")</f>
         <v/>
       </c>
       <c r="E11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$65,"FAIL")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$72,"FAIL")</f>
         <v/>
       </c>
       <c r="F11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$65,"PENDING")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$72,"PENDING")</f>
         <v/>
       </c>
       <c r="G11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$65,"BLOCKED")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$72,"BLOCKED")</f>
         <v/>
       </c>
       <c r="H11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$65,"N/A")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$72,"N/A")</f>
         <v/>
       </c>
       <c r="I11" s="21">
@@ -12617,7 +13059,7 @@
         </is>
       </c>
       <c r="D3" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR1.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR1.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.1*")</f>
         <v/>
       </c>
       <c r="E3" s="29">
@@ -12647,7 +13089,7 @@
         </is>
       </c>
       <c r="D4" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR1.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR1.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.2*")</f>
         <v/>
       </c>
       <c r="E4" s="32">
@@ -12677,7 +13119,7 @@
         </is>
       </c>
       <c r="D5" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR1.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR1.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.3*")</f>
         <v/>
       </c>
       <c r="E5" s="29">
@@ -12707,7 +13149,7 @@
         </is>
       </c>
       <c r="D6" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR1.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR1.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.4*")</f>
         <v/>
       </c>
       <c r="E6" s="32">
@@ -12737,7 +13179,7 @@
         </is>
       </c>
       <c r="D7" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR1.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR1.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.5*")</f>
         <v/>
       </c>
       <c r="E7" s="29">
@@ -12767,7 +13209,7 @@
         </is>
       </c>
       <c r="D8" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR1.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR1.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.6*")</f>
         <v/>
       </c>
       <c r="E8" s="32">
@@ -12797,7 +13239,7 @@
         </is>
       </c>
       <c r="D9" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR2.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR2.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.1*")</f>
         <v/>
       </c>
       <c r="E9" s="29">
@@ -12827,7 +13269,7 @@
         </is>
       </c>
       <c r="D10" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR2.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR2.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.2*")</f>
         <v/>
       </c>
       <c r="E10" s="32">
@@ -12857,7 +13299,7 @@
         </is>
       </c>
       <c r="D11" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR2.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR2.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.3*")</f>
         <v/>
       </c>
       <c r="E11" s="29">
@@ -12887,7 +13329,7 @@
         </is>
       </c>
       <c r="D12" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR2.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR2.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.4*")</f>
         <v/>
       </c>
       <c r="E12" s="32">
@@ -12917,7 +13359,7 @@
         </is>
       </c>
       <c r="D13" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR2.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR2.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.5*")</f>
         <v/>
       </c>
       <c r="E13" s="29">
@@ -12947,7 +13389,7 @@
         </is>
       </c>
       <c r="D14" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR2.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR2.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.6*")</f>
         <v/>
       </c>
       <c r="E14" s="32">
@@ -12977,7 +13419,7 @@
         </is>
       </c>
       <c r="D15" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR3.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR3.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.1*")</f>
         <v/>
       </c>
       <c r="E15" s="29">
@@ -13007,7 +13449,7 @@
         </is>
       </c>
       <c r="D16" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR3.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR3.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.2*")</f>
         <v/>
       </c>
       <c r="E16" s="32">
@@ -13037,7 +13479,7 @@
         </is>
       </c>
       <c r="D17" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR3.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR3.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.3*")</f>
         <v/>
       </c>
       <c r="E17" s="29">
@@ -13067,7 +13509,7 @@
         </is>
       </c>
       <c r="D18" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR3.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR3.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.4*")</f>
         <v/>
       </c>
       <c r="E18" s="32">
@@ -13097,7 +13539,7 @@
         </is>
       </c>
       <c r="D19" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR3.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR3.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.5*")</f>
         <v/>
       </c>
       <c r="E19" s="29">
@@ -13127,7 +13569,7 @@
         </is>
       </c>
       <c r="D20" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR4.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR4.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.1*")</f>
         <v/>
       </c>
       <c r="E20" s="32">
@@ -13157,7 +13599,7 @@
         </is>
       </c>
       <c r="D21" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR4.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR4.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.2*")</f>
         <v/>
       </c>
       <c r="E21" s="29">
@@ -13187,7 +13629,7 @@
         </is>
       </c>
       <c r="D22" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR4.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR4.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.3*")</f>
         <v/>
       </c>
       <c r="E22" s="32">
@@ -13217,7 +13659,7 @@
         </is>
       </c>
       <c r="D23" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR4.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR4.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.4*")</f>
         <v/>
       </c>
       <c r="E23" s="29">
@@ -13247,7 +13689,7 @@
         </is>
       </c>
       <c r="D24" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR4.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR4.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.5*")</f>
         <v/>
       </c>
       <c r="E24" s="32">
@@ -13277,7 +13719,7 @@
         </is>
       </c>
       <c r="D25" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR4.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR4.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.6*")</f>
         <v/>
       </c>
       <c r="E25" s="29">
@@ -13307,7 +13749,7 @@
         </is>
       </c>
       <c r="D26" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR5.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR5.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.1*")</f>
         <v/>
       </c>
       <c r="E26" s="32">
@@ -13337,7 +13779,7 @@
         </is>
       </c>
       <c r="D27" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR5.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR5.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.2*")</f>
         <v/>
       </c>
       <c r="E27" s="29">
@@ -13367,7 +13809,7 @@
         </is>
       </c>
       <c r="D28" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR5.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR5.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.3*")</f>
         <v/>
       </c>
       <c r="E28" s="32">
@@ -13397,7 +13839,7 @@
         </is>
       </c>
       <c r="D29" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR5.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR5.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.4*")</f>
         <v/>
       </c>
       <c r="E29" s="29">
@@ -13427,7 +13869,7 @@
         </is>
       </c>
       <c r="D30" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR6.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR6.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.1*")</f>
         <v/>
       </c>
       <c r="E30" s="32">
@@ -13457,7 +13899,7 @@
         </is>
       </c>
       <c r="D31" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR6.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR6.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.2*")</f>
         <v/>
       </c>
       <c r="E31" s="29">
@@ -13487,7 +13929,7 @@
         </is>
       </c>
       <c r="D32" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR6.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR6.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.3*")</f>
         <v/>
       </c>
       <c r="E32" s="32">
@@ -13517,7 +13959,7 @@
         </is>
       </c>
       <c r="D33" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR6.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR6.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.4*")</f>
         <v/>
       </c>
       <c r="E33" s="29">
@@ -13547,7 +13989,7 @@
         </is>
       </c>
       <c r="D34" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR7.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR7.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.1*")</f>
         <v/>
       </c>
       <c r="E34" s="32">
@@ -13577,7 +14019,7 @@
         </is>
       </c>
       <c r="D35" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR7.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR7.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.2*")</f>
         <v/>
       </c>
       <c r="E35" s="29">
@@ -13607,7 +14049,7 @@
         </is>
       </c>
       <c r="D36" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR7.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR7.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.3*")</f>
         <v/>
       </c>
       <c r="E36" s="32">
@@ -13637,7 +14079,7 @@
         </is>
       </c>
       <c r="D37" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR7.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR7.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.4*")</f>
         <v/>
       </c>
       <c r="E37" s="29">
@@ -13667,7 +14109,7 @@
         </is>
       </c>
       <c r="D38" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR7.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR7.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.5*")</f>
         <v/>
       </c>
       <c r="E38" s="32">
@@ -13697,7 +14139,7 @@
         </is>
       </c>
       <c r="D39" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR8.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR8.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.1*")</f>
         <v/>
       </c>
       <c r="E39" s="29">
@@ -13727,7 +14169,7 @@
         </is>
       </c>
       <c r="D40" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR8.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR8.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.2*")</f>
         <v/>
       </c>
       <c r="E40" s="32">
@@ -13757,7 +14199,7 @@
         </is>
       </c>
       <c r="D41" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR8.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR8.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.3*")</f>
         <v/>
       </c>
       <c r="E41" s="29">
@@ -13787,7 +14229,7 @@
         </is>
       </c>
       <c r="D42" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR8.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR8.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.4*")</f>
         <v/>
       </c>
       <c r="E42" s="32">
@@ -13817,7 +14259,7 @@
         </is>
       </c>
       <c r="D43" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR9.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR9.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.1*")</f>
         <v/>
       </c>
       <c r="E43" s="29">
@@ -13847,7 +14289,7 @@
         </is>
       </c>
       <c r="D44" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR9.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR9.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.2*")</f>
         <v/>
       </c>
       <c r="E44" s="32">
@@ -13877,7 +14319,7 @@
         </is>
       </c>
       <c r="D45" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR9.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR9.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.3*")</f>
         <v/>
       </c>
       <c r="E45" s="29">
@@ -13907,7 +14349,7 @@
         </is>
       </c>
       <c r="D46" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR9.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR9.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.4*")</f>
         <v/>
       </c>
       <c r="E46" s="32">
@@ -13937,7 +14379,7 @@
         </is>
       </c>
       <c r="D47" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR9.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR9.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.5*")</f>
         <v/>
       </c>
       <c r="E47" s="29">
@@ -13967,7 +14409,7 @@
         </is>
       </c>
       <c r="D48" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR9.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR9.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.6*")</f>
         <v/>
       </c>
       <c r="E48" s="32">
@@ -13997,7 +14439,7 @@
         </is>
       </c>
       <c r="D49" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.7*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.7*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.7*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.7*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.7*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.7*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.7*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$65,"*FR9.7*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.7*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.7*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.7*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.7*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.7*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.7*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.7*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.7*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.7*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.7*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.7*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.7*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.7*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR9.7*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.7*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.7*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.7*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.7*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.7*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.7*")</f>
         <v/>
       </c>
       <c r="E49" s="29">

</xml_diff>

<commit_message>
test(sheet): record real-phone results for calls, voice notes, chat and REL-03
</commit_message>
<xml_diff>
--- a/MediFind_Test_Requirements_v2.xlsx
+++ b/MediFind_Test_Requirements_v2.xlsx
@@ -1762,7 +1762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3050,44 +3050,44 @@
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  PERFORMANCE &amp; AI</t>
+          <t xml:space="preserve">  REAL PHONE CHECKS</t>
         </is>
       </c>
     </row>
     <row r="33" ht="40" customHeight="1">
       <c r="A33" s="37" t="inlineStr">
         <is>
-          <t>PERF-01</t>
-        </is>
-      </c>
-      <c r="B33" s="38" t="inlineStr">
-        <is>
-          <t>FR8.4</t>
+          <t>CALL-13</t>
+        </is>
+      </c>
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t>Beyond SRS</t>
         </is>
       </c>
       <c r="C33" s="39" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Call quality</t>
         </is>
       </c>
       <c r="D33" s="39" t="inlineStr">
         <is>
-          <t>SOS countdown opens immediately after Send SOS</t>
+          <t>Voice call on real phones is clear</t>
         </is>
       </c>
       <c r="E33" s="39" t="inlineStr">
         <is>
-          <t>Send SOS with location already known</t>
+          <t>Two phones in separate rooms; make a voice call and talk</t>
         </is>
       </c>
       <c r="F33" s="39" t="inlineStr">
         <is>
-          <t>Countdown visible within 1 s (location refined during the countdown)</t>
+          <t>Sound from the earpiece; no echo, hiss or background noise</t>
         </is>
       </c>
       <c r="G33" s="38" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H33" s="45" t="inlineStr">
@@ -3097,39 +3097,39 @@
       </c>
       <c r="I33" s="39" t="inlineStr">
         <is>
-          <t>2026-09-17: emulator recording — countdown visible ~0.1 s after Send SOS (was 8–10 s waiting for GPS)</t>
+          <t>2026-09-19: real phones in separate rooms — voice call clear through the earpiece, no echo or background noise (fixed: calls were routed to the loudspeaker; WebRTC communication audio mode + echo/noise constraints)</t>
         </is>
       </c>
     </row>
     <row r="34" ht="40" customHeight="1">
       <c r="A34" s="41" t="inlineStr">
         <is>
-          <t>PERF-02</t>
-        </is>
-      </c>
-      <c r="B34" s="42" t="inlineStr">
-        <is>
-          <t>FR8.4</t>
+          <t>CALL-14</t>
+        </is>
+      </c>
+      <c r="B34" s="46" t="inlineStr">
+        <is>
+          <t>Beyond SRS</t>
         </is>
       </c>
       <c r="C34" s="43" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Call quality</t>
         </is>
       </c>
       <c r="D34" s="43" t="inlineStr">
         <is>
-          <t>Responder reaches navigation right after accepting</t>
+          <t>Video call on real phones is clear</t>
         </is>
       </c>
       <c r="E34" s="43" t="inlineStr">
         <is>
-          <t>Accept an emergency</t>
+          <t>Two phones in separate rooms; make a video call and talk</t>
         </is>
       </c>
       <c r="F34" s="43" t="inlineStr">
         <is>
-          <t>Active emergency screen within ~1 s</t>
+          <t>Speaker audio without echo or noise; video both ways</t>
         </is>
       </c>
       <c r="G34" s="42" t="inlineStr">
@@ -3144,44 +3144,44 @@
       </c>
       <c r="I34" s="43" t="inlineStr">
         <is>
-          <t>2026-09-17: responder reaches navigation ~1 s after Accept (was ~15 s)</t>
+          <t>2026-09-19: real phones — video call on speaker without echo or noise</t>
         </is>
       </c>
     </row>
     <row r="35" ht="40" customHeight="1">
       <c r="A35" s="37" t="inlineStr">
         <is>
-          <t>PERF-03</t>
+          <t>MSG-01</t>
         </is>
       </c>
       <c r="B35" s="38" t="inlineStr">
         <is>
-          <t>FR6.2</t>
+          <t>FR7.3</t>
         </is>
       </c>
       <c r="C35" s="39" t="inlineStr">
         <is>
-          <t>Tracking</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="D35" s="39" t="inlineStr">
         <is>
-          <t>Responder marker moves smoothly along the road</t>
+          <t>Voice note is sent and plays</t>
         </is>
       </c>
       <c r="E35" s="39" t="inlineStr">
         <is>
-          <t>Watch the tracking map during a drive</t>
+          <t>Record a voice note in chat and send it</t>
         </is>
       </c>
       <c r="F35" s="39" t="inlineStr">
         <is>
-          <t>No backward jumps or U-turn loops; heading follows the road</t>
+          <t>Voice note appears for both sides and plays</t>
         </is>
       </c>
       <c r="G35" s="38" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H35" s="45" t="inlineStr">
@@ -3191,1564 +3191,1760 @@
       </c>
       <c r="I35" s="39" t="inlineStr">
         <is>
-          <t>2026-09-17: frame analysis — no backward jumps or U-turn loops; remaining ~0.3 s marker blink about every 16 s on the emulator (route redraw)</t>
+          <t>2026-09-19: real phone — voice note records, sends and plays on the other side (fixed: upload response shape and relative media URL)</t>
         </is>
       </c>
     </row>
     <row r="36" ht="40" customHeight="1">
       <c r="A36" s="41" t="inlineStr">
         <is>
+          <t>MSG-02</t>
+        </is>
+      </c>
+      <c r="B36" s="42" t="inlineStr">
+        <is>
+          <t>FR7.3</t>
+        </is>
+      </c>
+      <c r="C36" s="43" t="inlineStr">
+        <is>
+          <t>Chat</t>
+        </is>
+      </c>
+      <c r="D36" s="43" t="inlineStr">
+        <is>
+          <t>Text chat works between real phones</t>
+        </is>
+      </c>
+      <c r="E36" s="43" t="inlineStr">
+        <is>
+          <t>Send messages from both phones</t>
+        </is>
+      </c>
+      <c r="F36" s="43" t="inlineStr">
+        <is>
+          <t>Messages delivered both ways in real time</t>
+        </is>
+      </c>
+      <c r="G36" s="42" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H36" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I36" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-19: real phones — text chat messages delivered both ways in real time</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PERFORMANCE &amp; AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="40" customHeight="1">
+      <c r="A38" s="37" t="inlineStr">
+        <is>
+          <t>PERF-01</t>
+        </is>
+      </c>
+      <c r="B38" s="38" t="inlineStr">
+        <is>
+          <t>FR8.4</t>
+        </is>
+      </c>
+      <c r="C38" s="39" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="D38" s="39" t="inlineStr">
+        <is>
+          <t>SOS countdown opens immediately after Send SOS</t>
+        </is>
+      </c>
+      <c r="E38" s="39" t="inlineStr">
+        <is>
+          <t>Send SOS with location already known</t>
+        </is>
+      </c>
+      <c r="F38" s="39" t="inlineStr">
+        <is>
+          <t>Countdown visible within 1 s (location refined during the countdown)</t>
+        </is>
+      </c>
+      <c r="G38" s="38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H38" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I38" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-17: emulator recording — countdown visible ~0.1 s after Send SOS (was 8–10 s waiting for GPS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="40" customHeight="1">
+      <c r="A39" s="41" t="inlineStr">
+        <is>
+          <t>PERF-02</t>
+        </is>
+      </c>
+      <c r="B39" s="42" t="inlineStr">
+        <is>
+          <t>FR8.4</t>
+        </is>
+      </c>
+      <c r="C39" s="43" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="D39" s="43" t="inlineStr">
+        <is>
+          <t>Responder reaches navigation right after accepting</t>
+        </is>
+      </c>
+      <c r="E39" s="43" t="inlineStr">
+        <is>
+          <t>Accept an emergency</t>
+        </is>
+      </c>
+      <c r="F39" s="43" t="inlineStr">
+        <is>
+          <t>Active emergency screen within ~1 s</t>
+        </is>
+      </c>
+      <c r="G39" s="42" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H39" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I39" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-17: responder reaches navigation ~1 s after Accept (was ~15 s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="40" customHeight="1">
+      <c r="A40" s="37" t="inlineStr">
+        <is>
+          <t>PERF-03</t>
+        </is>
+      </c>
+      <c r="B40" s="38" t="inlineStr">
+        <is>
+          <t>FR6.2</t>
+        </is>
+      </c>
+      <c r="C40" s="39" t="inlineStr">
+        <is>
+          <t>Tracking</t>
+        </is>
+      </c>
+      <c r="D40" s="39" t="inlineStr">
+        <is>
+          <t>Responder marker moves smoothly along the road</t>
+        </is>
+      </c>
+      <c r="E40" s="39" t="inlineStr">
+        <is>
+          <t>Watch the tracking map during a drive</t>
+        </is>
+      </c>
+      <c r="F40" s="39" t="inlineStr">
+        <is>
+          <t>No backward jumps or U-turn loops; heading follows the road</t>
+        </is>
+      </c>
+      <c r="G40" s="38" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H40" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I40" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-17: frame analysis — no backward jumps or U-turn loops; remaining ~0.3 s marker blink about every 16 s on the emulator (route redraw)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="40" customHeight="1">
+      <c r="A41" s="41" t="inlineStr">
+        <is>
           <t>AI-01</t>
         </is>
       </c>
-      <c r="B36" s="46" t="inlineStr">
+      <c r="B41" s="46" t="inlineStr">
         <is>
           <t>Beyond SRS</t>
         </is>
       </c>
-      <c r="C36" s="43" t="inlineStr">
+      <c r="C41" s="43" t="inlineStr">
         <is>
           <t>AI</t>
         </is>
       </c>
-      <c r="D36" s="43" t="inlineStr">
+      <c r="D41" s="43" t="inlineStr">
         <is>
           <t>AI symptom check suggests the emergency type</t>
         </is>
       </c>
-      <c r="E36" s="43" t="inlineStr">
+      <c r="E41" s="43" t="inlineStr">
         <is>
           <t>Type symptoms on the emergency type screen and tap Suggest</t>
         </is>
       </c>
-      <c r="F36" s="43" t="inlineStr">
+      <c r="F41" s="43" t="inlineStr">
         <is>
           <t>Suggested type with confidence and reason; type preselected</t>
         </is>
       </c>
-      <c r="G36" s="42" t="inlineStr">
+      <c r="G41" s="42" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H36" s="45" t="inlineStr">
+      <c r="H41" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I36" s="43" t="inlineStr">
+      <c r="I41" s="43" t="inlineStr">
         <is>
           <t>2026-09-17: Gemini free tier (gemini-3.1-flash-lite) — "chest pain spreading to left arm" → Cardiac 98%, ~2 s</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="40" customHeight="1">
-      <c r="A37" s="37" t="inlineStr">
+    <row r="42" ht="40" customHeight="1">
+      <c r="A42" s="37" t="inlineStr">
         <is>
           <t>AI-02</t>
         </is>
       </c>
-      <c r="B37" s="44" t="inlineStr">
+      <c r="B42" s="44" t="inlineStr">
         <is>
           <t>Beyond SRS</t>
         </is>
       </c>
-      <c r="C37" s="39" t="inlineStr">
+      <c r="C42" s="39" t="inlineStr">
         <is>
           <t>AI</t>
         </is>
       </c>
-      <c r="D37" s="39" t="inlineStr">
+      <c r="D42" s="39" t="inlineStr">
         <is>
           <t>AI quick replies are personalised for a Deaf patient</t>
         </is>
       </c>
-      <c r="E37" s="39" t="inlineStr">
+      <c r="E42" s="39" t="inlineStr">
         <is>
           <t>Deaf patient opens Quick messages during an emergency</t>
         </is>
       </c>
-      <c r="F37" s="39" t="inlineStr">
+      <c r="F42" s="39" t="inlineStr">
         <is>
           <t>Suggestions reflect the medical profile</t>
         </is>
       </c>
-      <c r="G37" s="38" t="inlineStr">
+      <c r="G42" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H37" s="45" t="inlineStr">
+      <c r="H42" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I37" s="39" t="inlineStr">
+      <c r="I42" s="39" t="inlineStr">
         <is>
           <t>2026-09-17: quick replies personalised from medical profile (asthma, Salbutamol, Penicillin allergy)</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="36" t="inlineStr">
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  PAYMENTS (STRIPE SANDBOX)</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="40" customHeight="1">
-      <c r="A39" s="37" t="inlineStr">
+    <row r="44" ht="40" customHeight="1">
+      <c r="A44" s="37" t="inlineStr">
         <is>
           <t>PAY-01</t>
         </is>
       </c>
-      <c r="B39" s="44" t="inlineStr">
+      <c r="B44" s="44" t="inlineStr">
         <is>
           <t>Beyond SRS</t>
         </is>
       </c>
-      <c r="C39" s="39" t="inlineStr">
+      <c r="C44" s="39" t="inlineStr">
         <is>
           <t>Payments</t>
         </is>
       </c>
-      <c r="D39" s="39" t="inlineStr">
+      <c r="D44" s="39" t="inlineStr">
         <is>
           <t>Stripe card form opens quickly after tapping Pay</t>
         </is>
       </c>
-      <c r="E39" s="39" t="inlineStr">
+      <c r="E44" s="39" t="inlineStr">
         <is>
           <t>Open checkout for a paid plan, wait a moment, tap Pay</t>
         </is>
       </c>
-      <c r="F39" s="39" t="inlineStr">
+      <c r="F44" s="39" t="inlineStr">
         <is>
           <t>Card form ready within ~5 s on the emulator (no long spinner)</t>
         </is>
       </c>
-      <c r="G39" s="38" t="inlineStr">
+      <c r="G44" s="38" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H39" s="45" t="inlineStr">
+      <c r="H44" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I39" s="39" t="inlineStr">
+      <c r="I44" s="39" t="inlineStr">
         <is>
           <t>2026-09-18: emulator — Pay tap to card form ~4.8 s (was ~9.5 s: intent + sheet now prepared when checkout opens, FlowController)</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="40" customHeight="1">
-      <c r="A40" s="41" t="inlineStr">
+    <row r="45" ht="40" customHeight="1">
+      <c r="A45" s="41" t="inlineStr">
         <is>
           <t>PAY-02</t>
         </is>
       </c>
-      <c r="B40" s="46" t="inlineStr">
+      <c r="B45" s="46" t="inlineStr">
         <is>
           <t>Beyond SRS</t>
         </is>
       </c>
-      <c r="C40" s="43" t="inlineStr">
+      <c r="C45" s="43" t="inlineStr">
         <is>
           <t>Payments</t>
         </is>
       </c>
-      <c r="D40" s="43" t="inlineStr">
+      <c r="D45" s="43" t="inlineStr">
         <is>
           <t>Test card payment upgrades the plan</t>
         </is>
       </c>
-      <c r="E40" s="43" t="inlineStr">
+      <c r="E45" s="43" t="inlineStr">
         <is>
           <t>Pay with 4242 4242 4242 4242, any future date, any CVC</t>
         </is>
       </c>
-      <c r="F40" s="43" t="inlineStr">
+      <c r="F45" s="43" t="inlineStr">
         <is>
           <t>Payment successful screen with receipt; plan upgraded on the server</t>
         </is>
       </c>
-      <c r="G40" s="42" t="inlineStr">
+      <c r="G45" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="H40" s="45" t="inlineStr">
+      <c r="H45" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I40" s="43" t="inlineStr">
+      <c r="I45" s="43" t="inlineStr">
         <is>
           <t>2026-09-18: test card 4242 → "Payment successful" ~4.5 s after Continue; receipt shown; user plan FREE → PROFESSIONAL (demo reset after)</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="40" customHeight="1">
-      <c r="A41" s="37" t="inlineStr">
+    <row r="46" ht="40" customHeight="1">
+      <c r="A46" s="37" t="inlineStr">
         <is>
           <t>PAY-03</t>
         </is>
       </c>
-      <c r="B41" s="44" t="inlineStr">
+      <c r="B46" s="44" t="inlineStr">
         <is>
           <t>Beyond SRS</t>
         </is>
       </c>
-      <c r="C41" s="39" t="inlineStr">
+      <c r="C46" s="39" t="inlineStr">
         <is>
           <t>Payments</t>
         </is>
       </c>
-      <c r="D41" s="39" t="inlineStr">
+      <c r="D46" s="39" t="inlineStr">
         <is>
           <t>Cancelling the payment sheet does not charge</t>
         </is>
       </c>
-      <c r="E41" s="39" t="inlineStr">
+      <c r="E46" s="39" t="inlineStr">
         <is>
           <t>Open the sheet and close it</t>
         </is>
       </c>
-      <c r="F41" s="39" t="inlineStr">
+      <c r="F46" s="39" t="inlineStr">
         <is>
           <t>Message: payment cancelled, not charged; Pay works again</t>
         </is>
       </c>
-      <c r="G41" s="38" t="inlineStr">
+      <c r="G46" s="38" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H41" s="45" t="inlineStr">
+      <c r="H46" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I41" s="39" t="inlineStr">
+      <c r="I46" s="39" t="inlineStr">
         <is>
           <t>2026-09-18: closing the sheet shows "Payment cancelled. You have not been charged."; Pay again opens a fresh prepared sheet</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="36" t="inlineStr">
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  REGRESSION, RELEASE &amp; PERFORMANCE</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="40" customHeight="1">
-      <c r="A43" s="37" t="inlineStr">
+    <row r="48" ht="40" customHeight="1">
+      <c r="A48" s="37" t="inlineStr">
         <is>
           <t>REG-01</t>
         </is>
       </c>
-      <c r="B43" s="38" t="inlineStr">
+      <c r="B48" s="38" t="inlineStr">
         <is>
           <t>NFR</t>
         </is>
       </c>
-      <c r="C43" s="39" t="inlineStr">
+      <c r="C48" s="39" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
       </c>
-      <c r="D43" s="39" t="inlineStr">
+      <c r="D48" s="39" t="inlineStr">
         <is>
           <t>Automated suites pass after all changes</t>
         </is>
       </c>
-      <c r="E43" s="39" t="inlineStr">
+      <c r="E48" s="39" t="inlineStr">
         <is>
           <t>Run backend unit tests, type-check, privacy and call e2e, portal build, mobile analyzer</t>
         </is>
       </c>
-      <c r="F43" s="39" t="inlineStr">
+      <c r="F48" s="39" t="inlineStr">
         <is>
           <t>All green</t>
         </is>
       </c>
-      <c r="G43" s="38" t="inlineStr">
+      <c r="G48" s="38" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="H43" s="45" t="inlineStr">
+      <c r="H48" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I43" s="39" t="inlineStr">
+      <c r="I48" s="39" t="inlineStr">
         <is>
           <t>2026-09-18: re-check after laptop reboot — backend unit 94/94, tsc clean, privacy e2e 35/35, call signalling e2e 23/23, portal build OK, mobile analyzer 0 errors</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="40" customHeight="1">
-      <c r="A44" s="41" t="inlineStr">
+    <row r="49" ht="40" customHeight="1">
+      <c r="A49" s="41" t="inlineStr">
         <is>
           <t>REG-02</t>
         </is>
       </c>
-      <c r="B44" s="42" t="inlineStr">
+      <c r="B49" s="42" t="inlineStr">
         <is>
           <t>FR1</t>
         </is>
       </c>
-      <c r="C44" s="43" t="inlineStr">
+      <c r="C49" s="43" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
       </c>
-      <c r="D44" s="43" t="inlineStr">
+      <c r="D49" s="43" t="inlineStr">
         <is>
           <t>Full SOS cycle works end to end in the app</t>
         </is>
       </c>
-      <c r="E44" s="43" t="inlineStr">
+      <c r="E49" s="43" t="inlineStr">
         <is>
           <t>Patient sends SOS, responder accepts, call, resolve</t>
         </is>
       </c>
-      <c r="F44" s="43" t="inlineStr">
+      <c r="F49" s="43" t="inlineStr">
         <is>
           <t>Every step shown correctly; chat locked after resolve</t>
         </is>
       </c>
-      <c r="G44" s="42" t="inlineStr">
+      <c r="G49" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="H44" s="45" t="inlineStr">
+      <c r="H49" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I44" s="43" t="inlineStr">
+      <c r="I49" s="43" t="inlineStr">
         <is>
           <t>2026-09-18: app SOS on emulator → countdown → SOS active → responder assigned (ETA 1 min · 751 m, route) → in-app voice call connected (audio flowing) → resolved + rating screen → emergency chat locked</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="40" customHeight="1">
-      <c r="A45" s="37" t="inlineStr">
+    <row r="50" ht="40" customHeight="1">
+      <c r="A50" s="37" t="inlineStr">
         <is>
           <t>REG-03</t>
         </is>
       </c>
-      <c r="B45" s="38" t="inlineStr">
+      <c r="B50" s="38" t="inlineStr">
         <is>
           <t>NFR</t>
         </is>
       </c>
-      <c r="C45" s="39" t="inlineStr">
+      <c r="C50" s="39" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
       </c>
-      <c r="D45" s="39" t="inlineStr">
+      <c r="D50" s="39" t="inlineStr">
         <is>
           <t>Every role still opens and main screens load</t>
         </is>
       </c>
-      <c r="E45" s="39" t="inlineStr">
+      <c r="E50" s="39" t="inlineStr">
         <is>
           <t>Open responder, caregiver, Deaf patient and checkout</t>
         </is>
       </c>
-      <c r="F45" s="39" t="inlineStr">
+      <c r="F50" s="39" t="inlineStr">
         <is>
           <t>Screens load without errors</t>
         </is>
       </c>
-      <c r="G45" s="38" t="inlineStr">
+      <c r="G50" s="38" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H45" s="45" t="inlineStr">
+      <c r="H50" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I45" s="39" t="inlineStr">
+      <c r="I50" s="39" t="inlineStr">
         <is>
           <t>2026-09-18: responder, caregiver, Deaf patient home screens and checkout (sheet opens, cancel message) re-checked</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="40" customHeight="1">
-      <c r="A46" s="41" t="inlineStr">
+    <row r="51" ht="40" customHeight="1">
+      <c r="A51" s="41" t="inlineStr">
         <is>
           <t>PERF-04</t>
         </is>
       </c>
-      <c r="B46" s="42" t="inlineStr">
+      <c r="B51" s="42" t="inlineStr">
         <is>
           <t>FR8.4</t>
         </is>
       </c>
-      <c r="C46" s="43" t="inlineStr">
+      <c r="C51" s="43" t="inlineStr">
         <is>
           <t>Performance</t>
         </is>
       </c>
-      <c r="D46" s="43" t="inlineStr">
+      <c r="D51" s="43" t="inlineStr">
         <is>
           <t>App reopens quickly from the background</t>
         </is>
       </c>
-      <c r="E46" s="43" t="inlineStr">
+      <c r="E51" s="43" t="inlineStr">
         <is>
           <t>Put the app in background and open it again</t>
         </is>
       </c>
-      <c r="F46" s="43" t="inlineStr">
+      <c r="F51" s="43" t="inlineStr">
         <is>
           <t>Visible within 1 s</t>
         </is>
       </c>
-      <c r="G46" s="42" t="inlineStr">
+      <c r="G51" s="42" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H46" s="45" t="inlineStr">
+      <c r="H51" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I46" s="43" t="inlineStr">
+      <c r="I51" s="43" t="inlineStr">
         <is>
           <t>2026-09-18: warm start (app in background) 0.4–0.5 s</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="40" customHeight="1">
-      <c r="A47" s="37" t="inlineStr">
+    <row r="52" ht="40" customHeight="1">
+      <c r="A52" s="37" t="inlineStr">
         <is>
           <t>PERF-05</t>
         </is>
       </c>
-      <c r="B47" s="38" t="inlineStr">
+      <c r="B52" s="38" t="inlineStr">
         <is>
           <t>FR8.4</t>
         </is>
       </c>
-      <c r="C47" s="39" t="inlineStr">
+      <c r="C52" s="39" t="inlineStr">
         <is>
           <t>Performance</t>
         </is>
       </c>
-      <c r="D47" s="39" t="inlineStr">
+      <c r="D52" s="39" t="inlineStr">
         <is>
           <t>App cold start time</t>
         </is>
       </c>
-      <c r="E47" s="39" t="inlineStr">
+      <c r="E52" s="39" t="inlineStr">
         <is>
           <t>Force-stop the app and open it</t>
         </is>
       </c>
-      <c r="F47" s="39" t="inlineStr">
+      <c r="F52" s="39" t="inlineStr">
         <is>
           <t>Home screen within ~5 s on a normal phone</t>
         </is>
       </c>
-      <c r="G47" s="38" t="inlineStr">
+      <c r="G52" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H47" s="47" t="inlineStr">
+      <c r="H52" s="47" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="I47" s="39" t="inlineStr">
+      <c r="I52" s="39" t="inlineStr">
         <is>
           <t>2026-09-18: cold start 9.0–9.9 s on the emulator (profile build). Cause: app engine + background alert service engine start together. Stripe setup moved after first frame (no measurable change). To re-measure on a real phone</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="40" customHeight="1">
-      <c r="A48" s="41" t="inlineStr">
+    <row r="53" ht="40" customHeight="1">
+      <c r="A53" s="41" t="inlineStr">
         <is>
           <t>PERF-06</t>
         </is>
       </c>
-      <c r="B48" s="42" t="inlineStr">
+      <c r="B53" s="42" t="inlineStr">
         <is>
           <t>NFR</t>
         </is>
       </c>
-      <c r="C48" s="43" t="inlineStr">
+      <c r="C53" s="43" t="inlineStr">
         <is>
           <t>Performance</t>
         </is>
       </c>
-      <c r="D48" s="43" t="inlineStr">
+      <c r="D53" s="43" t="inlineStr">
         <is>
           <t>Backend starts quickly for development and production</t>
         </is>
       </c>
-      <c r="E48" s="43" t="inlineStr">
+      <c r="E53" s="43" t="inlineStr">
         <is>
           <t>Run npm run dev and npm start</t>
         </is>
       </c>
-      <c r="F48" s="43" t="inlineStr">
+      <c r="F53" s="43" t="inlineStr">
         <is>
           <t>Ready within ~10 s; npm start runs the current build</t>
         </is>
       </c>
-      <c r="G48" s="42" t="inlineStr">
+      <c r="G53" s="42" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H48" s="45" t="inlineStr">
+      <c r="H53" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I48" s="43" t="inlineStr">
+      <c r="I53" s="43" t="inlineStr">
         <is>
           <t>2026-09-18: backend dev start 29.5 s → 7.3 s (ts-node transpile-only); npm start 3.1 s and now runs the current build (was an April build)</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="40" customHeight="1">
-      <c r="A49" s="37" t="inlineStr">
+    <row r="54" ht="40" customHeight="1">
+      <c r="A54" s="37" t="inlineStr">
         <is>
           <t>REL-01</t>
         </is>
       </c>
-      <c r="B49" s="38" t="inlineStr">
+      <c r="B54" s="38" t="inlineStr">
         <is>
           <t>NFR</t>
         </is>
       </c>
-      <c r="C49" s="39" t="inlineStr">
+      <c r="C54" s="39" t="inlineStr">
         <is>
           <t>Release</t>
         </is>
       </c>
-      <c r="D49" s="39" t="inlineStr">
+      <c r="D54" s="39" t="inlineStr">
         <is>
           <t>Release APK builds</t>
         </is>
       </c>
-      <c r="E49" s="39" t="inlineStr">
+      <c r="E54" s="39" t="inlineStr">
         <is>
           <t>flutter build apk --release --split-per-abi</t>
         </is>
       </c>
-      <c r="F49" s="39" t="inlineStr">
+      <c r="F54" s="39" t="inlineStr">
         <is>
           <t>APKs produced without R8 errors</t>
         </is>
       </c>
-      <c r="G49" s="38" t="inlineStr">
+      <c r="G54" s="38" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H49" s="45" t="inlineStr">
+      <c r="H54" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I49" s="39" t="inlineStr">
+      <c r="I54" s="39" t="inlineStr">
         <is>
           <t>2026-09-18: release APK builds (was failing in R8 on Stripe push-provisioning classes; keep-rule added). arm64 APK 47 MB</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="40" customHeight="1">
-      <c r="A50" s="41" t="inlineStr">
+    <row r="55" ht="40" customHeight="1">
+      <c r="A55" s="41" t="inlineStr">
         <is>
           <t>REL-02</t>
         </is>
       </c>
-      <c r="B50" s="42" t="inlineStr">
+      <c r="B55" s="42" t="inlineStr">
         <is>
           <t>NFR</t>
         </is>
       </c>
-      <c r="C50" s="43" t="inlineStr">
+      <c r="C55" s="43" t="inlineStr">
         <is>
           <t>Release</t>
         </is>
       </c>
-      <c r="D50" s="43" t="inlineStr">
+      <c r="D55" s="43" t="inlineStr">
         <is>
           <t>Release APK runs</t>
         </is>
       </c>
-      <c r="E50" s="43" t="inlineStr">
+      <c r="E55" s="43" t="inlineStr">
         <is>
           <t>Install the release APK and open it</t>
         </is>
       </c>
-      <c r="F50" s="43" t="inlineStr">
+      <c r="F55" s="43" t="inlineStr">
         <is>
           <t>Login screen, no crash</t>
         </is>
       </c>
-      <c r="G50" s="42" t="inlineStr">
+      <c r="G55" s="42" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H50" s="45" t="inlineStr">
+      <c r="H55" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I50" s="43" t="inlineStr">
+      <c r="I55" s="43" t="inlineStr">
         <is>
           <t>2026-09-18: release x86_64 APK installed on emulator, launches to the login screen without crashes</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="40" customHeight="1">
-      <c r="A51" s="37" t="inlineStr">
+    <row r="56" ht="40" customHeight="1">
+      <c r="A56" s="37" t="inlineStr">
         <is>
           <t>REL-03</t>
         </is>
       </c>
-      <c r="B51" s="38" t="inlineStr">
+      <c r="B56" s="38" t="inlineStr">
         <is>
           <t>NFR</t>
         </is>
       </c>
-      <c r="C51" s="39" t="inlineStr">
+      <c r="C56" s="39" t="inlineStr">
         <is>
           <t>Release</t>
         </is>
       </c>
-      <c r="D51" s="39" t="inlineStr">
+      <c r="D56" s="39" t="inlineStr">
         <is>
           <t>Release APK works on a real phone over Wi-Fi</t>
         </is>
       </c>
-      <c r="E51" s="39" t="inlineStr">
+      <c r="E56" s="39" t="inlineStr">
         <is>
           <t>Phone on the same Wi-Fi as the laptop backend; log in and use SOS</t>
         </is>
       </c>
-      <c r="F51" s="39" t="inlineStr">
+      <c r="F56" s="39" t="inlineStr">
         <is>
           <t>App connects and works</t>
         </is>
       </c>
-      <c r="G51" s="38" t="inlineStr">
+      <c r="G56" s="38" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H51" s="40" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="I51" s="39" t="inlineStr">
-        <is>
-          <t>Phone APK built for http://192.168.100.5:3000 (backend answers on that IP); to be installed and logged in on the real phone</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="36" t="inlineStr">
+      <c r="H56" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I56" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-19: release APK (MediFind-2026-09-19-1515) installed on real phones, logged in and used over the tunnel backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  WEB PORTAL LANDING PAGE</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="50" customHeight="1">
-      <c r="A53" s="37" t="inlineStr">
+    <row r="58" ht="50" customHeight="1">
+      <c r="A58" s="37" t="inlineStr">
         <is>
           <t>WEB-01</t>
         </is>
       </c>
-      <c r="B53" s="44" t="inlineStr">
+      <c r="B58" s="44" t="inlineStr">
         <is>
           <t>Beyond SRS</t>
         </is>
       </c>
-      <c r="C53" s="39" t="inlineStr">
+      <c r="C58" s="39" t="inlineStr">
         <is>
           <t>Landing</t>
         </is>
       </c>
-      <c r="D53" s="39" t="inlineStr">
+      <c r="D58" s="39" t="inlineStr">
         <is>
           <t>Animated background matches the app’s purpose and keeps text readable</t>
         </is>
       </c>
-      <c r="E53" s="39" t="inlineStr">
+      <c r="E58" s="39" t="inlineStr">
         <is>
           <t>Open the landing page</t>
         </is>
       </c>
-      <c r="F53" s="39" t="inlineStr">
+      <c r="F58" s="39" t="inlineStr">
         <is>
           <t>Map/route/pulse/heartbeat effects; headline readable; off with reduced motion</t>
         </is>
       </c>
-      <c r="G53" s="38" t="inlineStr">
+      <c r="G58" s="38" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H53" s="45" t="inlineStr">
+      <c r="H58" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I53" s="39" t="inlineStr">
+      <c r="I58" s="39" t="inlineStr">
         <is>
           <t>2026-09-18: landing hero animated background (grid, routes, riding dots, pulse rings, ECG) faded behind the headline; section glows; trust band sweep</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="40" customHeight="1">
-      <c r="A54" s="41" t="inlineStr">
+    <row r="59" ht="40" customHeight="1">
+      <c r="A59" s="41" t="inlineStr">
         <is>
           <t>WEB-02</t>
         </is>
       </c>
-      <c r="B54" s="46" t="inlineStr">
+      <c r="B59" s="46" t="inlineStr">
         <is>
           <t>Beyond SRS</t>
         </is>
       </c>
-      <c r="C54" s="43" t="inlineStr">
+      <c r="C59" s="43" t="inlineStr">
         <is>
           <t>Landing</t>
         </is>
       </c>
-      <c r="D54" s="43" t="inlineStr">
+      <c r="D59" s="43" t="inlineStr">
         <is>
           <t>Interactive elements respond on hover</t>
         </is>
       </c>
-      <c r="E54" s="43" t="inlineStr">
+      <c r="E59" s="43" t="inlineStr">
         <is>
           <t>Hover cards, steps, FAQ, buttons, links</t>
         </is>
       </c>
-      <c r="F54" s="43" t="inlineStr">
+      <c r="F59" s="43" t="inlineStr">
         <is>
           <t>Visible hover state on each</t>
         </is>
       </c>
-      <c r="G54" s="42" t="inlineStr">
+      <c r="G59" s="42" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H54" s="45" t="inlineStr">
+      <c r="H59" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I54" s="43" t="inlineStr">
+      <c r="I59" s="43" t="inlineStr">
         <is>
           <t>2026-09-18: hover verified with mouse events — card lift + teal border, step slide, FAQ shadow, secondary button tint, trust card brighten</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="40" customHeight="1">
-      <c r="A55" s="37" t="inlineStr">
+    <row r="60" ht="40" customHeight="1">
+      <c r="A60" s="37" t="inlineStr">
         <is>
           <t>WEB-03</t>
         </is>
       </c>
-      <c r="B55" s="44" t="inlineStr">
+      <c r="B60" s="44" t="inlineStr">
         <is>
           <t>Beyond SRS</t>
         </is>
       </c>
-      <c r="C55" s="39" t="inlineStr">
+      <c r="C60" s="39" t="inlineStr">
         <is>
           <t>Landing</t>
         </is>
       </c>
-      <c r="D55" s="39" t="inlineStr">
+      <c r="D60" s="39" t="inlineStr">
         <is>
           <t>Icons match their headings</t>
         </is>
       </c>
-      <c r="E55" s="39" t="inlineStr">
+      <c r="E60" s="39" t="inlineStr">
         <is>
           <t>Review every icon with its heading</t>
         </is>
       </c>
-      <c r="F55" s="39" t="inlineStr">
+      <c r="F60" s="39" t="inlineStr">
         <is>
           <t>Each icon fits its topic</t>
         </is>
       </c>
-      <c r="G55" s="38" t="inlineStr">
+      <c r="G60" s="38" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H55" s="45" t="inlineStr">
+      <c r="H60" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I55" s="39" t="inlineStr">
+      <c r="I60" s="39" t="inlineStr">
         <is>
           <t>2026-09-18: icons match headings (EarOff for Deaf, Ambulance for responders, MicOff, LocateFixed, ClipboardPlus, ScrollText …)</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="40" customHeight="1">
-      <c r="A56" s="41" t="inlineStr">
+    <row r="61" ht="40" customHeight="1">
+      <c r="A61" s="41" t="inlineStr">
         <is>
           <t>WEB-04</t>
         </is>
       </c>
-      <c r="B56" s="46" t="inlineStr">
+      <c r="B61" s="46" t="inlineStr">
         <is>
           <t>Beyond SRS</t>
         </is>
       </c>
-      <c r="C56" s="43" t="inlineStr">
+      <c r="C61" s="43" t="inlineStr">
         <is>
           <t>Landing</t>
         </is>
       </c>
-      <c r="D56" s="43" t="inlineStr">
+      <c r="D61" s="43" t="inlineStr">
         <is>
           <t>Mockups use the real app look</t>
         </is>
       </c>
-      <c r="E56" s="43" t="inlineStr">
+      <c r="E61" s="43" t="inlineStr">
         <is>
           <t>View the tracking mockup</t>
         </is>
       </c>
-      <c r="F56" s="43" t="inlineStr">
+      <c r="F61" s="43" t="inlineStr">
         <is>
           <t>App mascot on the route; no filler captions</t>
         </is>
       </c>
-      <c r="G56" s="42" t="inlineStr">
+      <c r="G61" s="42" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H56" s="45" t="inlineStr">
+      <c r="H61" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I56" s="43" t="inlineStr">
+      <c r="I61" s="43" t="inlineStr">
         <is>
           <t>2026-09-18: tracking mockup uses the app mascot (turns along the route, siren flashes); "App preview" captions removed</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="40" customHeight="1">
-      <c r="A57" s="37" t="inlineStr">
+    <row r="62" ht="40" customHeight="1">
+      <c r="A62" s="37" t="inlineStr">
         <is>
           <t>WEB-05</t>
         </is>
       </c>
-      <c r="B57" s="44" t="inlineStr">
+      <c r="B62" s="44" t="inlineStr">
         <is>
           <t>Beyond SRS</t>
         </is>
       </c>
-      <c r="C57" s="39" t="inlineStr">
+      <c r="C62" s="39" t="inlineStr">
         <is>
           <t>Landing</t>
         </is>
       </c>
-      <c r="D57" s="39" t="inlineStr">
+      <c r="D62" s="39" t="inlineStr">
         <is>
           <t>Footer is organised and branded</t>
         </is>
       </c>
-      <c r="E57" s="39" t="inlineStr">
+      <c r="E62" s="39" t="inlineStr">
         <is>
           <t>View the footer</t>
         </is>
       </c>
-      <c r="F57" s="39" t="inlineStr">
+      <c r="F62" s="39" t="inlineStr">
         <is>
           <t>Header-style logo; grouped links; legal links at the bottom</t>
         </is>
       </c>
-      <c r="G57" s="38" t="inlineStr">
+      <c r="G62" s="38" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H57" s="45" t="inlineStr">
+      <c r="H62" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I57" s="39" t="inlineStr">
+      <c r="I62" s="39" t="inlineStr">
         <is>
           <t>2026-09-18: footer logo = header logo on white badge; links organised Product / Who it’s for / Support; legal links in bottom row</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="36" t="inlineStr">
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  ADMIN CONSOLE UPDATES</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="40" customHeight="1">
-      <c r="A59" s="37" t="inlineStr">
+    <row r="64" ht="40" customHeight="1">
+      <c r="A64" s="37" t="inlineStr">
         <is>
           <t>ADM-01</t>
         </is>
       </c>
-      <c r="B59" s="38" t="inlineStr">
+      <c r="B64" s="38" t="inlineStr">
         <is>
           <t>FR10</t>
         </is>
       </c>
-      <c r="C59" s="39" t="inlineStr">
+      <c r="C64" s="39" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D59" s="39" t="inlineStr">
+      <c r="D64" s="39" t="inlineStr">
         <is>
           <t>Branded admin sign-in page</t>
         </is>
       </c>
-      <c r="E59" s="39" t="inlineStr">
+      <c r="E64" s="39" t="inlineStr">
         <is>
           <t>Open /login on desktop and mobile</t>
         </is>
       </c>
-      <c r="F59" s="39" t="inlineStr">
+      <c r="F64" s="39" t="inlineStr">
         <is>
           <t>Brand panel + form; animations; works on mobile</t>
         </is>
       </c>
-      <c r="G59" s="38" t="inlineStr">
+      <c r="G64" s="38" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H59" s="45" t="inlineStr">
+      <c r="H64" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I59" s="39" t="inlineStr">
+      <c r="I64" s="39" t="inlineStr">
         <is>
           <t>2026-09-18: admin sign-in page split layout (brand panel + form), animated map backdrop on both sides, compact header on mobile; sign-in logic unchanged</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="40" customHeight="1">
-      <c r="A60" s="41" t="inlineStr">
+    <row r="65" ht="40" customHeight="1">
+      <c r="A65" s="41" t="inlineStr">
         <is>
           <t>ADM-02</t>
         </is>
       </c>
-      <c r="B60" s="42" t="inlineStr">
+      <c r="B65" s="42" t="inlineStr">
         <is>
           <t>FR10</t>
         </is>
       </c>
-      <c r="C60" s="43" t="inlineStr">
+      <c r="C65" s="43" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D60" s="43" t="inlineStr">
+      <c r="D65" s="43" t="inlineStr">
         <is>
           <t>Maps follow dark mode</t>
         </is>
       </c>
-      <c r="E60" s="43" t="inlineStr">
+      <c r="E65" s="43" t="inlineStr">
         <is>
           <t>Switch the admin theme to dark and open Overview and SOS Logistics</t>
         </is>
       </c>
-      <c r="F60" s="43" t="inlineStr">
+      <c r="F65" s="43" t="inlineStr">
         <is>
           <t>Dark map tiles, no watermark</t>
         </is>
       </c>
-      <c r="G60" s="42" t="inlineStr">
+      <c r="G65" s="42" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H60" s="45" t="inlineStr">
+      <c r="H65" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I60" s="43" t="inlineStr">
+      <c r="I65" s="43" t="inlineStr">
         <is>
           <t>2026-09-18: Overview and SOS Logistics maps use dark tiles in dark mode (filtered OSM, no API key) and light OSM in light mode</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="40" customHeight="1">
-      <c r="A61" s="37" t="inlineStr">
-        <is>
-          <t>ADM-03</t>
-        </is>
-      </c>
-      <c r="B61" s="38" t="inlineStr">
-        <is>
-          <t>FR10</t>
-        </is>
-      </c>
-      <c r="C61" s="39" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="D61" s="39" t="inlineStr">
-        <is>
-          <t>User details open in a centred dialog</t>
-        </is>
-      </c>
-      <c r="E61" s="39" t="inlineStr">
-        <is>
-          <t>Click a user in User Management</t>
-        </is>
-      </c>
-      <c r="F61" s="39" t="inlineStr">
-        <is>
-          <t>Centred dialog with full details</t>
-        </is>
-      </c>
-      <c r="G61" s="38" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H61" s="45" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="I61" s="39" t="inlineStr">
-        <is>
-          <t>2026-09-18: user details open as a centred dialog (light and dark), Escape/outside click close it</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="40" customHeight="1">
-      <c r="A62" s="41" t="inlineStr">
-        <is>
-          <t>ADM-04</t>
-        </is>
-      </c>
-      <c r="B62" s="42" t="inlineStr">
-        <is>
-          <t>FR10</t>
-        </is>
-      </c>
-      <c r="C62" s="43" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="D62" s="43" t="inlineStr">
-        <is>
-          <t>Header search only navigates to real matches</t>
-        </is>
-      </c>
-      <c r="E62" s="43" t="inlineStr">
-        <is>
-          <t>Type random text, a page keyword and a user name; press Enter</t>
-        </is>
-      </c>
-      <c r="F62" s="43" t="inlineStr">
-        <is>
-          <t>Random text stays with a no-match message; matches open</t>
-        </is>
-      </c>
-      <c r="G62" s="42" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H62" s="45" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="I62" s="43" t="inlineStr">
-        <is>
-          <t>2026-09-18: header search — random text shows "No pages or users match" and stays; "map" → SOS Logistics; "bilal" → user; ↑/↓ + Enter opens highlighted result</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="40" customHeight="1">
-      <c r="A63" s="37" t="inlineStr">
-        <is>
-          <t>ADM-05</t>
-        </is>
-      </c>
-      <c r="B63" s="38" t="inlineStr">
-        <is>
-          <t>NFR</t>
-        </is>
-      </c>
-      <c r="C63" s="39" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="D63" s="39" t="inlineStr">
-        <is>
-          <t>Unknown URLs show a 404 page</t>
-        </is>
-      </c>
-      <c r="E63" s="39" t="inlineStr">
-        <is>
-          <t>Open a wrong public URL and a wrong /admin URL</t>
-        </is>
-      </c>
-      <c r="F63" s="39" t="inlineStr">
-        <is>
-          <t>Branded 404 pages</t>
-        </is>
-      </c>
-      <c r="G63" s="38" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H63" s="45" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="I63" s="39" t="inlineStr">
-        <is>
-          <t>2026-09-18: wrong URLs show 404 — public /kuch-bhi-galat and admin /admin/galat-page</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="50" customHeight="1">
-      <c r="A64" s="41" t="inlineStr">
-        <is>
-          <t>CALL-12</t>
-        </is>
-      </c>
-      <c r="B64" s="46" t="inlineStr">
-        <is>
-          <t>Beyond SRS</t>
-        </is>
-      </c>
-      <c r="C64" s="43" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="D64" s="43" t="inlineStr">
-        <is>
-          <t>Admin can review emergency call records</t>
-        </is>
-      </c>
-      <c r="E64" s="43" t="inlineStr">
-        <is>
-          <t>Make responder ↔ patient/caregiver calls, open Communication &gt; Call Records</t>
-        </is>
-      </c>
-      <c r="F64" s="43" t="inlineStr">
-        <is>
-          <t>Each call listed with outcome and duration; family calls not shown; no audio stored</t>
-        </is>
-      </c>
-      <c r="G64" s="42" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H64" s="45" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="I64" s="43" t="inlineStr">
-        <is>
-          <t>2026-09-18: Call Records page lists responder ↔ patient/caregiver calls (4 test calls: 3 completed, 1 not connected) with duration, outcome, end reason and emergency; patient ↔ caregiver calls excluded; non-admin gets 401</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  LAYOUT &amp; ORIENTATION</t>
         </is>
       </c>
     </row>
     <row r="66" ht="40" customHeight="1">
       <c r="A66" s="37" t="inlineStr">
         <is>
-          <t>UX-01</t>
+          <t>ADM-03</t>
         </is>
       </c>
       <c r="B66" s="38" t="inlineStr">
         <is>
+          <t>FR10</t>
+        </is>
+      </c>
+      <c r="C66" s="39" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D66" s="39" t="inlineStr">
+        <is>
+          <t>User details open in a centred dialog</t>
+        </is>
+      </c>
+      <c r="E66" s="39" t="inlineStr">
+        <is>
+          <t>Click a user in User Management</t>
+        </is>
+      </c>
+      <c r="F66" s="39" t="inlineStr">
+        <is>
+          <t>Centred dialog with full details</t>
+        </is>
+      </c>
+      <c r="G66" s="38" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H66" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I66" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18: user details open as a centred dialog (light and dark), Escape/outside click close it</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="40" customHeight="1">
+      <c r="A67" s="41" t="inlineStr">
+        <is>
+          <t>ADM-04</t>
+        </is>
+      </c>
+      <c r="B67" s="42" t="inlineStr">
+        <is>
+          <t>FR10</t>
+        </is>
+      </c>
+      <c r="C67" s="43" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D67" s="43" t="inlineStr">
+        <is>
+          <t>Header search only navigates to real matches</t>
+        </is>
+      </c>
+      <c r="E67" s="43" t="inlineStr">
+        <is>
+          <t>Type random text, a page keyword and a user name; press Enter</t>
+        </is>
+      </c>
+      <c r="F67" s="43" t="inlineStr">
+        <is>
+          <t>Random text stays with a no-match message; matches open</t>
+        </is>
+      </c>
+      <c r="G67" s="42" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H67" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I67" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-18: header search — random text shows "No pages or users match" and stays; "map" → SOS Logistics; "bilal" → user; ↑/↓ + Enter opens highlighted result</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="40" customHeight="1">
+      <c r="A68" s="37" t="inlineStr">
+        <is>
+          <t>ADM-05</t>
+        </is>
+      </c>
+      <c r="B68" s="38" t="inlineStr">
+        <is>
           <t>NFR</t>
         </is>
       </c>
-      <c r="C66" s="39" t="inlineStr">
-        <is>
-          <t>Usability</t>
-        </is>
-      </c>
-      <c r="D66" s="39" t="inlineStr">
-        <is>
-          <t>App stays in portrait when the phone is rotated</t>
-        </is>
-      </c>
-      <c r="E66" s="39" t="inlineStr">
-        <is>
-          <t>Open the responder dashboard and rotate the phone</t>
-        </is>
-      </c>
-      <c r="F66" s="39" t="inlineStr">
-        <is>
-          <t>Screen stays portrait; nothing squeezed or cut off</t>
-        </is>
-      </c>
-      <c r="G66" s="38" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H66" s="45" t="inlineStr">
+      <c r="C68" s="39" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D68" s="39" t="inlineStr">
+        <is>
+          <t>Unknown URLs show a 404 page</t>
+        </is>
+      </c>
+      <c r="E68" s="39" t="inlineStr">
+        <is>
+          <t>Open a wrong public URL and a wrong /admin URL</t>
+        </is>
+      </c>
+      <c r="F68" s="39" t="inlineStr">
+        <is>
+          <t>Branded 404 pages</t>
+        </is>
+      </c>
+      <c r="G68" s="38" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H68" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I66" s="39" t="inlineStr">
-        <is>
-          <t>2026-09-18: responder app on emulator rotated to landscape stays portrait (before: dashboard squeezed into a strip)</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="50" customHeight="1">
-      <c r="A67" s="41" t="inlineStr">
-        <is>
-          <t>UX-02</t>
-        </is>
-      </c>
-      <c r="B67" s="42" t="inlineStr">
-        <is>
-          <t>NFR</t>
-        </is>
-      </c>
-      <c r="C67" s="43" t="inlineStr">
-        <is>
-          <t>Usability</t>
-        </is>
-      </c>
-      <c r="D67" s="43" t="inlineStr">
-        <is>
-          <t>On a tablet or wide screen the app is centred, not stretched or stuck to one side</t>
-        </is>
-      </c>
-      <c r="E67" s="43" t="inlineStr">
-        <is>
-          <t>Open the app on a tablet (or web/desktop)</t>
-        </is>
-      </c>
-      <c r="F67" s="43" t="inlineStr">
-        <is>
-          <t>App shown as a centred column with even margins</t>
-        </is>
-      </c>
-      <c r="G67" s="42" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H67" s="45" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="I67" s="43" t="inlineStr">
-        <is>
-          <t>2026-09-18: emulator resized to 1600x2560 tablet, portrait and landscape: centred 600dp column, no stretched or one-sided layout</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="50" customHeight="1">
-      <c r="A68" s="37" t="inlineStr">
-        <is>
-          <t>UX-04</t>
-        </is>
-      </c>
-      <c r="B68" s="44" t="inlineStr">
-        <is>
-          <t>Beyond SRS</t>
-        </is>
-      </c>
-      <c r="C68" s="39" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="D68" s="39" t="inlineStr">
-        <is>
-          <t>Checkout shows clear progress and a Stripe sheet in MediFind style</t>
-        </is>
-      </c>
-      <c r="E68" s="39" t="inlineStr">
-        <is>
-          <t>Tap Pay on checkout</t>
-        </is>
-      </c>
-      <c r="F68" s="39" t="inlineStr">
-        <is>
-          <t>Button says Opening secure payment…; sheet uses app colours and says Pay PKR …</t>
-        </is>
-      </c>
-      <c r="G68" s="38" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H68" s="45" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
       <c r="I68" s="39" t="inlineStr">
         <is>
-          <t>2026-09-18: Pay shows "Opening secure payment…" then "Confirming payment…"; Stripe sheet in app colours (light) with "Pay PKR 499" button</t>
+          <t>2026-09-18: wrong URLs show 404 — public /kuch-bhi-galat and admin /admin/galat-page</t>
         </is>
       </c>
     </row>
     <row r="69" ht="50" customHeight="1">
       <c r="A69" s="41" t="inlineStr">
         <is>
+          <t>CALL-12</t>
+        </is>
+      </c>
+      <c r="B69" s="46" t="inlineStr">
+        <is>
+          <t>Beyond SRS</t>
+        </is>
+      </c>
+      <c r="C69" s="43" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D69" s="43" t="inlineStr">
+        <is>
+          <t>Admin can review emergency call records</t>
+        </is>
+      </c>
+      <c r="E69" s="43" t="inlineStr">
+        <is>
+          <t>Make responder ↔ patient/caregiver calls, open Communication &gt; Call Records</t>
+        </is>
+      </c>
+      <c r="F69" s="43" t="inlineStr">
+        <is>
+          <t>Each call listed with outcome and duration; family calls not shown; no audio stored</t>
+        </is>
+      </c>
+      <c r="G69" s="42" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H69" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I69" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-18: Call Records page lists responder ↔ patient/caregiver calls (4 test calls: 3 completed, 1 not connected) with duration, outcome, end reason and emergency; patient ↔ caregiver calls excluded; non-admin gets 401</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="18" customHeight="1">
+      <c r="A70" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  LAYOUT &amp; ORIENTATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="40" customHeight="1">
+      <c r="A71" s="37" t="inlineStr">
+        <is>
+          <t>UX-01</t>
+        </is>
+      </c>
+      <c r="B71" s="38" t="inlineStr">
+        <is>
+          <t>NFR</t>
+        </is>
+      </c>
+      <c r="C71" s="39" t="inlineStr">
+        <is>
+          <t>Usability</t>
+        </is>
+      </c>
+      <c r="D71" s="39" t="inlineStr">
+        <is>
+          <t>App stays in portrait when the phone is rotated</t>
+        </is>
+      </c>
+      <c r="E71" s="39" t="inlineStr">
+        <is>
+          <t>Open the responder dashboard and rotate the phone</t>
+        </is>
+      </c>
+      <c r="F71" s="39" t="inlineStr">
+        <is>
+          <t>Screen stays portrait; nothing squeezed or cut off</t>
+        </is>
+      </c>
+      <c r="G71" s="38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H71" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I71" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18: responder app on emulator rotated to landscape stays portrait (before: dashboard squeezed into a strip)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="50" customHeight="1">
+      <c r="A72" s="41" t="inlineStr">
+        <is>
+          <t>UX-02</t>
+        </is>
+      </c>
+      <c r="B72" s="42" t="inlineStr">
+        <is>
+          <t>NFR</t>
+        </is>
+      </c>
+      <c r="C72" s="43" t="inlineStr">
+        <is>
+          <t>Usability</t>
+        </is>
+      </c>
+      <c r="D72" s="43" t="inlineStr">
+        <is>
+          <t>On a tablet or wide screen the app is centred, not stretched or stuck to one side</t>
+        </is>
+      </c>
+      <c r="E72" s="43" t="inlineStr">
+        <is>
+          <t>Open the app on a tablet (or web/desktop)</t>
+        </is>
+      </c>
+      <c r="F72" s="43" t="inlineStr">
+        <is>
+          <t>App shown as a centred column with even margins</t>
+        </is>
+      </c>
+      <c r="G72" s="42" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H72" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I72" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-18: emulator resized to 1600x2560 tablet, portrait and landscape: centred 600dp column, no stretched or one-sided layout</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="50" customHeight="1">
+      <c r="A73" s="37" t="inlineStr">
+        <is>
+          <t>UX-04</t>
+        </is>
+      </c>
+      <c r="B73" s="44" t="inlineStr">
+        <is>
+          <t>Beyond SRS</t>
+        </is>
+      </c>
+      <c r="C73" s="39" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="D73" s="39" t="inlineStr">
+        <is>
+          <t>Checkout shows clear progress and a Stripe sheet in MediFind style</t>
+        </is>
+      </c>
+      <c r="E73" s="39" t="inlineStr">
+        <is>
+          <t>Tap Pay on checkout</t>
+        </is>
+      </c>
+      <c r="F73" s="39" t="inlineStr">
+        <is>
+          <t>Button says Opening secure payment…; sheet uses app colours and says Pay PKR …</t>
+        </is>
+      </c>
+      <c r="G73" s="38" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H73" s="45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I73" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18: Pay shows "Opening secure payment…" then "Confirming payment…"; Stripe sheet in app colours (light) with "Pay PKR 499" button</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="50" customHeight="1">
+      <c r="A74" s="41" t="inlineStr">
+        <is>
           <t>UX-05</t>
         </is>
       </c>
-      <c r="B69" s="42" t="inlineStr">
+      <c r="B74" s="42" t="inlineStr">
         <is>
           <t>FR6.2</t>
         </is>
       </c>
-      <c r="C69" s="43" t="inlineStr">
+      <c r="C74" s="43" t="inlineStr">
         <is>
           <t>Tracking</t>
         </is>
       </c>
-      <c r="D69" s="43" t="inlineStr">
+      <c r="D74" s="43" t="inlineStr">
         <is>
           <t>Unrealistic GPS distance is not shown as an ETA</t>
         </is>
       </c>
-      <c r="E69" s="43" t="inlineStr">
+      <c r="E74" s="43" t="inlineStr">
         <is>
           <t>Responder phone reports a location hundreds of km away</t>
         </is>
       </c>
-      <c r="F69" s="43" t="inlineStr">
+      <c r="F74" s="43" t="inlineStr">
         <is>
           <t>Shows Locating / Waiting for GPS; no route line; map stays on the patient</t>
         </is>
       </c>
-      <c r="G69" s="42" t="inlineStr">
+      <c r="G74" s="42" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H69" s="45" t="inlineStr">
+      <c r="H74" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I69" s="43" t="inlineStr">
+      <c r="I74" s="43" t="inlineStr">
         <is>
           <t>2026-09-18: responder GPS set to California: "Locating you / Waiting for GPS", no route line, camera on patient (was "17913 min, 11941 km"); back to Lahore: marker placed directly, "2 min · 1.3 km", normal zoom</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="40" customHeight="1">
-      <c r="A70" s="37" t="inlineStr">
+    <row r="75" ht="40" customHeight="1">
+      <c r="A75" s="37" t="inlineStr">
         <is>
           <t>UX-06</t>
         </is>
       </c>
-      <c r="B70" s="38" t="inlineStr">
+      <c r="B75" s="38" t="inlineStr">
         <is>
           <t>NFR</t>
         </is>
       </c>
-      <c r="C70" s="39" t="inlineStr">
+      <c r="C75" s="39" t="inlineStr">
         <is>
           <t>Usability</t>
         </is>
       </c>
-      <c r="D70" s="39" t="inlineStr">
+      <c r="D75" s="39" t="inlineStr">
         <is>
           <t>Maps show a loading state instead of a blank box</t>
         </is>
       </c>
-      <c r="E70" s="39" t="inlineStr">
+      <c r="E75" s="39" t="inlineStr">
         <is>
           <t>Open a tracking screen</t>
         </is>
       </c>
-      <c r="F70" s="39" t="inlineStr">
+      <c r="F75" s="39" t="inlineStr">
         <is>
           <t>Loading map… until the map appears</t>
         </is>
       </c>
-      <c r="G70" s="38" t="inlineStr">
+      <c r="G75" s="38" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H70" s="45" t="inlineStr">
+      <c r="H75" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I70" s="39" t="inlineStr">
+      <c r="I75" s="39" t="inlineStr">
         <is>
           <t>2026-09-18: responder / patient / caregiver tracking maps show "Loading map…" until the map is ready (was a blank grey box)</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="40" customHeight="1">
-      <c r="A71" s="41" t="inlineStr">
+    <row r="76" ht="40" customHeight="1">
+      <c r="A76" s="41" t="inlineStr">
         <is>
           <t>UX-07</t>
         </is>
       </c>
-      <c r="B71" s="42" t="inlineStr">
+      <c r="B76" s="42" t="inlineStr">
         <is>
           <t>FR3.1</t>
         </is>
       </c>
-      <c r="C71" s="43" t="inlineStr">
+      <c r="C76" s="43" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D71" s="43" t="inlineStr">
+      <c r="D76" s="43" t="inlineStr">
         <is>
           <t>Deaf quick phrases are fully readable on the home screen</t>
         </is>
       </c>
-      <c r="E71" s="43" t="inlineStr">
+      <c r="E76" s="43" t="inlineStr">
         <is>
           <t>Open the Deaf patient home screen</t>
         </is>
       </c>
-      <c r="F71" s="43" t="inlineStr">
+      <c r="F76" s="43" t="inlineStr">
         <is>
           <t>Each phrase shown in full, wrapping onto lines</t>
         </is>
       </c>
-      <c r="G71" s="42" t="inlineStr">
+      <c r="G76" s="42" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H71" s="45" t="inlineStr">
+      <c r="H76" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I71" s="43" t="inlineStr">
+      <c r="I76" s="43" t="inlineStr">
         <is>
           <t>2026-09-18: Deaf home quick phrases wrap onto lines and are fully readable (was cut off "I am de…")</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="40" customHeight="1">
-      <c r="A72" s="37" t="inlineStr">
+    <row r="77" ht="40" customHeight="1">
+      <c r="A77" s="37" t="inlineStr">
         <is>
           <t>UX-03</t>
         </is>
       </c>
-      <c r="B72" s="38" t="inlineStr">
+      <c r="B77" s="38" t="inlineStr">
         <is>
           <t>NFR</t>
         </is>
       </c>
-      <c r="C72" s="39" t="inlineStr">
+      <c r="C77" s="39" t="inlineStr">
         <is>
           <t>Branding</t>
         </is>
       </c>
-      <c r="D72" s="39" t="inlineStr">
+      <c r="D77" s="39" t="inlineStr">
         <is>
           <t>The same MediFind logo is used in the mobile app and the web portal</t>
         </is>
       </c>
-      <c r="E72" s="39" t="inlineStr">
+      <c r="E77" s="39" t="inlineStr">
         <is>
           <t>Compare app launcher, splash, headers with portal sidebar, login, landing, 404, legal, favicon</t>
         </is>
       </c>
-      <c r="F72" s="39" t="inlineStr">
+      <c r="F77" s="39" t="inlineStr">
         <is>
           <t>One consistent logo everywhere</t>
         </is>
       </c>
-      <c r="G72" s="38" t="inlineStr">
+      <c r="G77" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H72" s="45" t="inlineStr">
+      <c r="H77" s="45" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I72" s="39" t="inlineStr">
+      <c r="I77" s="39" t="inlineStr">
         <is>
           <t>2026-09-18: portal sidebar, login, landing, 404, legal and favicon use the same pin-with-rings logo as the mobile app</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="A15:I15"/>
-    <mergeCell ref="A52:I52"/>
-    <mergeCell ref="A65:I65"/>
+    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="A57:I57"/>
     <mergeCell ref="A11:I11"/>
-    <mergeCell ref="A42:I42"/>
+    <mergeCell ref="A63:I63"/>
+    <mergeCell ref="A47:I47"/>
+    <mergeCell ref="A37:I37"/>
     <mergeCell ref="A32:I32"/>
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A70:I70"/>
     <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A58:I58"/>
     <mergeCell ref="A20:I20"/>
-    <mergeCell ref="A38:I38"/>
   </mergeCells>
-  <conditionalFormatting sqref="H4:H72">
+  <conditionalFormatting sqref="H4:H77">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -4766,7 +4962,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H4:H72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid status" error="Choose PASS, FAIL, PENDING, BLOCKED or N/A" type="list">
+    <dataValidation sqref="H4:H77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid status" error="Choose PASS, FAIL, PENDING, BLOCKED or N/A" type="list">
       <formula1>"PENDING,PASS,FAIL,BLOCKED,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8477,7 +8673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D175"/>
+  <dimension ref="A1:D179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10564,7 +10760,7 @@
     <row r="96">
       <c r="A96" s="49" t="inlineStr">
         <is>
-          <t>PERF-01</t>
+          <t>CALL-13</t>
         </is>
       </c>
       <c r="B96" s="49" t="inlineStr">
@@ -10574,19 +10770,19 @@
       </c>
       <c r="C96" s="49" t="inlineStr">
         <is>
-          <t>SOS countdown opens immediately after Send SOS</t>
+          <t>Voice call on real phones is clear</t>
         </is>
       </c>
       <c r="D96" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS FR8.4</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="49" t="inlineStr">
         <is>
-          <t>PERF-02</t>
+          <t>CALL-14</t>
         </is>
       </c>
       <c r="B97" s="49" t="inlineStr">
@@ -10596,19 +10792,19 @@
       </c>
       <c r="C97" s="49" t="inlineStr">
         <is>
-          <t>Responder reaches navigation right after accepting</t>
+          <t>Video call on real phones is clear</t>
         </is>
       </c>
       <c r="D97" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS FR8.4</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="49" t="inlineStr">
         <is>
-          <t>PERF-03</t>
+          <t>MSG-01</t>
         </is>
       </c>
       <c r="B98" s="49" t="inlineStr">
@@ -10618,19 +10814,19 @@
       </c>
       <c r="C98" s="49" t="inlineStr">
         <is>
-          <t>Responder marker moves smoothly along the road</t>
+          <t>Voice note is sent and plays</t>
         </is>
       </c>
       <c r="D98" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS FR6.2</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR7.3</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="49" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>MSG-02</t>
         </is>
       </c>
       <c r="B99" s="49" t="inlineStr">
@@ -10640,19 +10836,19 @@
       </c>
       <c r="C99" s="49" t="inlineStr">
         <is>
-          <t>AI symptom check suggests the emergency type</t>
+          <t>Text chat works between real phones</t>
         </is>
       </c>
       <c r="D99" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR7.3</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="49" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>PERF-01</t>
         </is>
       </c>
       <c r="B100" s="49" t="inlineStr">
@@ -10662,19 +10858,19 @@
       </c>
       <c r="C100" s="49" t="inlineStr">
         <is>
-          <t>AI quick replies are personalised for a Deaf patient</t>
+          <t>SOS countdown opens immediately after Send SOS</t>
         </is>
       </c>
       <c r="D100" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR8.4</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="49" t="inlineStr">
         <is>
-          <t>PAY-01</t>
+          <t>PERF-02</t>
         </is>
       </c>
       <c r="B101" s="49" t="inlineStr">
@@ -10684,19 +10880,19 @@
       </c>
       <c r="C101" s="49" t="inlineStr">
         <is>
-          <t>Stripe card form opens quickly after tapping Pay</t>
+          <t>Responder reaches navigation right after accepting</t>
         </is>
       </c>
       <c r="D101" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR8.4</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="49" t="inlineStr">
         <is>
-          <t>PAY-02</t>
+          <t>PERF-03</t>
         </is>
       </c>
       <c r="B102" s="49" t="inlineStr">
@@ -10706,19 +10902,19 @@
       </c>
       <c r="C102" s="49" t="inlineStr">
         <is>
-          <t>Test card payment upgrades the plan</t>
+          <t>Responder marker moves smoothly along the road</t>
         </is>
       </c>
       <c r="D102" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR6.2</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="49" t="inlineStr">
         <is>
-          <t>PAY-03</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B103" s="49" t="inlineStr">
@@ -10728,7 +10924,7 @@
       </c>
       <c r="C103" s="49" t="inlineStr">
         <is>
-          <t>Cancelling the payment sheet does not charge</t>
+          <t>AI symptom check suggests the emergency type</t>
         </is>
       </c>
       <c r="D103" s="49" t="inlineStr">
@@ -10740,7 +10936,7 @@
     <row r="104">
       <c r="A104" s="49" t="inlineStr">
         <is>
-          <t>REG-01</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B104" s="49" t="inlineStr">
@@ -10750,19 +10946,19 @@
       </c>
       <c r="C104" s="49" t="inlineStr">
         <is>
-          <t>Automated suites pass after all changes</t>
+          <t>AI quick replies are personalised for a Deaf patient</t>
         </is>
       </c>
       <c r="D104" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="49" t="inlineStr">
         <is>
-          <t>REG-02</t>
+          <t>PAY-01</t>
         </is>
       </c>
       <c r="B105" s="49" t="inlineStr">
@@ -10772,19 +10968,19 @@
       </c>
       <c r="C105" s="49" t="inlineStr">
         <is>
-          <t>Full SOS cycle works end to end in the app</t>
+          <t>Stripe card form opens quickly after tapping Pay</t>
         </is>
       </c>
       <c r="D105" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS FR1</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="49" t="inlineStr">
         <is>
-          <t>REG-03</t>
+          <t>PAY-02</t>
         </is>
       </c>
       <c r="B106" s="49" t="inlineStr">
@@ -10794,19 +10990,19 @@
       </c>
       <c r="C106" s="49" t="inlineStr">
         <is>
-          <t>Every role still opens and main screens load</t>
+          <t>Test card payment upgrades the plan</t>
         </is>
       </c>
       <c r="D106" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="49" t="inlineStr">
         <is>
-          <t>PERF-04</t>
+          <t>PAY-03</t>
         </is>
       </c>
       <c r="B107" s="49" t="inlineStr">
@@ -10816,19 +11012,19 @@
       </c>
       <c r="C107" s="49" t="inlineStr">
         <is>
-          <t>App reopens quickly from the background</t>
+          <t>Cancelling the payment sheet does not charge</t>
         </is>
       </c>
       <c r="D107" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS FR8.4</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="49" t="inlineStr">
         <is>
-          <t>PERF-05</t>
+          <t>REG-01</t>
         </is>
       </c>
       <c r="B108" s="49" t="inlineStr">
@@ -10838,19 +11034,19 @@
       </c>
       <c r="C108" s="49" t="inlineStr">
         <is>
-          <t>App cold start time</t>
+          <t>Automated suites pass after all changes</t>
         </is>
       </c>
       <c r="D108" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS FR8.4</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="49" t="inlineStr">
         <is>
-          <t>PERF-06</t>
+          <t>REG-02</t>
         </is>
       </c>
       <c r="B109" s="49" t="inlineStr">
@@ -10860,19 +11056,19 @@
       </c>
       <c r="C109" s="49" t="inlineStr">
         <is>
-          <t>Backend starts quickly for development and production</t>
+          <t>Full SOS cycle works end to end in the app</t>
         </is>
       </c>
       <c r="D109" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR1</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="49" t="inlineStr">
         <is>
-          <t>REL-01</t>
+          <t>REG-03</t>
         </is>
       </c>
       <c r="B110" s="49" t="inlineStr">
@@ -10882,7 +11078,7 @@
       </c>
       <c r="C110" s="49" t="inlineStr">
         <is>
-          <t>Release APK builds</t>
+          <t>Every role still opens and main screens load</t>
         </is>
       </c>
       <c r="D110" s="49" t="inlineStr">
@@ -10894,7 +11090,7 @@
     <row r="111">
       <c r="A111" s="49" t="inlineStr">
         <is>
-          <t>REL-02</t>
+          <t>PERF-04</t>
         </is>
       </c>
       <c r="B111" s="49" t="inlineStr">
@@ -10904,19 +11100,19 @@
       </c>
       <c r="C111" s="49" t="inlineStr">
         <is>
-          <t>Release APK runs</t>
+          <t>App reopens quickly from the background</t>
         </is>
       </c>
       <c r="D111" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR8.4</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="49" t="inlineStr">
         <is>
-          <t>REL-03</t>
+          <t>PERF-05</t>
         </is>
       </c>
       <c r="B112" s="49" t="inlineStr">
@@ -10926,19 +11122,19 @@
       </c>
       <c r="C112" s="49" t="inlineStr">
         <is>
-          <t>Release APK works on a real phone over Wi-Fi</t>
+          <t>App cold start time</t>
         </is>
       </c>
       <c r="D112" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR8.4</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="49" t="inlineStr">
         <is>
-          <t>WEB-01</t>
+          <t>PERF-06</t>
         </is>
       </c>
       <c r="B113" s="49" t="inlineStr">
@@ -10948,19 +11144,19 @@
       </c>
       <c r="C113" s="49" t="inlineStr">
         <is>
-          <t>Animated background matches the app’s purpose and keeps text readable</t>
+          <t>Backend starts quickly for development and production</t>
         </is>
       </c>
       <c r="D113" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="49" t="inlineStr">
         <is>
-          <t>WEB-02</t>
+          <t>REL-01</t>
         </is>
       </c>
       <c r="B114" s="49" t="inlineStr">
@@ -10970,19 +11166,19 @@
       </c>
       <c r="C114" s="49" t="inlineStr">
         <is>
-          <t>Interactive elements respond on hover</t>
+          <t>Release APK builds</t>
         </is>
       </c>
       <c r="D114" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="49" t="inlineStr">
         <is>
-          <t>WEB-03</t>
+          <t>REL-02</t>
         </is>
       </c>
       <c r="B115" s="49" t="inlineStr">
@@ -10992,19 +11188,19 @@
       </c>
       <c r="C115" s="49" t="inlineStr">
         <is>
-          <t>Icons match their headings</t>
+          <t>Release APK runs</t>
         </is>
       </c>
       <c r="D115" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="49" t="inlineStr">
         <is>
-          <t>WEB-04</t>
+          <t>REL-03</t>
         </is>
       </c>
       <c r="B116" s="49" t="inlineStr">
@@ -11014,19 +11210,19 @@
       </c>
       <c r="C116" s="49" t="inlineStr">
         <is>
-          <t>Mockups use the real app look</t>
+          <t>Release APK works on a real phone over Wi-Fi</t>
         </is>
       </c>
       <c r="D116" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="49" t="inlineStr">
         <is>
-          <t>WEB-05</t>
+          <t>WEB-01</t>
         </is>
       </c>
       <c r="B117" s="49" t="inlineStr">
@@ -11036,7 +11232,7 @@
       </c>
       <c r="C117" s="49" t="inlineStr">
         <is>
-          <t>Footer is organised and branded</t>
+          <t>Animated background matches the app’s purpose and keeps text readable</t>
         </is>
       </c>
       <c r="D117" s="49" t="inlineStr">
@@ -11048,7 +11244,7 @@
     <row r="118">
       <c r="A118" s="49" t="inlineStr">
         <is>
-          <t>ADM-01</t>
+          <t>WEB-02</t>
         </is>
       </c>
       <c r="B118" s="49" t="inlineStr">
@@ -11058,19 +11254,19 @@
       </c>
       <c r="C118" s="49" t="inlineStr">
         <is>
-          <t>Branded admin sign-in page</t>
+          <t>Interactive elements respond on hover</t>
         </is>
       </c>
       <c r="D118" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS FR10</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="49" t="inlineStr">
         <is>
-          <t>ADM-02</t>
+          <t>WEB-03</t>
         </is>
       </c>
       <c r="B119" s="49" t="inlineStr">
@@ -11080,19 +11276,19 @@
       </c>
       <c r="C119" s="49" t="inlineStr">
         <is>
-          <t>Maps follow dark mode</t>
+          <t>Icons match their headings</t>
         </is>
       </c>
       <c r="D119" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS FR10</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="49" t="inlineStr">
         <is>
-          <t>ADM-03</t>
+          <t>WEB-04</t>
         </is>
       </c>
       <c r="B120" s="49" t="inlineStr">
@@ -11102,19 +11298,19 @@
       </c>
       <c r="C120" s="49" t="inlineStr">
         <is>
-          <t>User details open in a centred dialog</t>
+          <t>Mockups use the real app look</t>
         </is>
       </c>
       <c r="D120" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS FR10</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="49" t="inlineStr">
         <is>
-          <t>ADM-04</t>
+          <t>WEB-05</t>
         </is>
       </c>
       <c r="B121" s="49" t="inlineStr">
@@ -11124,19 +11320,19 @@
       </c>
       <c r="C121" s="49" t="inlineStr">
         <is>
-          <t>Header search only navigates to real matches</t>
+          <t>Footer is organised and branded</t>
         </is>
       </c>
       <c r="D121" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS FR10</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="49" t="inlineStr">
         <is>
-          <t>ADM-05</t>
+          <t>ADM-01</t>
         </is>
       </c>
       <c r="B122" s="49" t="inlineStr">
@@ -11146,19 +11342,19 @@
       </c>
       <c r="C122" s="49" t="inlineStr">
         <is>
-          <t>Unknown URLs show a 404 page</t>
+          <t>Branded admin sign-in page</t>
         </is>
       </c>
       <c r="D122" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR10</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="49" t="inlineStr">
         <is>
-          <t>CALL-12</t>
+          <t>ADM-02</t>
         </is>
       </c>
       <c r="B123" s="49" t="inlineStr">
@@ -11168,19 +11364,19 @@
       </c>
       <c r="C123" s="49" t="inlineStr">
         <is>
-          <t>Admin can review emergency call records</t>
+          <t>Maps follow dark mode</t>
         </is>
       </c>
       <c r="D123" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR10</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="49" t="inlineStr">
         <is>
-          <t>UX-01</t>
+          <t>ADM-03</t>
         </is>
       </c>
       <c r="B124" s="49" t="inlineStr">
@@ -11190,19 +11386,19 @@
       </c>
       <c r="C124" s="49" t="inlineStr">
         <is>
-          <t>App stays in portrait when the phone is rotated</t>
+          <t>User details open in a centred dialog</t>
         </is>
       </c>
       <c r="D124" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR10</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="49" t="inlineStr">
         <is>
-          <t>UX-02</t>
+          <t>ADM-04</t>
         </is>
       </c>
       <c r="B125" s="49" t="inlineStr">
@@ -11212,19 +11408,19 @@
       </c>
       <c r="C125" s="49" t="inlineStr">
         <is>
-          <t>On a tablet or wide screen the app is centred, not stretched or stuck to one side</t>
+          <t>Header search only navigates to real matches</t>
         </is>
       </c>
       <c r="D125" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR10</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="49" t="inlineStr">
         <is>
-          <t>UX-04</t>
+          <t>ADM-05</t>
         </is>
       </c>
       <c r="B126" s="49" t="inlineStr">
@@ -11234,19 +11430,19 @@
       </c>
       <c r="C126" s="49" t="inlineStr">
         <is>
-          <t>Checkout shows clear progress and a Stripe sheet in MediFind style</t>
+          <t>Unknown URLs show a 404 page</t>
         </is>
       </c>
       <c r="D126" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="49" t="inlineStr">
         <is>
-          <t>UX-05</t>
+          <t>CALL-12</t>
         </is>
       </c>
       <c r="B127" s="49" t="inlineStr">
@@ -11256,19 +11452,19 @@
       </c>
       <c r="C127" s="49" t="inlineStr">
         <is>
-          <t>Unrealistic GPS distance is not shown as an ETA</t>
+          <t>Admin can review emergency call records</t>
         </is>
       </c>
       <c r="D127" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS FR6.2</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="49" t="inlineStr">
         <is>
-          <t>UX-06</t>
+          <t>UX-01</t>
         </is>
       </c>
       <c r="B128" s="49" t="inlineStr">
@@ -11278,7 +11474,7 @@
       </c>
       <c r="C128" s="49" t="inlineStr">
         <is>
-          <t>Maps show a loading state instead of a blank box</t>
+          <t>App stays in portrait when the phone is rotated</t>
         </is>
       </c>
       <c r="D128" s="49" t="inlineStr">
@@ -11290,7 +11486,7 @@
     <row r="129">
       <c r="A129" s="49" t="inlineStr">
         <is>
-          <t>UX-07</t>
+          <t>UX-02</t>
         </is>
       </c>
       <c r="B129" s="49" t="inlineStr">
@@ -11300,19 +11496,19 @@
       </c>
       <c r="C129" s="49" t="inlineStr">
         <is>
-          <t>Deaf quick phrases are fully readable on the home screen</t>
+          <t>On a tablet or wide screen the app is centred, not stretched or stuck to one side</t>
         </is>
       </c>
       <c r="D129" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS FR3.1</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="49" t="inlineStr">
         <is>
-          <t>UX-03</t>
+          <t>UX-04</t>
         </is>
       </c>
       <c r="B130" s="49" t="inlineStr">
@@ -11322,19 +11518,19 @@
       </c>
       <c r="C130" s="49" t="inlineStr">
         <is>
-          <t>The same MediFind logo is used in the mobile app and the web portal</t>
+          <t>Checkout shows clear progress and a Stripe sheet in MediFind style</t>
         </is>
       </c>
       <c r="D130" s="49" t="inlineStr">
         <is>
-          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
+          <t>New sheet PRIVACY_CALLS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="49" t="inlineStr">
         <is>
-          <t>MED-01</t>
+          <t>UX-05</t>
         </is>
       </c>
       <c r="B131" s="49" t="inlineStr">
@@ -11344,19 +11540,19 @@
       </c>
       <c r="C131" s="49" t="inlineStr">
         <is>
-          <t>Patient creates and edits the medical profile</t>
+          <t>Unrealistic GPS distance is not shown as an ETA</t>
         </is>
       </c>
       <c r="D131" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.1, FR2.2</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR6.2</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="49" t="inlineStr">
         <is>
-          <t>MED-02</t>
+          <t>UX-06</t>
         </is>
       </c>
       <c r="B132" s="49" t="inlineStr">
@@ -11366,19 +11562,19 @@
       </c>
       <c r="C132" s="49" t="inlineStr">
         <is>
-          <t>Saving the medical profile keeps emergency contacts and quick phrases</t>
+          <t>Maps show a loading state instead of a blank box</t>
         </is>
       </c>
       <c r="D132" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.1</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="49" t="inlineStr">
         <is>
-          <t>MED-03</t>
+          <t>UX-07</t>
         </is>
       </c>
       <c r="B133" s="49" t="inlineStr">
@@ -11388,19 +11584,19 @@
       </c>
       <c r="C133" s="49" t="inlineStr">
         <is>
-          <t>Patient adds, calls and deletes emergency contacts</t>
+          <t>Deaf quick phrases are fully readable on the home screen</t>
         </is>
       </c>
       <c r="D133" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.1</t>
+          <t>New sheet PRIVACY_CALLS; SRS FR3.1</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="49" t="inlineStr">
         <is>
-          <t>MED-04</t>
+          <t>UX-03</t>
         </is>
       </c>
       <c r="B134" s="49" t="inlineStr">
@@ -11410,19 +11606,19 @@
       </c>
       <c r="C134" s="49" t="inlineStr">
         <is>
-          <t>Sensitive medical fields are encrypted at rest</t>
+          <t>The same MediFind logo is used in the mobile app and the web portal</t>
         </is>
       </c>
       <c r="D134" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.2</t>
+          <t>New sheet PRIVACY_CALLS; SRS NFR</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="49" t="inlineStr">
         <is>
-          <t>MED-05</t>
+          <t>MED-01</t>
         </is>
       </c>
       <c r="B135" s="49" t="inlineStr">
@@ -11432,19 +11628,19 @@
       </c>
       <c r="C135" s="49" t="inlineStr">
         <is>
-          <t>Upload a report from camera, gallery (image) and PDF</t>
+          <t>Patient creates and edits the medical profile</t>
         </is>
       </c>
       <c r="D135" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.3</t>
+          <t>New sheet MEDICAL; SRS FR2.1, FR2.2</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="49" t="inlineStr">
         <is>
-          <t>MED-06</t>
+          <t>MED-02</t>
         </is>
       </c>
       <c r="B136" s="49" t="inlineStr">
@@ -11454,19 +11650,19 @@
       </c>
       <c r="C136" s="49" t="inlineStr">
         <is>
-          <t>Unsupported or oversized files are rejected with a clear message</t>
+          <t>Saving the medical profile keeps emergency contacts and quick phrases</t>
         </is>
       </c>
       <c r="D136" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.3</t>
+          <t>New sheet MEDICAL; SRS FR2.1</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="49" t="inlineStr">
         <is>
-          <t>MED-07</t>
+          <t>MED-03</t>
         </is>
       </c>
       <c r="B137" s="49" t="inlineStr">
@@ -11476,19 +11672,19 @@
       </c>
       <c r="C137" s="49" t="inlineStr">
         <is>
-          <t>View, rename and delete a report</t>
+          <t>Patient adds, calls and deletes emergency contacts</t>
         </is>
       </c>
       <c r="D137" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.4</t>
+          <t>New sheet MEDICAL; SRS FR2.1</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="49" t="inlineStr">
         <is>
-          <t>MED-08</t>
+          <t>MED-04</t>
         </is>
       </c>
       <c r="B138" s="49" t="inlineStr">
@@ -11498,19 +11694,19 @@
       </c>
       <c r="C138" s="49" t="inlineStr">
         <is>
-          <t>Assigned responder receives the patient medical summary on accept</t>
+          <t>Sensitive medical fields are encrypted at rest</t>
         </is>
       </c>
       <c r="D138" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.5</t>
+          <t>New sheet MEDICAL; SRS FR2.2</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="49" t="inlineStr">
         <is>
-          <t>MED-09</t>
+          <t>MED-05</t>
         </is>
       </c>
       <c r="B139" s="49" t="inlineStr">
@@ -11520,19 +11716,19 @@
       </c>
       <c r="C139" s="49" t="inlineStr">
         <is>
-          <t>Report files are visible only to the patient, linked caregivers, the active responder and admins</t>
+          <t>Upload a report from camera, gallery (image) and PDF</t>
         </is>
       </c>
       <c r="D139" s="49" t="inlineStr">
         <is>
-          <t>New sheet MEDICAL; SRS FR2.6</t>
+          <t>New sheet MEDICAL; SRS FR2.3</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="49" t="inlineStr">
         <is>
-          <t>SEC-01</t>
+          <t>MED-06</t>
         </is>
       </c>
       <c r="B140" s="49" t="inlineStr">
@@ -11542,19 +11738,19 @@
       </c>
       <c r="C140" s="49" t="inlineStr">
         <is>
-          <t>SOS requires press-and-hold before it starts</t>
+          <t>Unsupported or oversized files are rejected with a clear message</t>
         </is>
       </c>
       <c r="D140" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.1</t>
+          <t>New sheet MEDICAL; SRS FR2.3</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="49" t="inlineStr">
         <is>
-          <t>SEC-02</t>
+          <t>MED-07</t>
         </is>
       </c>
       <c r="B141" s="49" t="inlineStr">
@@ -11564,19 +11760,19 @@
       </c>
       <c r="C141" s="49" t="inlineStr">
         <is>
-          <t>Cancelling during the 60-second countdown sends nothing to the server</t>
+          <t>View, rename and delete a report</t>
         </is>
       </c>
       <c r="D141" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.3</t>
+          <t>New sheet MEDICAL; SRS FR2.4</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="49" t="inlineStr">
         <is>
-          <t>SEC-03</t>
+          <t>MED-08</t>
         </is>
       </c>
       <c r="B142" s="49" t="inlineStr">
@@ -11586,19 +11782,19 @@
       </c>
       <c r="C142" s="49" t="inlineStr">
         <is>
-          <t>SOS from a mock (fake) GPS location is refused in production</t>
+          <t>Assigned responder receives the patient medical summary on accept</t>
         </is>
       </c>
       <c r="D142" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
+          <t>New sheet MEDICAL; SRS FR2.5</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="49" t="inlineStr">
         <is>
-          <t>SEC-04</t>
+          <t>MED-09</t>
         </is>
       </c>
       <c r="B143" s="49" t="inlineStr">
@@ -11608,19 +11804,19 @@
       </c>
       <c r="C143" s="49" t="inlineStr">
         <is>
-          <t>More than 5 SOS in one hour is refused</t>
+          <t>Report files are visible only to the patient, linked caregivers, the active responder and admins</t>
         </is>
       </c>
       <c r="D143" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.5</t>
+          <t>New sheet MEDICAL; SRS FR2.6</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="49" t="inlineStr">
         <is>
-          <t>SEC-05</t>
+          <t>SEC-01</t>
         </is>
       </c>
       <c r="B144" s="49" t="inlineStr">
@@ -11630,19 +11826,19 @@
       </c>
       <c r="C144" s="49" t="inlineStr">
         <is>
-          <t>SOS outside Pakistan coordinates is refused</t>
+          <t>SOS requires press-and-hold before it starts</t>
         </is>
       </c>
       <c r="D144" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.1</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="49" t="inlineStr">
         <is>
-          <t>SEC-06</t>
+          <t>SEC-02</t>
         </is>
       </c>
       <c r="B145" s="49" t="inlineStr">
@@ -11652,19 +11848,19 @@
       </c>
       <c r="C145" s="49" t="inlineStr">
         <is>
-          <t>Responder must add a note when closing as False alarm or Patient not found</t>
+          <t>Cancelling during the 60-second countdown sends nothing to the server</t>
         </is>
       </c>
       <c r="D145" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR6.2</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.3</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="49" t="inlineStr">
         <is>
-          <t>SEC-07</t>
+          <t>SEC-03</t>
         </is>
       </c>
       <c r="B146" s="49" t="inlineStr">
@@ -11674,19 +11870,19 @@
       </c>
       <c r="C146" s="49" t="inlineStr">
         <is>
-          <t>Patient is warned when an SOS is marked as a false alarm</t>
+          <t>SOS from a mock (fake) GPS location is refused in production</t>
         </is>
       </c>
       <c r="D146" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; beyond SRS</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="49" t="inlineStr">
         <is>
-          <t>SEC-08</t>
+          <t>SEC-04</t>
         </is>
       </c>
       <c r="B147" s="49" t="inlineStr">
@@ -11696,19 +11892,19 @@
       </c>
       <c r="C147" s="49" t="inlineStr">
         <is>
-          <t>3 false alarms in 30 days alerts admins for review</t>
+          <t>More than 5 SOS in one hour is refused</t>
         </is>
       </c>
       <c r="D147" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; beyond SRS</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.5</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="49" t="inlineStr">
         <is>
-          <t>SEC-09</t>
+          <t>SEC-05</t>
         </is>
       </c>
       <c r="B148" s="49" t="inlineStr">
@@ -11718,19 +11914,19 @@
       </c>
       <c r="C148" s="49" t="inlineStr">
         <is>
-          <t>Patient-cancelled SOS never counts as a false alarm</t>
+          <t>SOS outside Pakistan coordinates is refused</t>
         </is>
       </c>
       <c r="D148" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; beyond SRS</t>
+          <t>New sheet SECURITY_SOS; SRS FR4.2</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="49" t="inlineStr">
         <is>
-          <t>SEC-10</t>
+          <t>SEC-06</t>
         </is>
       </c>
       <c r="B149" s="49" t="inlineStr">
@@ -11740,19 +11936,19 @@
       </c>
       <c r="C149" s="49" t="inlineStr">
         <is>
-          <t>Refresh token cannot be used as an access token</t>
+          <t>Responder must add a note when closing as False alarm or Patient not found</t>
         </is>
       </c>
       <c r="D149" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
+          <t>New sheet SECURITY_SOS; SRS FR6.2</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="49" t="inlineStr">
         <is>
-          <t>SEC-11</t>
+          <t>SEC-07</t>
         </is>
       </c>
       <c r="B150" s="49" t="inlineStr">
@@ -11762,19 +11958,19 @@
       </c>
       <c r="C150" s="49" t="inlineStr">
         <is>
-          <t>Users cannot join emergency or chat rooms they do not belong to</t>
+          <t>Patient is warned when an SOS is marked as a false alarm</t>
         </is>
       </c>
       <c r="D150" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
+          <t>New sheet SECURITY_SOS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="49" t="inlineStr">
         <is>
-          <t>SEC-12</t>
+          <t>SEC-08</t>
         </is>
       </c>
       <c r="B151" s="49" t="inlineStr">
@@ -11784,7 +11980,7 @@
       </c>
       <c r="C151" s="49" t="inlineStr">
         <is>
-          <t>Paid plan upgrade requires a verified Stripe payment</t>
+          <t>3 false alarms in 30 days alerts admins for review</t>
         </is>
       </c>
       <c r="D151" s="49" t="inlineStr">
@@ -11796,7 +11992,7 @@
     <row r="152">
       <c r="A152" s="49" t="inlineStr">
         <is>
-          <t>SEC-13</t>
+          <t>SEC-09</t>
         </is>
       </c>
       <c r="B152" s="49" t="inlineStr">
@@ -11806,19 +12002,19 @@
       </c>
       <c r="C152" s="49" t="inlineStr">
         <is>
-          <t>Only the assigned responder can update or resolve an emergency</t>
+          <t>Patient-cancelled SOS never counts as a false alarm</t>
         </is>
       </c>
       <c r="D152" s="49" t="inlineStr">
         <is>
-          <t>New sheet SECURITY_SOS; SRS FR5.1</t>
+          <t>New sheet SECURITY_SOS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="49" t="inlineStr">
         <is>
-          <t>NAV-01</t>
+          <t>SEC-10</t>
         </is>
       </c>
       <c r="B153" s="49" t="inlineStr">
@@ -11828,19 +12024,19 @@
       </c>
       <c r="C153" s="49" t="inlineStr">
         <is>
-          <t>Each role has a unified sidebar (AppDrawer) with role-specific items</t>
+          <t>Refresh token cannot be used as an access token</t>
         </is>
       </c>
       <c r="D153" s="49" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.1</t>
+          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="49" t="inlineStr">
         <is>
-          <t>NAV-02</t>
+          <t>SEC-11</t>
         </is>
       </c>
       <c r="B154" s="49" t="inlineStr">
@@ -11850,19 +12046,19 @@
       </c>
       <c r="C154" s="49" t="inlineStr">
         <is>
-          <t>Switching tabs preserves each tab's state and back navigation works</t>
+          <t>Users cannot join emergency or chat rooms they do not belong to</t>
         </is>
       </c>
       <c r="D154" s="49" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.2</t>
+          <t>New sheet SECURITY_SOS; SRS FR1.6</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="49" t="inlineStr">
         <is>
-          <t>NAV-03</t>
+          <t>SEC-12</t>
         </is>
       </c>
       <c r="B155" s="49" t="inlineStr">
@@ -11872,19 +12068,19 @@
       </c>
       <c r="C155" s="49" t="inlineStr">
         <is>
-          <t>Role dashboards show quick action grids</t>
+          <t>Paid plan upgrade requires a verified Stripe payment</t>
         </is>
       </c>
       <c r="D155" s="49" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.3</t>
+          <t>New sheet SECURITY_SOS; beyond SRS</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="49" t="inlineStr">
         <is>
-          <t>NAV-04</t>
+          <t>SEC-13</t>
         </is>
       </c>
       <c r="B156" s="49" t="inlineStr">
@@ -11894,19 +12090,19 @@
       </c>
       <c r="C156" s="49" t="inlineStr">
         <is>
-          <t>Map and chat screens render smoothly (~60 FPS)</t>
+          <t>Only the assigned responder can update or resolve an emergency</t>
         </is>
       </c>
       <c r="D156" s="49" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR8.4</t>
+          <t>New sheet SECURITY_SOS; SRS FR5.1</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="49" t="inlineStr">
         <is>
-          <t>NAV-05</t>
+          <t>NAV-01</t>
         </is>
       </c>
       <c r="B157" s="49" t="inlineStr">
@@ -11916,107 +12112,107 @@
       </c>
       <c r="C157" s="49" t="inlineStr">
         <is>
-          <t>Large buttons mode enlarges tap targets across screens</t>
+          <t>Each role has a unified sidebar (AppDrawer) with role-specific items</t>
         </is>
       </c>
       <c r="D157" s="49" t="inlineStr">
         <is>
-          <t>New sheet NAVIGATION_UI; SRS FR3.5</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.1</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="49" t="inlineStr">
         <is>
-          <t>PRF-01</t>
+          <t>NAV-02</t>
         </is>
       </c>
       <c r="B158" s="49" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C158" s="49" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Switching tabs preserves each tab's state and back navigation works</t>
         </is>
       </c>
       <c r="D158" s="49" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.2</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="49" t="inlineStr">
         <is>
-          <t>PRF-02</t>
+          <t>NAV-03</t>
         </is>
       </c>
       <c r="B159" s="49" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C159" s="49" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Role dashboards show quick action grids</t>
         </is>
       </c>
       <c r="D159" s="49" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.3</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="49" t="inlineStr">
         <is>
-          <t>PRF-03</t>
+          <t>NAV-04</t>
         </is>
       </c>
       <c r="B160" s="49" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C160" s="49" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Map and chat screens render smoothly (~60 FPS)</t>
         </is>
       </c>
       <c r="D160" s="49" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR8.4</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="49" t="inlineStr">
         <is>
-          <t>PRF-05</t>
+          <t>NAV-05</t>
         </is>
       </c>
       <c r="B161" s="49" t="inlineStr">
         <is>
-          <t>Re-classified</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="C161" s="49" t="inlineStr">
         <is>
-          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+          <t>Large buttons mode enlarges tap targets across screens</t>
         </is>
       </c>
       <c r="D161" s="49" t="inlineStr">
         <is>
-          <t>Valid feature test with no matching SRS functional requirement</t>
+          <t>New sheet NAVIGATION_UI; SRS FR3.5</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="49" t="inlineStr">
         <is>
-          <t>NTF-01</t>
+          <t>PRF-01</t>
         </is>
       </c>
       <c r="B162" s="49" t="inlineStr">
@@ -12038,7 +12234,7 @@
     <row r="163">
       <c r="A163" s="49" t="inlineStr">
         <is>
-          <t>NTF-02</t>
+          <t>PRF-02</t>
         </is>
       </c>
       <c r="B163" s="49" t="inlineStr">
@@ -12060,7 +12256,7 @@
     <row r="164">
       <c r="A164" s="49" t="inlineStr">
         <is>
-          <t>NTF-03</t>
+          <t>PRF-03</t>
         </is>
       </c>
       <c r="B164" s="49" t="inlineStr">
@@ -12082,7 +12278,7 @@
     <row r="165">
       <c r="A165" s="49" t="inlineStr">
         <is>
-          <t>NTF-04</t>
+          <t>PRF-05</t>
         </is>
       </c>
       <c r="B165" s="49" t="inlineStr">
@@ -12104,7 +12300,7 @@
     <row r="166">
       <c r="A166" s="49" t="inlineStr">
         <is>
-          <t>NTF-05</t>
+          <t>NTF-01</t>
         </is>
       </c>
       <c r="B166" s="49" t="inlineStr">
@@ -12126,7 +12322,7 @@
     <row r="167">
       <c r="A167" s="49" t="inlineStr">
         <is>
-          <t>NTF-07</t>
+          <t>NTF-02</t>
         </is>
       </c>
       <c r="B167" s="49" t="inlineStr">
@@ -12148,7 +12344,7 @@
     <row r="168">
       <c r="A168" s="49" t="inlineStr">
         <is>
-          <t>NTF-08</t>
+          <t>NTF-03</t>
         </is>
       </c>
       <c r="B168" s="49" t="inlineStr">
@@ -12170,7 +12366,7 @@
     <row r="169">
       <c r="A169" s="49" t="inlineStr">
         <is>
-          <t>ACC-06</t>
+          <t>NTF-04</t>
         </is>
       </c>
       <c r="B169" s="49" t="inlineStr">
@@ -12192,7 +12388,7 @@
     <row r="170">
       <c r="A170" s="49" t="inlineStr">
         <is>
-          <t>ACC-07</t>
+          <t>NTF-05</t>
         </is>
       </c>
       <c r="B170" s="49" t="inlineStr">
@@ -12214,7 +12410,7 @@
     <row r="171">
       <c r="A171" s="49" t="inlineStr">
         <is>
-          <t>ACC-11</t>
+          <t>NTF-07</t>
         </is>
       </c>
       <c r="B171" s="49" t="inlineStr">
@@ -12236,7 +12432,7 @@
     <row r="172">
       <c r="A172" s="49" t="inlineStr">
         <is>
-          <t>AUTH-12</t>
+          <t>NTF-08</t>
         </is>
       </c>
       <c r="B172" s="49" t="inlineStr">
@@ -12258,7 +12454,7 @@
     <row r="173">
       <c r="A173" s="49" t="inlineStr">
         <is>
-          <t>API-04</t>
+          <t>ACC-06</t>
         </is>
       </c>
       <c r="B173" s="49" t="inlineStr">
@@ -12280,7 +12476,7 @@
     <row r="174">
       <c r="A174" s="49" t="inlineStr">
         <is>
-          <t>API-08</t>
+          <t>ACC-07</t>
         </is>
       </c>
       <c r="B174" s="49" t="inlineStr">
@@ -12302,20 +12498,108 @@
     <row r="175">
       <c r="A175" s="49" t="inlineStr">
         <is>
+          <t>ACC-11</t>
+        </is>
+      </c>
+      <c r="B175" s="49" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C175" s="49" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D175" s="49" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="49" t="inlineStr">
+        <is>
+          <t>AUTH-12</t>
+        </is>
+      </c>
+      <c r="B176" s="49" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C176" s="49" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D176" s="49" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="49" t="inlineStr">
+        <is>
+          <t>API-04</t>
+        </is>
+      </c>
+      <c r="B177" s="49" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C177" s="49" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D177" s="49" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="49" t="inlineStr">
+        <is>
+          <t>API-08</t>
+        </is>
+      </c>
+      <c r="B178" s="49" t="inlineStr">
+        <is>
+          <t>Re-classified</t>
+        </is>
+      </c>
+      <c r="C178" s="49" t="inlineStr">
+        <is>
+          <t>Marked "Beyond SRS" in the SRS Ref column</t>
+        </is>
+      </c>
+      <c r="D178" s="49" t="inlineStr">
+        <is>
+          <t>Valid feature test with no matching SRS functional requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="49" t="inlineStr">
+        <is>
           <t>API-09</t>
         </is>
       </c>
-      <c r="B175" s="49" t="inlineStr">
+      <c r="B179" s="49" t="inlineStr">
         <is>
           <t>Re-classified</t>
         </is>
       </c>
-      <c r="C175" s="49" t="inlineStr">
+      <c r="C179" s="49" t="inlineStr">
         <is>
           <t>Marked "Beyond SRS" in the SRS Ref column</t>
         </is>
       </c>
-      <c r="D175" s="49" t="inlineStr">
+      <c r="D179" s="49" t="inlineStr">
         <is>
           <t>Valid feature test with no matching SRS functional requirement</t>
         </is>
@@ -12679,27 +12963,27 @@
         </is>
       </c>
       <c r="C11" s="19">
-        <f>COUNTA(PRIVACY_CALLS!$A$4:$A$72)-COUNTIF(PRIVACY_CALLS!$A$4:$A$72,"  *")</f>
+        <f>COUNTA(PRIVACY_CALLS!$A$4:$A$77)-COUNTIF(PRIVACY_CALLS!$A$4:$A$77,"  *")</f>
         <v/>
       </c>
       <c r="D11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$72,"PASS")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$77,"PASS")</f>
         <v/>
       </c>
       <c r="E11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$72,"FAIL")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$77,"FAIL")</f>
         <v/>
       </c>
       <c r="F11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$72,"PENDING")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$77,"PENDING")</f>
         <v/>
       </c>
       <c r="G11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$72,"BLOCKED")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$77,"BLOCKED")</f>
         <v/>
       </c>
       <c r="H11" s="19">
-        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$72,"N/A")</f>
+        <f>COUNTIF(PRIVACY_CALLS!$H$4:$H$77,"N/A")</f>
         <v/>
       </c>
       <c r="I11" s="21">
@@ -13059,7 +13343,7 @@
         </is>
       </c>
       <c r="D3" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR1.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR1.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.1*")</f>
         <v/>
       </c>
       <c r="E3" s="29">
@@ -13089,7 +13373,7 @@
         </is>
       </c>
       <c r="D4" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR1.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR1.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.2*")</f>
         <v/>
       </c>
       <c r="E4" s="32">
@@ -13119,7 +13403,7 @@
         </is>
       </c>
       <c r="D5" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR1.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR1.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.3*")</f>
         <v/>
       </c>
       <c r="E5" s="29">
@@ -13149,7 +13433,7 @@
         </is>
       </c>
       <c r="D6" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR1.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR1.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.4*")</f>
         <v/>
       </c>
       <c r="E6" s="32">
@@ -13179,7 +13463,7 @@
         </is>
       </c>
       <c r="D7" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR1.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR1.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.5*")</f>
         <v/>
       </c>
       <c r="E7" s="29">
@@ -13209,7 +13493,7 @@
         </is>
       </c>
       <c r="D8" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR1.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR1.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR1.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR1.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR1.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR1.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR1.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR1.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR1.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR1.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR1.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR1.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR1.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR1.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR1.6*")</f>
         <v/>
       </c>
       <c r="E8" s="32">
@@ -13239,7 +13523,7 @@
         </is>
       </c>
       <c r="D9" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR2.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR2.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.1*")</f>
         <v/>
       </c>
       <c r="E9" s="29">
@@ -13269,7 +13553,7 @@
         </is>
       </c>
       <c r="D10" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR2.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR2.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.2*")</f>
         <v/>
       </c>
       <c r="E10" s="32">
@@ -13299,7 +13583,7 @@
         </is>
       </c>
       <c r="D11" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR2.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR2.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.3*")</f>
         <v/>
       </c>
       <c r="E11" s="29">
@@ -13329,7 +13613,7 @@
         </is>
       </c>
       <c r="D12" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR2.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR2.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.4*")</f>
         <v/>
       </c>
       <c r="E12" s="32">
@@ -13359,7 +13643,7 @@
         </is>
       </c>
       <c r="D13" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR2.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR2.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.5*")</f>
         <v/>
       </c>
       <c r="E13" s="29">
@@ -13389,7 +13673,7 @@
         </is>
       </c>
       <c r="D14" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR2.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR2.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR2.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR2.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR2.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR2.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR2.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR2.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR2.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR2.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR2.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR2.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR2.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR2.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR2.6*")</f>
         <v/>
       </c>
       <c r="E14" s="32">
@@ -13419,7 +13703,7 @@
         </is>
       </c>
       <c r="D15" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR3.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR3.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.1*")</f>
         <v/>
       </c>
       <c r="E15" s="29">
@@ -13449,7 +13733,7 @@
         </is>
       </c>
       <c r="D16" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR3.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR3.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.2*")</f>
         <v/>
       </c>
       <c r="E16" s="32">
@@ -13479,7 +13763,7 @@
         </is>
       </c>
       <c r="D17" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR3.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR3.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.3*")</f>
         <v/>
       </c>
       <c r="E17" s="29">
@@ -13509,7 +13793,7 @@
         </is>
       </c>
       <c r="D18" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR3.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR3.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.4*")</f>
         <v/>
       </c>
       <c r="E18" s="32">
@@ -13539,7 +13823,7 @@
         </is>
       </c>
       <c r="D19" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR3.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR3.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR3.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR3.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR3.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR3.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR3.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR3.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR3.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR3.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR3.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR3.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR3.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR3.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR3.5*")</f>
         <v/>
       </c>
       <c r="E19" s="29">
@@ -13569,7 +13853,7 @@
         </is>
       </c>
       <c r="D20" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR4.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR4.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.1*")</f>
         <v/>
       </c>
       <c r="E20" s="32">
@@ -13599,7 +13883,7 @@
         </is>
       </c>
       <c r="D21" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR4.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR4.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.2*")</f>
         <v/>
       </c>
       <c r="E21" s="29">
@@ -13629,7 +13913,7 @@
         </is>
       </c>
       <c r="D22" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR4.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR4.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.3*")</f>
         <v/>
       </c>
       <c r="E22" s="32">
@@ -13659,7 +13943,7 @@
         </is>
       </c>
       <c r="D23" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR4.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR4.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.4*")</f>
         <v/>
       </c>
       <c r="E23" s="29">
@@ -13689,7 +13973,7 @@
         </is>
       </c>
       <c r="D24" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR4.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR4.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.5*")</f>
         <v/>
       </c>
       <c r="E24" s="32">
@@ -13719,7 +14003,7 @@
         </is>
       </c>
       <c r="D25" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR4.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR4.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR4.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR4.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR4.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR4.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR4.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR4.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR4.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR4.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR4.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR4.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR4.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR4.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR4.6*")</f>
         <v/>
       </c>
       <c r="E25" s="29">
@@ -13749,7 +14033,7 @@
         </is>
       </c>
       <c r="D26" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR5.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR5.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.1*")</f>
         <v/>
       </c>
       <c r="E26" s="32">
@@ -13779,7 +14063,7 @@
         </is>
       </c>
       <c r="D27" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR5.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR5.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.2*")</f>
         <v/>
       </c>
       <c r="E27" s="29">
@@ -13809,7 +14093,7 @@
         </is>
       </c>
       <c r="D28" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR5.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR5.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.3*")</f>
         <v/>
       </c>
       <c r="E28" s="32">
@@ -13839,7 +14123,7 @@
         </is>
       </c>
       <c r="D29" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR5.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR5.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR5.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR5.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR5.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR5.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR5.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR5.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR5.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR5.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR5.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR5.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR5.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR5.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR5.4*")</f>
         <v/>
       </c>
       <c r="E29" s="29">
@@ -13869,7 +14153,7 @@
         </is>
       </c>
       <c r="D30" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR6.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR6.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.1*")</f>
         <v/>
       </c>
       <c r="E30" s="32">
@@ -13899,7 +14183,7 @@
         </is>
       </c>
       <c r="D31" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR6.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR6.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.2*")</f>
         <v/>
       </c>
       <c r="E31" s="29">
@@ -13929,7 +14213,7 @@
         </is>
       </c>
       <c r="D32" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR6.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR6.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.3*")</f>
         <v/>
       </c>
       <c r="E32" s="32">
@@ -13959,7 +14243,7 @@
         </is>
       </c>
       <c r="D33" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR6.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR6.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR6.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR6.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR6.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR6.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR6.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR6.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR6.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR6.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR6.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR6.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR6.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR6.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR6.4*")</f>
         <v/>
       </c>
       <c r="E33" s="29">
@@ -13989,7 +14273,7 @@
         </is>
       </c>
       <c r="D34" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR7.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR7.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.1*")</f>
         <v/>
       </c>
       <c r="E34" s="32">
@@ -14019,7 +14303,7 @@
         </is>
       </c>
       <c r="D35" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR7.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR7.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.2*")</f>
         <v/>
       </c>
       <c r="E35" s="29">
@@ -14049,7 +14333,7 @@
         </is>
       </c>
       <c r="D36" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR7.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR7.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.3*")</f>
         <v/>
       </c>
       <c r="E36" s="32">
@@ -14058,7 +14342,7 @@
       </c>
       <c r="F36" s="31" t="inlineStr">
         <is>
-          <t>CHT-09, PRV-01, PRV-02, LCK-01</t>
+          <t>CHT-09, PRV-01, PRV-02, LCK-01, MSG-01, MSG-02</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14363,7 @@
         </is>
       </c>
       <c r="D37" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR7.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR7.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.4*")</f>
         <v/>
       </c>
       <c r="E37" s="29">
@@ -14109,7 +14393,7 @@
         </is>
       </c>
       <c r="D38" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR7.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR7.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR7.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR7.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR7.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR7.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR7.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR7.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR7.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR7.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR7.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR7.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR7.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR7.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR7.5*")</f>
         <v/>
       </c>
       <c r="E38" s="32">
@@ -14139,7 +14423,7 @@
         </is>
       </c>
       <c r="D39" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR8.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR8.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.1*")</f>
         <v/>
       </c>
       <c r="E39" s="29">
@@ -14169,7 +14453,7 @@
         </is>
       </c>
       <c r="D40" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR8.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR8.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.2*")</f>
         <v/>
       </c>
       <c r="E40" s="32">
@@ -14199,7 +14483,7 @@
         </is>
       </c>
       <c r="D41" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR8.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR8.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.3*")</f>
         <v/>
       </c>
       <c r="E41" s="29">
@@ -14229,7 +14513,7 @@
         </is>
       </c>
       <c r="D42" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR8.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR8.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR8.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR8.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR8.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR8.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR8.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR8.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR8.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR8.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR8.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR8.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR8.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR8.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR8.4*")</f>
         <v/>
       </c>
       <c r="E42" s="32">
@@ -14259,7 +14543,7 @@
         </is>
       </c>
       <c r="D43" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR9.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.1*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.1*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.1*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.1*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.1*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.1*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.1*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.1*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR9.1*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.1*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.1*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.1*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.1*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.1*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.1*")</f>
         <v/>
       </c>
       <c r="E43" s="29">
@@ -14289,7 +14573,7 @@
         </is>
       </c>
       <c r="D44" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR9.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.2*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.2*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.2*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.2*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.2*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.2*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.2*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.2*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR9.2*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.2*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.2*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.2*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.2*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.2*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.2*")</f>
         <v/>
       </c>
       <c r="E44" s="32">
@@ -14319,7 +14603,7 @@
         </is>
       </c>
       <c r="D45" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR9.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.3*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.3*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.3*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.3*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.3*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.3*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.3*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.3*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR9.3*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.3*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.3*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.3*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.3*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.3*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.3*")</f>
         <v/>
       </c>
       <c r="E45" s="29">
@@ -14349,7 +14633,7 @@
         </is>
       </c>
       <c r="D46" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR9.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.4*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.4*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.4*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.4*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.4*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.4*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.4*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.4*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR9.4*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.4*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.4*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.4*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.4*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.4*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.4*")</f>
         <v/>
       </c>
       <c r="E46" s="32">
@@ -14379,7 +14663,7 @@
         </is>
       </c>
       <c r="D47" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR9.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.5*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.5*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.5*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.5*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.5*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.5*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.5*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.5*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR9.5*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.5*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.5*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.5*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.5*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.5*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.5*")</f>
         <v/>
       </c>
       <c r="E47" s="29">
@@ -14409,7 +14693,7 @@
         </is>
       </c>
       <c r="D48" s="32">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR9.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.6*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.6*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.6*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.6*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.6*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.6*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.6*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.6*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR9.6*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.6*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.6*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.6*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.6*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.6*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.6*")</f>
         <v/>
       </c>
       <c r="E48" s="32">
@@ -14439,7 +14723,7 @@
         </is>
       </c>
       <c r="D49" s="29">
-        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.7*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.7*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.7*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.7*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.7*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.7*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.7*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$72,"*FR9.7*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.7*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.7*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.7*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.7*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.7*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.7*")</f>
+        <f>COUNTIF(AUTH!$B$4:$B$23,"*FR9.7*")+COUNTIF(PATIENT_SOS!$B$4:$B$21,"*FR9.7*")+COUNTIF(SECURITY_SOS!$B$4:$B$18,"*FR9.7*")+COUNTIF(RESPONDER!$B$4:$B$21,"*FR9.7*")+COUNTIF(CAREGIVER!$B$4:$B$15,"*FR9.7*")+COUNTIF(MEDICAL!$B$4:$B$14,"*FR9.7*")+COUNTIF(CHAT!$B$4:$B$17,"*FR9.7*")+COUNTIF(PRIVACY_CALLS!$B$4:$B$77,"*FR9.7*")+COUNTIF(PROFILE!$B$4:$B$9,"*FR9.7*")+COUNTIF(ACCESSIBILITY!$B$4:$B$22,"*FR9.7*")+COUNTIF(NOTIFICATIONS!$B$4:$B$19,"*FR9.7*")+COUNTIF(NAVIGATION_UI!$B$4:$B$8,"*FR9.7*")+COUNTIF(ADMIN_PORTAL!$B$4:$B$19,"*FR9.7*")+COUNTIF(BACKEND_API!$B$4:$B$23,"*FR9.7*")</f>
         <v/>
       </c>
       <c r="E49" s="29">

</xml_diff>